<commit_message>
midterm report with demo video
</commit_message>
<xml_diff>
--- a/DocumentsAndReports/0. WorkLog_Charts.xlsx
+++ b/DocumentsAndReports/0. WorkLog_Charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qhung\Videos\CSIS4495 - Applied Research  Project\W26_4495_S2_HughT\DocumentsAndReports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C9A8528-F9A3-49F1-A1D2-2BFC803C95B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FF5E6F1-94D2-49BB-B230-C471500E2002}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E067A1E6-0DC4-42DD-AAF8-D95EFF7A112F}"/>
+    <workbookView xWindow="30720" yWindow="1920" windowWidth="21600" windowHeight="11235" xr2:uid="{E067A1E6-0DC4-42DD-AAF8-D95EFF7A112F}"/>
   </bookViews>
   <sheets>
     <sheet name="Work_Log" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="87">
   <si>
     <t>January</t>
   </si>
@@ -278,12 +278,87 @@
   <si>
     <t>“why should use jinja template?, what if not using it”</t>
   </si>
+  <si>
+    <t>INITIAL PLAN</t>
+  </si>
+  <si>
+    <t>“debug these code”</t>
+  </si>
+  <si>
+    <t>- Kept developing the FastAPI backend structure.</t>
+  </si>
+  <si>
+    <t>- Tested basic API endpoint to confirm backend server runs correctly.</t>
+  </si>
+  <si>
+    <t>- ChatGPT’s prompts:</t>
+  </si>
+  <si>
+    <t>- Started developing the FastAPI backend structure.</t>
+  </si>
+  <si>
+    <t>- Developed file upload endpoint in FastAPI</t>
+  </si>
+  <si>
+    <t>- Tested uploading CSV files from local machine.</t>
+  </si>
+  <si>
+    <t>- Developed basic HTML form for dataset upload.</t>
+  </si>
+  <si>
+    <t>- Integrated frontend form with FastAPI backend endpoint.</t>
+  </si>
+  <si>
+    <t>"how to connect html form with fastapi backend?”</t>
+  </si>
+  <si>
+    <t>- Improved frontend layout using Bootstrap.</t>
+  </si>
+  <si>
+    <t>- Organized upload section and status display messages.</t>
+  </si>
+  <si>
+    <t>- Tested full upload-to-database pipeline again.</t>
+  </si>
+  <si>
+    <t>“how to display successful response in html”</t>
+  </si>
+  <si>
+    <t>- Tested layering process in SQL Server after frontend upload.</t>
+  </si>
+  <si>
+    <t>- Verified raw -&gt; clean -&gt; analytics transformation works correctly.</t>
+  </si>
+  <si>
+    <t>- Fixed issues in foreign key relationships.</t>
+  </si>
+  <si>
+    <t>“why foreign key constraint failed?”</t>
+  </si>
+  <si>
+    <t>- Improved SQL aggregation queries in analytics layer.</t>
+  </si>
+  <si>
+    <t>- Tested daily and monthly summary tables.</t>
+  </si>
+  <si>
+    <t>- Draft the midterm report</t>
+  </si>
+  <si>
+    <t>- Outlined structure of the demo video:</t>
+  </si>
+  <si>
+    <t>- Made the video, finalized the midterm report</t>
+  </si>
+  <si>
+    <t>THE ADJUSTED PLAN</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -361,6 +436,12 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -382,7 +463,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="33">
+  <borders count="37">
     <border>
       <left/>
       <right/>
@@ -780,11 +861,55 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -844,9 +969,6 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
@@ -891,8 +1013,27 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="31" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="25" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -900,22 +1041,6 @@
     <xf numFmtId="15" fontId="7" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="25" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="15" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -933,6 +1058,51 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="35" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="36" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="33" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="34" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1407,6 +1577,501 @@
         <a:xfrm>
           <a:off x="9422131" y="2407919"/>
           <a:ext cx="548639" cy="146685"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent6">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent6">
+              <a:lumMod val="40000"/>
+              <a:lumOff val="60000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent2"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>30480</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>59057</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>592455</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>209550</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="Rectangle: Rounded Corners 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8E62D547-AE50-41A2-938A-7AEBC03D61AF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3933825" y="807722"/>
+          <a:ext cx="1169670" cy="150493"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent2"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent6">
+              <a:lumMod val="40000"/>
+              <a:lumOff val="60000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent2"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>59054</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>590550</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>219075</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="9" name="Rectangle: Rounded Corners 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BBDE214E-5F2C-4863-8024-58B81202D4A8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4530090" y="1074419"/>
+          <a:ext cx="571500" cy="161926"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent2"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent6">
+              <a:lumMod val="40000"/>
+              <a:lumOff val="60000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent2"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>26671</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>55246</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>592455</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>209550</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="Rectangle: Rounded Corners 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{68CA394E-A3C1-47CB-B02A-FAEAB9B3C1F4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5149216" y="1344931"/>
+          <a:ext cx="1173479" cy="146684"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent2"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent6">
+              <a:lumMod val="40000"/>
+              <a:lumOff val="60000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent2"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>28574</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>53341</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>569595</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>205740</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="12" name="Rectangle: Rounded Corners 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3C98D914-DC20-4240-BEA5-E35C2E7F9033}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5762624" y="4396741"/>
+          <a:ext cx="1760221" cy="152399"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent6">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent6">
+              <a:lumMod val="40000"/>
+              <a:lumOff val="60000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent2"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>26669</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>57149</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>592454</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>209550</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="13" name="Rectangle: Rounded Corners 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5F8E7C8A-4BCE-40BD-9A45-6BC2D352D136}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6370319" y="4667249"/>
+          <a:ext cx="2394585" cy="152401"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent6">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent6">
+              <a:lumMod val="40000"/>
+              <a:lumOff val="60000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent2"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>55246</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>573405</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>209550</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="14" name="Rectangle: Rounded Corners 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8B84E06C-A146-4C22-9DF2-7C958393DAD1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7578090" y="2145031"/>
+          <a:ext cx="1777365" cy="146684"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent6">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent6">
+              <a:lumMod val="40000"/>
+              <a:lumOff val="60000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent2"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>30481</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>55244</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>579120</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>201929</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="15" name="Rectangle: Rounded Corners 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A3962869-F336-4058-AE09-B9F6064F8BE4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9420226" y="2411729"/>
+          <a:ext cx="552449" cy="144780"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -1774,7 +2439,7 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="B1:D99"/>
+  <dimension ref="B1:D141"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="2"/>
@@ -1797,328 +2462,328 @@
       </c>
     </row>
     <row r="3" spans="2:4" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="54">
+      <c r="B3" s="60">
         <v>45683</v>
       </c>
-      <c r="C3" s="53">
+      <c r="C3" s="59">
         <v>2</v>
       </c>
-      <c r="D3" s="36" t="s">
+      <c r="D3" s="35" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="4" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="54"/>
-      <c r="C4" s="53"/>
-      <c r="D4" s="36" t="s">
+      <c r="B4" s="60"/>
+      <c r="C4" s="59"/>
+      <c r="D4" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="54"/>
-      <c r="C5" s="53"/>
-      <c r="D5" s="42" t="s">
+      <c r="B5" s="60"/>
+      <c r="C5" s="59"/>
+      <c r="D5" s="41" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="54"/>
-      <c r="C6" s="53"/>
-      <c r="D6" s="43" t="s">
+      <c r="B6" s="60"/>
+      <c r="C6" s="59"/>
+      <c r="D6" s="42" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="7" spans="2:4" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="54">
+      <c r="B7" s="60">
         <v>45684</v>
       </c>
-      <c r="C7" s="53">
+      <c r="C7" s="59">
         <v>1.5</v>
       </c>
-      <c r="D7" s="37" t="s">
+      <c r="D7" s="36" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="8" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="54"/>
-      <c r="C8" s="53"/>
-      <c r="D8" s="38" t="s">
+      <c r="B8" s="60"/>
+      <c r="C8" s="59"/>
+      <c r="D8" s="37" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="9" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="54"/>
-      <c r="C9" s="53"/>
-      <c r="D9" s="44" t="s">
+      <c r="B9" s="60"/>
+      <c r="C9" s="59"/>
+      <c r="D9" s="43" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="10" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="54"/>
-      <c r="C10" s="53"/>
-      <c r="D10" s="45" t="s">
+      <c r="B10" s="60"/>
+      <c r="C10" s="59"/>
+      <c r="D10" s="44" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="54">
+      <c r="B11" s="60">
         <v>45686</v>
       </c>
-      <c r="C11" s="53">
+      <c r="C11" s="59">
         <v>3</v>
       </c>
-      <c r="D11" s="36" t="s">
+      <c r="D11" s="35" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="12" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="54"/>
-      <c r="C12" s="53"/>
-      <c r="D12" s="36" t="s">
+      <c r="B12" s="60"/>
+      <c r="C12" s="59"/>
+      <c r="D12" s="35" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="54"/>
-      <c r="C13" s="53"/>
-      <c r="D13" s="36" t="s">
+      <c r="B13" s="60"/>
+      <c r="C13" s="59"/>
+      <c r="D13" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="54"/>
-      <c r="C14" s="53"/>
-      <c r="D14" s="46" t="s">
+      <c r="B14" s="60"/>
+      <c r="C14" s="59"/>
+      <c r="D14" s="45" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="54"/>
-      <c r="C15" s="53"/>
-      <c r="D15" s="43" t="s">
+      <c r="B15" s="60"/>
+      <c r="C15" s="59"/>
+      <c r="D15" s="42" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="54">
+      <c r="B16" s="60">
         <v>46053</v>
       </c>
-      <c r="C16" s="53">
+      <c r="C16" s="59">
         <v>4</v>
       </c>
-      <c r="D16" s="39" t="s">
+      <c r="D16" s="38" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="54"/>
-      <c r="C17" s="53"/>
-      <c r="D17" s="36" t="s">
+      <c r="B17" s="60"/>
+      <c r="C17" s="59"/>
+      <c r="D17" s="35" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="54"/>
-      <c r="C18" s="53"/>
-      <c r="D18" s="36" t="s">
+      <c r="B18" s="60"/>
+      <c r="C18" s="59"/>
+      <c r="D18" s="35" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="19" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="54"/>
-      <c r="C19" s="53"/>
-      <c r="D19" s="36" t="s">
+      <c r="B19" s="60"/>
+      <c r="C19" s="59"/>
+      <c r="D19" s="35" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="20" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="54"/>
-      <c r="C20" s="53"/>
-      <c r="D20" s="36" t="s">
+      <c r="B20" s="60"/>
+      <c r="C20" s="59"/>
+      <c r="D20" s="35" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="21" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="54"/>
-      <c r="C21" s="53"/>
-      <c r="D21" s="36" t="s">
+      <c r="B21" s="60"/>
+      <c r="C21" s="59"/>
+      <c r="D21" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="54"/>
-      <c r="C22" s="53"/>
-      <c r="D22" s="46" t="s">
+      <c r="B22" s="60"/>
+      <c r="C22" s="59"/>
+      <c r="D22" s="45" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="23" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="54"/>
-      <c r="C23" s="53"/>
-      <c r="D23" s="42" t="s">
+      <c r="B23" s="60"/>
+      <c r="C23" s="59"/>
+      <c r="D23" s="41" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="24" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="54"/>
-      <c r="C24" s="53"/>
-      <c r="D24" s="42" t="s">
+      <c r="B24" s="60"/>
+      <c r="C24" s="59"/>
+      <c r="D24" s="41" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="25" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="54"/>
-      <c r="C25" s="53"/>
-      <c r="D25" s="42" t="s">
+      <c r="B25" s="60"/>
+      <c r="C25" s="59"/>
+      <c r="D25" s="41" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="26" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="54"/>
-      <c r="C26" s="53"/>
-      <c r="D26" s="47" t="s">
+      <c r="B26" s="60"/>
+      <c r="C26" s="59"/>
+      <c r="D26" s="46" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="27" spans="2:4" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="54">
+      <c r="B27" s="60">
         <v>46054</v>
       </c>
-      <c r="C27" s="53">
+      <c r="C27" s="59">
         <v>1</v>
       </c>
-      <c r="D27" s="36" t="s">
+      <c r="D27" s="35" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="28" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="54"/>
-      <c r="C28" s="53"/>
-      <c r="D28" s="36" t="s">
+      <c r="B28" s="60"/>
+      <c r="C28" s="59"/>
+      <c r="D28" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="29" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="54"/>
-      <c r="C29" s="53"/>
-      <c r="D29" s="42" t="s">
+      <c r="B29" s="60"/>
+      <c r="C29" s="59"/>
+      <c r="D29" s="41" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="30" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="54"/>
-      <c r="C30" s="53"/>
-      <c r="D30" s="43" t="s">
+      <c r="B30" s="60"/>
+      <c r="C30" s="59"/>
+      <c r="D30" s="42" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="31" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B31" s="54">
+      <c r="B31" s="60">
         <v>46055</v>
       </c>
-      <c r="C31" s="53">
+      <c r="C31" s="59">
         <v>4</v>
       </c>
-      <c r="D31" s="40" t="s">
+      <c r="D31" s="39" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="32" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B32" s="54"/>
-      <c r="C32" s="53"/>
-      <c r="D32" s="41" t="s">
+      <c r="B32" s="60"/>
+      <c r="C32" s="59"/>
+      <c r="D32" s="40" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="33" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="54"/>
-      <c r="C33" s="53"/>
-      <c r="D33" s="41" t="s">
+      <c r="B33" s="60"/>
+      <c r="C33" s="59"/>
+      <c r="D33" s="40" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="34" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B34" s="54"/>
-      <c r="C34" s="53"/>
-      <c r="D34" s="41" t="s">
+      <c r="B34" s="60"/>
+      <c r="C34" s="59"/>
+      <c r="D34" s="40" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="35" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B35" s="54"/>
-      <c r="C35" s="53"/>
-      <c r="D35" s="48" t="s">
+      <c r="B35" s="60"/>
+      <c r="C35" s="59"/>
+      <c r="D35" s="47" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="36" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B36" s="54"/>
-      <c r="C36" s="53"/>
-      <c r="D36" s="49" t="s">
+      <c r="B36" s="60"/>
+      <c r="C36" s="59"/>
+      <c r="D36" s="48" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="37" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="54">
+      <c r="B37" s="60">
         <v>46056</v>
       </c>
-      <c r="C37" s="53">
+      <c r="C37" s="59">
         <v>3</v>
       </c>
-      <c r="D37" s="36" t="s">
+      <c r="D37" s="35" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="38" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B38" s="54"/>
-      <c r="C38" s="53"/>
-      <c r="D38" s="36" t="s">
+      <c r="B38" s="60"/>
+      <c r="C38" s="59"/>
+      <c r="D38" s="35" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="39" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B39" s="54"/>
-      <c r="C39" s="53"/>
-      <c r="D39" s="36" t="s">
+      <c r="B39" s="60"/>
+      <c r="C39" s="59"/>
+      <c r="D39" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="40" spans="2:4" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B40" s="54"/>
-      <c r="C40" s="53"/>
-      <c r="D40" s="42" t="s">
+      <c r="B40" s="60"/>
+      <c r="C40" s="59"/>
+      <c r="D40" s="41" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="41" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B41" s="54"/>
-      <c r="C41" s="53"/>
-      <c r="D41" s="43" t="s">
+      <c r="B41" s="60"/>
+      <c r="C41" s="59"/>
+      <c r="D41" s="42" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="42" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B42" s="54">
+      <c r="B42" s="60">
         <v>46057</v>
       </c>
-      <c r="C42" s="53">
+      <c r="C42" s="59">
         <v>4</v>
       </c>
-      <c r="D42" s="39" t="s">
+      <c r="D42" s="38" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="43" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B43" s="54"/>
-      <c r="C43" s="53"/>
-      <c r="D43" s="36" t="s">
+      <c r="B43" s="60"/>
+      <c r="C43" s="59"/>
+      <c r="D43" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="44" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B44" s="54"/>
-      <c r="C44" s="53"/>
-      <c r="D44" s="43" t="s">
+      <c r="B44" s="60"/>
+      <c r="C44" s="59"/>
+      <c r="D44" s="42" t="s">
         <v>23</v>
       </c>
     </row>
@@ -2129,35 +2794,35 @@
       <c r="C45" s="64">
         <v>2</v>
       </c>
-      <c r="D45" s="51" t="s">
+      <c r="D45" s="50" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="46" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B46" s="62"/>
       <c r="C46" s="65"/>
-      <c r="D46" s="50" t="s">
+      <c r="D46" s="49" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="47" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B47" s="62"/>
       <c r="C47" s="65"/>
-      <c r="D47" s="36" t="s">
+      <c r="D47" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="48" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B48" s="62"/>
       <c r="C48" s="65"/>
-      <c r="D48" s="43" t="s">
+      <c r="D48" s="42" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="49" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B49" s="63"/>
       <c r="C49" s="66"/>
-      <c r="D49" s="47" t="s">
+      <c r="D49" s="46" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2168,265 +2833,627 @@
       <c r="C50" s="64">
         <v>1.5</v>
       </c>
-      <c r="D50" s="51" t="s">
+      <c r="D50" s="50" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="51" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B51" s="62"/>
       <c r="C51" s="65"/>
-      <c r="D51" s="36" t="s">
+      <c r="D51" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="52" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B52" s="62"/>
       <c r="C52" s="65"/>
-      <c r="D52" s="43" t="s">
+      <c r="D52" s="42" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="53" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B53" s="62"/>
       <c r="C53" s="65"/>
-      <c r="D53" s="43" t="s">
+      <c r="D53" s="42" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="54" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B54" s="63"/>
       <c r="C54" s="66"/>
-      <c r="D54" s="47" t="s">
+      <c r="D54" s="46" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="55" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B55" s="52"/>
-      <c r="C55" s="52"/>
-      <c r="D55" s="60"/>
-    </row>
-    <row r="56" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B56" s="35"/>
-      <c r="C56" s="35"/>
-      <c r="D56" s="33"/>
+    <row r="55" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B55" s="61">
+        <v>46062</v>
+      </c>
+      <c r="C55" s="64">
+        <v>2</v>
+      </c>
+      <c r="D55" s="67" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="56" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B56" s="62"/>
+      <c r="C56" s="65"/>
+      <c r="D56" s="68" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="57" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B57" s="35"/>
-      <c r="C57" s="35"/>
-      <c r="D57" s="33"/>
-    </row>
-    <row r="58" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B58" s="35"/>
-      <c r="C58" s="35"/>
-      <c r="D58" s="33"/>
-    </row>
-    <row r="59" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B59" s="35"/>
-      <c r="C59" s="35"/>
-      <c r="D59" s="33"/>
-    </row>
-    <row r="60" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B60" s="35"/>
-      <c r="C60" s="35"/>
-      <c r="D60" s="33"/>
-    </row>
-    <row r="61" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B61" s="35"/>
-      <c r="C61" s="35"/>
-      <c r="D61" s="33"/>
+      <c r="B57" s="62"/>
+      <c r="C57" s="65"/>
+      <c r="D57" s="42" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="58" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B58" s="63"/>
+      <c r="C58" s="66"/>
+      <c r="D58" s="46" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="59" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B59" s="61">
+        <v>46063</v>
+      </c>
+      <c r="C59" s="64">
+        <v>3</v>
+      </c>
+      <c r="D59" s="67" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="60" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B60" s="62"/>
+      <c r="C60" s="65"/>
+      <c r="D60" s="68" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="61" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B61" s="62"/>
+      <c r="C61" s="65"/>
+      <c r="D61" s="68" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="62" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B62" s="35"/>
-      <c r="C62" s="35"/>
-      <c r="D62" s="33"/>
-    </row>
-    <row r="63" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B63" s="35"/>
-      <c r="C63" s="35"/>
-      <c r="D63" s="33"/>
-    </row>
-    <row r="64" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B64" s="35"/>
-      <c r="C64" s="35"/>
-      <c r="D64" s="33"/>
-    </row>
-    <row r="65" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B65" s="35"/>
-      <c r="C65" s="35"/>
-      <c r="D65" s="33"/>
-    </row>
-    <row r="66" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B66" s="35"/>
-      <c r="C66" s="35"/>
-      <c r="D66" s="33"/>
+      <c r="B62" s="62"/>
+      <c r="C62" s="65"/>
+      <c r="D62" s="42" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="63" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B63" s="63"/>
+      <c r="C63" s="66"/>
+      <c r="D63" s="46" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="64" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B64" s="61">
+        <v>46064</v>
+      </c>
+      <c r="C64" s="64">
+        <v>3</v>
+      </c>
+      <c r="D64" s="67" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="65" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B65" s="62"/>
+      <c r="C65" s="65"/>
+      <c r="D65" s="68" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="66" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B66" s="62"/>
+      <c r="C66" s="65"/>
+      <c r="D66" s="68" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="67" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B67" s="35"/>
-      <c r="C67" s="35"/>
-      <c r="D67" s="33"/>
-    </row>
-    <row r="68" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B68" s="35"/>
-      <c r="C68" s="35"/>
-      <c r="D68" s="33"/>
-    </row>
-    <row r="69" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B69" s="35"/>
-      <c r="C69" s="35"/>
-      <c r="D69" s="33"/>
-    </row>
-    <row r="70" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B70" s="35"/>
-      <c r="C70" s="35"/>
-      <c r="D70" s="33"/>
-    </row>
-    <row r="71" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B71" s="35"/>
-      <c r="C71" s="35"/>
-      <c r="D71" s="33"/>
+      <c r="B67" s="62"/>
+      <c r="C67" s="65"/>
+      <c r="D67" s="42" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="68" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B68" s="63"/>
+      <c r="C68" s="66"/>
+      <c r="D68" s="46" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="69" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B69" s="69">
+        <v>46066</v>
+      </c>
+      <c r="C69" s="64">
+        <v>2</v>
+      </c>
+      <c r="D69" s="67" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="70" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B70" s="70"/>
+      <c r="C70" s="65"/>
+      <c r="D70" s="68" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="71" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B71" s="70"/>
+      <c r="C71" s="65"/>
+      <c r="D71" s="68" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="72" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B72" s="35"/>
-      <c r="C72" s="35"/>
-      <c r="D72" s="33"/>
-    </row>
-    <row r="73" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B73" s="32"/>
-      <c r="C73" s="32"/>
-      <c r="D73" s="33"/>
-    </row>
-    <row r="74" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B74" s="32"/>
-      <c r="C74" s="32"/>
-      <c r="D74" s="33"/>
+      <c r="B72" s="70"/>
+      <c r="C72" s="65"/>
+      <c r="D72" s="42" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="73" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B73" s="70"/>
+      <c r="C73" s="65"/>
+      <c r="D73" s="42" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="74" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B74" s="72"/>
+      <c r="C74" s="66"/>
+      <c r="D74" s="46" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="75" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B75" s="32"/>
-      <c r="C75" s="32"/>
-      <c r="D75" s="33"/>
+      <c r="B75" s="74">
+        <v>46068</v>
+      </c>
+      <c r="C75" s="75">
+        <v>2.5</v>
+      </c>
+      <c r="D75" s="67" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="76" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B76" s="32"/>
-      <c r="C76" s="32"/>
-      <c r="D76" s="33"/>
+      <c r="B76" s="76"/>
+      <c r="C76" s="77"/>
+      <c r="D76" s="68" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="77" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B77" s="32"/>
-      <c r="C77" s="32"/>
-      <c r="D77" s="33"/>
+      <c r="B77" s="76"/>
+      <c r="C77" s="77"/>
+      <c r="D77" s="68" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="78" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B78" s="32"/>
-      <c r="C78" s="32"/>
-      <c r="D78" s="33"/>
-    </row>
-    <row r="79" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B79" s="32"/>
-      <c r="C79" s="32"/>
-      <c r="D79" s="33"/>
-    </row>
-    <row r="80" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B80" s="32"/>
-      <c r="C80" s="32"/>
-      <c r="D80" s="33"/>
-    </row>
-    <row r="81" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B81" s="32"/>
-      <c r="C81" s="32"/>
-      <c r="D81" s="33"/>
+      <c r="B78" s="76"/>
+      <c r="C78" s="77"/>
+      <c r="D78" s="68" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="79" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B79" s="76"/>
+      <c r="C79" s="77"/>
+      <c r="D79" s="42" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="80" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B80" s="76"/>
+      <c r="C80" s="77"/>
+      <c r="D80" s="42" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="81" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B81" s="78"/>
+      <c r="C81" s="79"/>
+      <c r="D81" s="46" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="82" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B82" s="32"/>
-      <c r="C82" s="32"/>
-      <c r="D82" s="33"/>
+      <c r="B82" s="74">
+        <v>46070</v>
+      </c>
+      <c r="C82" s="75">
+        <v>3</v>
+      </c>
+      <c r="D82" s="67" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="83" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B83" s="32"/>
-      <c r="C83" s="32"/>
-      <c r="D83" s="33"/>
+      <c r="B83" s="76"/>
+      <c r="C83" s="77"/>
+      <c r="D83" s="68" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="84" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B84" s="32"/>
-      <c r="C84" s="32"/>
-      <c r="D84" s="33"/>
+      <c r="B84" s="76"/>
+      <c r="C84" s="77"/>
+      <c r="D84" s="68" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="85" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B85" s="32"/>
-      <c r="C85" s="32"/>
-      <c r="D85" s="33"/>
-    </row>
-    <row r="86" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B86" s="32"/>
-      <c r="C86" s="32"/>
-      <c r="D86" s="33"/>
-    </row>
-    <row r="87" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B87" s="32"/>
-      <c r="C87" s="32"/>
-      <c r="D87" s="33"/>
-    </row>
-    <row r="88" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B88" s="32"/>
-      <c r="C88" s="32"/>
-      <c r="D88" s="33"/>
+      <c r="B85" s="76"/>
+      <c r="C85" s="77"/>
+      <c r="D85" s="68" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="86" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B86" s="76"/>
+      <c r="C86" s="77"/>
+      <c r="D86" s="42" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="87" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B87" s="76"/>
+      <c r="C87" s="77"/>
+      <c r="D87" s="42" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="88" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B88" s="78"/>
+      <c r="C88" s="79"/>
+      <c r="D88" s="46" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="89" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B89" s="32"/>
-      <c r="C89" s="32"/>
-      <c r="D89" s="33"/>
+      <c r="B89" s="74">
+        <v>46071</v>
+      </c>
+      <c r="C89" s="75">
+        <v>2</v>
+      </c>
+      <c r="D89" s="67" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="90" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B90" s="32"/>
-      <c r="C90" s="32"/>
-      <c r="D90" s="33"/>
+      <c r="B90" s="76"/>
+      <c r="C90" s="77"/>
+      <c r="D90" s="68" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="91" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B91" s="32"/>
-      <c r="C91" s="32"/>
-      <c r="D91" s="33"/>
-    </row>
-    <row r="92" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B92" s="32"/>
-      <c r="C92" s="32"/>
-      <c r="D92" s="33"/>
-    </row>
-    <row r="93" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B93" s="32"/>
-      <c r="C93" s="32"/>
-      <c r="D93" s="33"/>
+      <c r="B91" s="76"/>
+      <c r="C91" s="77"/>
+      <c r="D91" s="68" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="92" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B92" s="76"/>
+      <c r="C92" s="77"/>
+      <c r="D92" s="42" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="93" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B93" s="78"/>
+      <c r="C93" s="79"/>
+      <c r="D93" s="46" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="94" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B94" s="32"/>
-      <c r="C94" s="32"/>
-      <c r="D94" s="33"/>
+      <c r="B94" s="74">
+        <v>46074</v>
+      </c>
+      <c r="C94" s="75">
+        <v>3</v>
+      </c>
+      <c r="D94" s="80" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="95" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B95" s="32"/>
-      <c r="C95" s="32"/>
-      <c r="D95" s="33"/>
-    </row>
-    <row r="96" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B96" s="32"/>
-      <c r="C96" s="32"/>
-      <c r="D96" s="33"/>
+      <c r="B95" s="76"/>
+      <c r="C95" s="77"/>
+      <c r="D95" s="81" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="96" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B96" s="78"/>
+      <c r="C96" s="79"/>
+      <c r="D96" s="46" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="97" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B97" s="32"/>
-      <c r="C97" s="32"/>
-      <c r="D97" s="33"/>
+      <c r="B97" s="74">
+        <v>46075</v>
+      </c>
+      <c r="C97" s="75">
+        <v>3</v>
+      </c>
+      <c r="D97" s="67" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="98" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B98" s="32"/>
-      <c r="C98" s="32"/>
-      <c r="D98" s="33"/>
+      <c r="B98" s="76"/>
+      <c r="C98" s="77"/>
+      <c r="D98" s="68" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="99" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B99" s="32"/>
-      <c r="C99" s="32"/>
-      <c r="D99" s="33"/>
+      <c r="B99" s="76"/>
+      <c r="C99" s="77"/>
+      <c r="D99" s="68" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="100" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B100" s="78"/>
+      <c r="C100" s="79"/>
+      <c r="D100" s="46" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="101" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B101" s="73">
+        <v>46076</v>
+      </c>
+      <c r="C101" s="71">
+        <v>4</v>
+      </c>
+      <c r="D101" s="67" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="102" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B102" s="32"/>
+      <c r="C102" s="32"/>
+      <c r="D102" s="33"/>
+    </row>
+    <row r="103" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B103" s="71"/>
+      <c r="C103" s="71"/>
+      <c r="D103" s="51"/>
+    </row>
+    <row r="104" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B104" s="32"/>
+      <c r="C104" s="32"/>
+      <c r="D104" s="33"/>
+    </row>
+    <row r="105" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B105" s="32"/>
+      <c r="C105" s="32"/>
+      <c r="D105" s="33"/>
+    </row>
+    <row r="106" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B106" s="71"/>
+      <c r="C106" s="71"/>
+      <c r="D106" s="51"/>
+    </row>
+    <row r="107" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B107" s="32"/>
+      <c r="C107" s="32"/>
+      <c r="D107" s="33"/>
+    </row>
+    <row r="108" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B108" s="32"/>
+      <c r="C108" s="32"/>
+      <c r="D108" s="33"/>
+    </row>
+    <row r="109" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B109" s="71"/>
+      <c r="C109" s="71"/>
+      <c r="D109" s="51"/>
+    </row>
+    <row r="110" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B110" s="32"/>
+      <c r="C110" s="32"/>
+      <c r="D110" s="33"/>
+    </row>
+    <row r="111" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B111" s="32"/>
+      <c r="C111" s="32"/>
+      <c r="D111" s="33"/>
+    </row>
+    <row r="112" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B112" s="71"/>
+      <c r="C112" s="71"/>
+      <c r="D112" s="51"/>
+    </row>
+    <row r="113" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B113" s="32"/>
+      <c r="C113" s="32"/>
+      <c r="D113" s="33"/>
+    </row>
+    <row r="114" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B114" s="32"/>
+      <c r="C114" s="32"/>
+      <c r="D114" s="33"/>
+    </row>
+    <row r="115" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B115" s="71"/>
+      <c r="C115" s="71"/>
+      <c r="D115" s="51"/>
+    </row>
+    <row r="116" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B116" s="32"/>
+      <c r="C116" s="32"/>
+      <c r="D116" s="33"/>
+    </row>
+    <row r="117" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B117" s="32"/>
+      <c r="C117" s="32"/>
+      <c r="D117" s="33"/>
+    </row>
+    <row r="118" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B118" s="71"/>
+      <c r="C118" s="71"/>
+      <c r="D118" s="51"/>
+    </row>
+    <row r="119" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B119" s="32"/>
+      <c r="C119" s="32"/>
+      <c r="D119" s="33"/>
+    </row>
+    <row r="120" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B120" s="32"/>
+      <c r="C120" s="32"/>
+      <c r="D120" s="33"/>
+    </row>
+    <row r="121" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B121" s="71"/>
+      <c r="C121" s="71"/>
+      <c r="D121" s="51"/>
+    </row>
+    <row r="122" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B122" s="32"/>
+      <c r="C122" s="32"/>
+      <c r="D122" s="33"/>
+    </row>
+    <row r="123" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B123" s="32"/>
+      <c r="C123" s="32"/>
+      <c r="D123" s="33"/>
+    </row>
+    <row r="124" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B124" s="71"/>
+      <c r="C124" s="71"/>
+      <c r="D124" s="51"/>
+    </row>
+    <row r="125" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B125" s="32"/>
+      <c r="C125" s="32"/>
+      <c r="D125" s="33"/>
+    </row>
+    <row r="126" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B126" s="32"/>
+      <c r="C126" s="32"/>
+      <c r="D126" s="33"/>
+    </row>
+    <row r="127" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B127" s="71"/>
+      <c r="C127" s="71"/>
+      <c r="D127" s="51"/>
+    </row>
+    <row r="128" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B128" s="32"/>
+      <c r="C128" s="32"/>
+      <c r="D128" s="33"/>
+    </row>
+    <row r="129" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B129" s="32"/>
+      <c r="C129" s="32"/>
+      <c r="D129" s="33"/>
+    </row>
+    <row r="130" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B130" s="71"/>
+      <c r="C130" s="71"/>
+      <c r="D130" s="51"/>
+    </row>
+    <row r="131" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B131" s="32"/>
+      <c r="C131" s="32"/>
+      <c r="D131" s="33"/>
+    </row>
+    <row r="132" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B132" s="32"/>
+      <c r="C132" s="32"/>
+      <c r="D132" s="33"/>
+    </row>
+    <row r="133" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B133" s="71"/>
+      <c r="C133" s="71"/>
+      <c r="D133" s="51"/>
+    </row>
+    <row r="134" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B134" s="32"/>
+      <c r="C134" s="32"/>
+      <c r="D134" s="33"/>
+    </row>
+    <row r="135" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B135" s="32"/>
+      <c r="C135" s="32"/>
+      <c r="D135" s="33"/>
+    </row>
+    <row r="136" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B136" s="71"/>
+      <c r="C136" s="71"/>
+      <c r="D136" s="51"/>
+    </row>
+    <row r="137" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B137" s="32"/>
+      <c r="C137" s="32"/>
+      <c r="D137" s="33"/>
+    </row>
+    <row r="138" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B138" s="32"/>
+      <c r="C138" s="32"/>
+      <c r="D138" s="33"/>
+    </row>
+    <row r="139" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B139" s="71"/>
+      <c r="C139" s="71"/>
+      <c r="D139" s="51"/>
+    </row>
+    <row r="140" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B140" s="32"/>
+      <c r="C140" s="32"/>
+      <c r="D140" s="33"/>
+    </row>
+    <row r="141" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B141" s="32"/>
+      <c r="C141" s="32"/>
+      <c r="D141" s="33"/>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="38">
+    <mergeCell ref="B97:B100"/>
+    <mergeCell ref="C97:C100"/>
+    <mergeCell ref="B82:B88"/>
+    <mergeCell ref="C82:C88"/>
+    <mergeCell ref="B89:B93"/>
+    <mergeCell ref="C89:C93"/>
+    <mergeCell ref="B94:B96"/>
+    <mergeCell ref="C94:C96"/>
+    <mergeCell ref="B64:B68"/>
+    <mergeCell ref="C64:C68"/>
+    <mergeCell ref="B69:B74"/>
+    <mergeCell ref="C69:C74"/>
+    <mergeCell ref="B75:B81"/>
+    <mergeCell ref="C75:C81"/>
+    <mergeCell ref="B55:B58"/>
+    <mergeCell ref="C55:C58"/>
+    <mergeCell ref="B59:B63"/>
+    <mergeCell ref="C59:C63"/>
     <mergeCell ref="B45:B49"/>
     <mergeCell ref="C45:C49"/>
     <mergeCell ref="B50:B54"/>
@@ -2457,7 +3484,7 @@
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
   </sheetPr>
-  <dimension ref="D2:R11"/>
+  <dimension ref="D2:R23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="8.88671875" style="2"/>
@@ -2469,38 +3496,42 @@
     <col min="18" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="4:18" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="4:18" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D2" s="52" t="s">
+        <v>62</v>
+      </c>
+    </row>
     <row r="3" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D3" s="58" t="s">
+      <c r="D3" s="57" t="s">
         <v>8</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F3" s="55" t="s">
+      <c r="F3" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="G3" s="56"/>
-      <c r="H3" s="56"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="55" t="s">
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="56"/>
+      <c r="J3" s="54" t="s">
         <v>2</v>
       </c>
-      <c r="K3" s="56"/>
-      <c r="L3" s="56"/>
-      <c r="M3" s="57"/>
-      <c r="N3" s="55" t="s">
+      <c r="K3" s="55"/>
+      <c r="L3" s="55"/>
+      <c r="M3" s="56"/>
+      <c r="N3" s="54" t="s">
         <v>3</v>
       </c>
-      <c r="O3" s="56"/>
-      <c r="P3" s="56"/>
-      <c r="Q3" s="57"/>
+      <c r="O3" s="55"/>
+      <c r="P3" s="55"/>
+      <c r="Q3" s="56"/>
       <c r="R3" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="4:18" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D4" s="59"/>
+      <c r="D4" s="58"/>
       <c r="E4" s="4" t="s">
         <v>4</v>
       </c>
@@ -2665,12 +3696,216 @@
       <c r="Q11" s="14"/>
       <c r="R11" s="11"/>
     </row>
+    <row r="14" spans="4:18" s="53" customFormat="1" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D14" s="52" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="15" spans="4:18" x14ac:dyDescent="0.3">
+      <c r="D15" s="57" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="F15" s="54" t="s">
+        <v>1</v>
+      </c>
+      <c r="G15" s="55"/>
+      <c r="H15" s="55"/>
+      <c r="I15" s="56"/>
+      <c r="J15" s="54" t="s">
+        <v>2</v>
+      </c>
+      <c r="K15" s="55"/>
+      <c r="L15" s="55"/>
+      <c r="M15" s="56"/>
+      <c r="N15" s="54" t="s">
+        <v>3</v>
+      </c>
+      <c r="O15" s="55"/>
+      <c r="P15" s="55"/>
+      <c r="Q15" s="56"/>
+      <c r="R15" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="4:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D16" s="58"/>
+      <c r="E16" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="J16" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="L16" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M16" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="N16" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="O16" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="P16" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q16" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="R16" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="4:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D17" s="27" t="s">
+        <v>9</v>
+      </c>
+      <c r="E17" s="8"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="24"/>
+      <c r="K17" s="16"/>
+      <c r="L17" s="16"/>
+      <c r="M17" s="17"/>
+      <c r="N17" s="9"/>
+      <c r="Q17" s="10"/>
+      <c r="R17" s="8"/>
+    </row>
+    <row r="18" spans="4:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D18" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" s="8"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="19"/>
+      <c r="H18" s="19"/>
+      <c r="I18" s="20"/>
+      <c r="J18" s="25"/>
+      <c r="K18" s="19"/>
+      <c r="L18" s="19"/>
+      <c r="M18" s="20"/>
+      <c r="N18" s="9"/>
+      <c r="Q18" s="10"/>
+      <c r="R18" s="8"/>
+    </row>
+    <row r="19" spans="4:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D19" s="28" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" s="8"/>
+      <c r="F19" s="18"/>
+      <c r="G19" s="19"/>
+      <c r="H19" s="19"/>
+      <c r="I19" s="20"/>
+      <c r="J19" s="25"/>
+      <c r="K19" s="19"/>
+      <c r="L19" s="19"/>
+      <c r="M19" s="20"/>
+      <c r="N19" s="9"/>
+      <c r="Q19" s="10"/>
+      <c r="R19" s="8"/>
+    </row>
+    <row r="20" spans="4:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D20" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="E20" s="8"/>
+      <c r="F20" s="18"/>
+      <c r="G20" s="19"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="20"/>
+      <c r="J20" s="25"/>
+      <c r="K20" s="19"/>
+      <c r="L20" s="19"/>
+      <c r="M20" s="20"/>
+      <c r="N20" s="9"/>
+      <c r="Q20" s="10"/>
+      <c r="R20" s="8"/>
+    </row>
+    <row r="21" spans="4:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D21" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" s="8"/>
+      <c r="F21" s="18"/>
+      <c r="G21" s="19"/>
+      <c r="H21" s="19"/>
+      <c r="I21" s="20"/>
+      <c r="J21" s="25"/>
+      <c r="K21" s="19"/>
+      <c r="L21" s="19"/>
+      <c r="M21" s="20"/>
+      <c r="N21" s="9"/>
+      <c r="Q21" s="10"/>
+      <c r="R21" s="8"/>
+    </row>
+    <row r="22" spans="4:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D22" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="E22" s="8"/>
+      <c r="F22" s="18"/>
+      <c r="G22" s="19"/>
+      <c r="H22" s="19"/>
+      <c r="I22" s="20"/>
+      <c r="J22" s="25"/>
+      <c r="K22" s="19"/>
+      <c r="L22" s="19"/>
+      <c r="M22" s="20"/>
+      <c r="N22" s="9"/>
+      <c r="Q22" s="10"/>
+      <c r="R22" s="8"/>
+    </row>
+    <row r="23" spans="4:18" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D23" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="E23" s="11"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="22"/>
+      <c r="H23" s="22"/>
+      <c r="I23" s="23"/>
+      <c r="J23" s="26"/>
+      <c r="K23" s="22"/>
+      <c r="L23" s="22"/>
+      <c r="M23" s="23"/>
+      <c r="N23" s="12"/>
+      <c r="O23" s="13"/>
+      <c r="P23" s="13"/>
+      <c r="Q23" s="14"/>
+      <c r="R23" s="11"/>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="8">
     <mergeCell ref="F3:I3"/>
     <mergeCell ref="J3:M3"/>
     <mergeCell ref="N3:Q3"/>
     <mergeCell ref="D3:D4"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="J15:M15"/>
+    <mergeCell ref="N15:Q15"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
built front end for dashboard
</commit_message>
<xml_diff>
--- a/DocumentsAndReports/0. WorkLog_Charts.xlsx
+++ b/DocumentsAndReports/0. WorkLog_Charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qhung\Videos\CSIS4495 - Applied Research  Project\W26_4495_S2_HughT\DocumentsAndReports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FF5E6F1-94D2-49BB-B230-C471500E2002}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33A14A7E-A6E3-4AC9-B75D-E2E3ACE017F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30720" yWindow="1920" windowWidth="21600" windowHeight="11235" xr2:uid="{E067A1E6-0DC4-42DD-AAF8-D95EFF7A112F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E067A1E6-0DC4-42DD-AAF8-D95EFF7A112F}"/>
   </bookViews>
   <sheets>
     <sheet name="Work_Log" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="91">
   <si>
     <t>January</t>
   </si>
@@ -352,6 +352,18 @@
   </si>
   <si>
     <t>THE ADJUSTED PLAN</t>
+  </si>
+  <si>
+    <t>- Build front-end for dashboard</t>
+  </si>
+  <si>
+    <t>- Reseached on html navigation in FastAPI</t>
+  </si>
+  <si>
+    <t>“why cannot navigate between html pages”</t>
+  </si>
+  <si>
+    <t>“how to do html navigation in fastApi?”</t>
   </si>
 </sst>
 </file>
@@ -463,7 +475,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="37">
+  <borders count="38">
     <border>
       <left/>
       <right/>
@@ -905,11 +917,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1020,6 +1045,75 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="35" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="36" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="33" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="34" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1035,74 +1129,14 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="15" fontId="7" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="15" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="15" fontId="7" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="15" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="35" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="37" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="36" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="33" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="34" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2462,10 +2496,10 @@
       </c>
     </row>
     <row r="3" spans="2:4" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="60">
+      <c r="B3" s="76">
         <v>45683</v>
       </c>
-      <c r="C3" s="59">
+      <c r="C3" s="75">
         <v>2</v>
       </c>
       <c r="D3" s="35" t="s">
@@ -2473,31 +2507,31 @@
       </c>
     </row>
     <row r="4" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="60"/>
-      <c r="C4" s="59"/>
+      <c r="B4" s="76"/>
+      <c r="C4" s="75"/>
       <c r="D4" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="60"/>
-      <c r="C5" s="59"/>
+      <c r="B5" s="76"/>
+      <c r="C5" s="75"/>
       <c r="D5" s="41" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="60"/>
-      <c r="C6" s="59"/>
+      <c r="B6" s="76"/>
+      <c r="C6" s="75"/>
       <c r="D6" s="42" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="7" spans="2:4" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="60">
+      <c r="B7" s="76">
         <v>45684</v>
       </c>
-      <c r="C7" s="59">
+      <c r="C7" s="75">
         <v>1.5</v>
       </c>
       <c r="D7" s="36" t="s">
@@ -2505,31 +2539,31 @@
       </c>
     </row>
     <row r="8" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="60"/>
-      <c r="C8" s="59"/>
+      <c r="B8" s="76"/>
+      <c r="C8" s="75"/>
       <c r="D8" s="37" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="9" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="60"/>
-      <c r="C9" s="59"/>
+      <c r="B9" s="76"/>
+      <c r="C9" s="75"/>
       <c r="D9" s="43" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="10" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="60"/>
-      <c r="C10" s="59"/>
+      <c r="B10" s="76"/>
+      <c r="C10" s="75"/>
       <c r="D10" s="44" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="60">
+      <c r="B11" s="76">
         <v>45686</v>
       </c>
-      <c r="C11" s="59">
+      <c r="C11" s="75">
         <v>3</v>
       </c>
       <c r="D11" s="35" t="s">
@@ -2537,38 +2571,38 @@
       </c>
     </row>
     <row r="12" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="60"/>
-      <c r="C12" s="59"/>
+      <c r="B12" s="76"/>
+      <c r="C12" s="75"/>
       <c r="D12" s="35" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="60"/>
-      <c r="C13" s="59"/>
+      <c r="B13" s="76"/>
+      <c r="C13" s="75"/>
       <c r="D13" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="60"/>
-      <c r="C14" s="59"/>
+      <c r="B14" s="76"/>
+      <c r="C14" s="75"/>
       <c r="D14" s="45" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="60"/>
-      <c r="C15" s="59"/>
+      <c r="B15" s="76"/>
+      <c r="C15" s="75"/>
       <c r="D15" s="42" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="60">
+      <c r="B16" s="76">
         <v>46053</v>
       </c>
-      <c r="C16" s="59">
+      <c r="C16" s="75">
         <v>4</v>
       </c>
       <c r="D16" s="38" t="s">
@@ -2576,80 +2610,80 @@
       </c>
     </row>
     <row r="17" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="60"/>
-      <c r="C17" s="59"/>
+      <c r="B17" s="76"/>
+      <c r="C17" s="75"/>
       <c r="D17" s="35" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="60"/>
-      <c r="C18" s="59"/>
+      <c r="B18" s="76"/>
+      <c r="C18" s="75"/>
       <c r="D18" s="35" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="19" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="60"/>
-      <c r="C19" s="59"/>
+      <c r="B19" s="76"/>
+      <c r="C19" s="75"/>
       <c r="D19" s="35" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="20" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="60"/>
-      <c r="C20" s="59"/>
+      <c r="B20" s="76"/>
+      <c r="C20" s="75"/>
       <c r="D20" s="35" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="21" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="60"/>
-      <c r="C21" s="59"/>
+      <c r="B21" s="76"/>
+      <c r="C21" s="75"/>
       <c r="D21" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="60"/>
-      <c r="C22" s="59"/>
+      <c r="B22" s="76"/>
+      <c r="C22" s="75"/>
       <c r="D22" s="45" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="23" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="60"/>
-      <c r="C23" s="59"/>
+      <c r="B23" s="76"/>
+      <c r="C23" s="75"/>
       <c r="D23" s="41" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="24" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="60"/>
-      <c r="C24" s="59"/>
+      <c r="B24" s="76"/>
+      <c r="C24" s="75"/>
       <c r="D24" s="41" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="25" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="60"/>
-      <c r="C25" s="59"/>
+      <c r="B25" s="76"/>
+      <c r="C25" s="75"/>
       <c r="D25" s="41" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="26" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="60"/>
-      <c r="C26" s="59"/>
+      <c r="B26" s="76"/>
+      <c r="C26" s="75"/>
       <c r="D26" s="46" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="27" spans="2:4" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="60">
+      <c r="B27" s="76">
         <v>46054</v>
       </c>
-      <c r="C27" s="59">
+      <c r="C27" s="75">
         <v>1</v>
       </c>
       <c r="D27" s="35" t="s">
@@ -2657,31 +2691,31 @@
       </c>
     </row>
     <row r="28" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="60"/>
-      <c r="C28" s="59"/>
+      <c r="B28" s="76"/>
+      <c r="C28" s="75"/>
       <c r="D28" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="29" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="60"/>
-      <c r="C29" s="59"/>
+      <c r="B29" s="76"/>
+      <c r="C29" s="75"/>
       <c r="D29" s="41" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="30" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="60"/>
-      <c r="C30" s="59"/>
+      <c r="B30" s="76"/>
+      <c r="C30" s="75"/>
       <c r="D30" s="42" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="31" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B31" s="60">
+      <c r="B31" s="76">
         <v>46055</v>
       </c>
-      <c r="C31" s="59">
+      <c r="C31" s="75">
         <v>4</v>
       </c>
       <c r="D31" s="39" t="s">
@@ -2689,45 +2723,45 @@
       </c>
     </row>
     <row r="32" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B32" s="60"/>
-      <c r="C32" s="59"/>
+      <c r="B32" s="76"/>
+      <c r="C32" s="75"/>
       <c r="D32" s="40" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="33" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="60"/>
-      <c r="C33" s="59"/>
+      <c r="B33" s="76"/>
+      <c r="C33" s="75"/>
       <c r="D33" s="40" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="34" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B34" s="60"/>
-      <c r="C34" s="59"/>
+      <c r="B34" s="76"/>
+      <c r="C34" s="75"/>
       <c r="D34" s="40" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="35" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B35" s="60"/>
-      <c r="C35" s="59"/>
+      <c r="B35" s="76"/>
+      <c r="C35" s="75"/>
       <c r="D35" s="47" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="36" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B36" s="60"/>
-      <c r="C36" s="59"/>
+      <c r="B36" s="76"/>
+      <c r="C36" s="75"/>
       <c r="D36" s="48" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="37" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="60">
+      <c r="B37" s="76">
         <v>46056</v>
       </c>
-      <c r="C37" s="59">
+      <c r="C37" s="75">
         <v>3</v>
       </c>
       <c r="D37" s="35" t="s">
@@ -2735,38 +2769,38 @@
       </c>
     </row>
     <row r="38" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B38" s="60"/>
-      <c r="C38" s="59"/>
+      <c r="B38" s="76"/>
+      <c r="C38" s="75"/>
       <c r="D38" s="35" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="39" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B39" s="60"/>
-      <c r="C39" s="59"/>
+      <c r="B39" s="76"/>
+      <c r="C39" s="75"/>
       <c r="D39" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="40" spans="2:4" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B40" s="60"/>
-      <c r="C40" s="59"/>
+      <c r="B40" s="76"/>
+      <c r="C40" s="75"/>
       <c r="D40" s="41" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="41" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B41" s="60"/>
-      <c r="C41" s="59"/>
+      <c r="B41" s="76"/>
+      <c r="C41" s="75"/>
       <c r="D41" s="42" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="42" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B42" s="60">
+      <c r="B42" s="76">
         <v>46057</v>
       </c>
-      <c r="C42" s="59">
+      <c r="C42" s="75">
         <v>4</v>
       </c>
       <c r="D42" s="38" t="s">
@@ -2774,24 +2808,24 @@
       </c>
     </row>
     <row r="43" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B43" s="60"/>
-      <c r="C43" s="59"/>
+      <c r="B43" s="76"/>
+      <c r="C43" s="75"/>
       <c r="D43" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="44" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B44" s="60"/>
-      <c r="C44" s="59"/>
+      <c r="B44" s="76"/>
+      <c r="C44" s="75"/>
       <c r="D44" s="42" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="45" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B45" s="61">
+      <c r="B45" s="66">
         <v>46059</v>
       </c>
-      <c r="C45" s="64">
+      <c r="C45" s="69">
         <v>2</v>
       </c>
       <c r="D45" s="50" t="s">
@@ -2799,38 +2833,38 @@
       </c>
     </row>
     <row r="46" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B46" s="62"/>
-      <c r="C46" s="65"/>
+      <c r="B46" s="67"/>
+      <c r="C46" s="70"/>
       <c r="D46" s="49" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="47" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B47" s="62"/>
-      <c r="C47" s="65"/>
+      <c r="B47" s="67"/>
+      <c r="C47" s="70"/>
       <c r="D47" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="48" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B48" s="62"/>
-      <c r="C48" s="65"/>
+      <c r="B48" s="67"/>
+      <c r="C48" s="70"/>
       <c r="D48" s="42" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="49" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B49" s="63"/>
-      <c r="C49" s="66"/>
+      <c r="B49" s="68"/>
+      <c r="C49" s="71"/>
       <c r="D49" s="46" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="50" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B50" s="61">
+      <c r="B50" s="66">
         <v>46061</v>
       </c>
-      <c r="C50" s="64">
+      <c r="C50" s="69">
         <v>1.5</v>
       </c>
       <c r="D50" s="50" t="s">
@@ -2838,426 +2872,440 @@
       </c>
     </row>
     <row r="51" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B51" s="62"/>
-      <c r="C51" s="65"/>
+      <c r="B51" s="67"/>
+      <c r="C51" s="70"/>
       <c r="D51" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="52" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B52" s="62"/>
-      <c r="C52" s="65"/>
+      <c r="B52" s="67"/>
+      <c r="C52" s="70"/>
       <c r="D52" s="42" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="53" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B53" s="62"/>
-      <c r="C53" s="65"/>
+      <c r="B53" s="67"/>
+      <c r="C53" s="70"/>
       <c r="D53" s="42" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="54" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B54" s="63"/>
-      <c r="C54" s="66"/>
+      <c r="B54" s="68"/>
+      <c r="C54" s="71"/>
       <c r="D54" s="46" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="55" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="61">
+      <c r="B55" s="66">
         <v>46062</v>
       </c>
-      <c r="C55" s="64">
+      <c r="C55" s="69">
         <v>2</v>
       </c>
-      <c r="D55" s="67" t="s">
+      <c r="D55" s="54" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="56" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B56" s="62"/>
-      <c r="C56" s="65"/>
-      <c r="D56" s="68" t="s">
+      <c r="B56" s="67"/>
+      <c r="C56" s="70"/>
+      <c r="D56" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="57" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B57" s="62"/>
-      <c r="C57" s="65"/>
+      <c r="B57" s="67"/>
+      <c r="C57" s="70"/>
       <c r="D57" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="58" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B58" s="63"/>
-      <c r="C58" s="66"/>
+      <c r="B58" s="68"/>
+      <c r="C58" s="71"/>
       <c r="D58" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="59" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="61">
+      <c r="B59" s="66">
         <v>46063</v>
       </c>
-      <c r="C59" s="64">
+      <c r="C59" s="69">
         <v>3</v>
       </c>
-      <c r="D59" s="67" t="s">
+      <c r="D59" s="54" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="60" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B60" s="62"/>
-      <c r="C60" s="65"/>
-      <c r="D60" s="68" t="s">
+      <c r="B60" s="67"/>
+      <c r="C60" s="70"/>
+      <c r="D60" s="55" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="61" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B61" s="62"/>
-      <c r="C61" s="65"/>
-      <c r="D61" s="68" t="s">
+      <c r="B61" s="67"/>
+      <c r="C61" s="70"/>
+      <c r="D61" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="62" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B62" s="62"/>
-      <c r="C62" s="65"/>
+      <c r="B62" s="67"/>
+      <c r="C62" s="70"/>
       <c r="D62" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="63" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B63" s="63"/>
-      <c r="C63" s="66"/>
+      <c r="B63" s="68"/>
+      <c r="C63" s="71"/>
       <c r="D63" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="64" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B64" s="61">
+      <c r="B64" s="66">
         <v>46064</v>
       </c>
-      <c r="C64" s="64">
+      <c r="C64" s="69">
         <v>3</v>
       </c>
-      <c r="D64" s="67" t="s">
+      <c r="D64" s="54" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="65" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B65" s="62"/>
-      <c r="C65" s="65"/>
-      <c r="D65" s="68" t="s">
+      <c r="B65" s="67"/>
+      <c r="C65" s="70"/>
+      <c r="D65" s="55" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="66" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B66" s="62"/>
-      <c r="C66" s="65"/>
-      <c r="D66" s="68" t="s">
+      <c r="B66" s="67"/>
+      <c r="C66" s="70"/>
+      <c r="D66" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="67" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B67" s="62"/>
-      <c r="C67" s="65"/>
+      <c r="B67" s="67"/>
+      <c r="C67" s="70"/>
       <c r="D67" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="68" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B68" s="63"/>
-      <c r="C68" s="66"/>
+      <c r="B68" s="68"/>
+      <c r="C68" s="71"/>
       <c r="D68" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="69" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B69" s="69">
+      <c r="B69" s="72">
         <v>46066</v>
       </c>
-      <c r="C69" s="64">
+      <c r="C69" s="69">
         <v>2</v>
       </c>
-      <c r="D69" s="67" t="s">
+      <c r="D69" s="54" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="70" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B70" s="70"/>
-      <c r="C70" s="65"/>
-      <c r="D70" s="68" t="s">
+      <c r="B70" s="73"/>
+      <c r="C70" s="70"/>
+      <c r="D70" s="55" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="71" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B71" s="70"/>
-      <c r="C71" s="65"/>
-      <c r="D71" s="68" t="s">
+      <c r="B71" s="73"/>
+      <c r="C71" s="70"/>
+      <c r="D71" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="72" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B72" s="70"/>
-      <c r="C72" s="65"/>
+      <c r="B72" s="73"/>
+      <c r="C72" s="70"/>
       <c r="D72" s="42" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="73" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B73" s="70"/>
-      <c r="C73" s="65"/>
+      <c r="B73" s="73"/>
+      <c r="C73" s="70"/>
       <c r="D73" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="74" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B74" s="72"/>
-      <c r="C74" s="66"/>
+      <c r="B74" s="74"/>
+      <c r="C74" s="71"/>
       <c r="D74" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="75" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B75" s="74">
+      <c r="B75" s="60">
         <v>46068</v>
       </c>
-      <c r="C75" s="75">
+      <c r="C75" s="63">
         <v>2.5</v>
       </c>
-      <c r="D75" s="67" t="s">
+      <c r="D75" s="54" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="76" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B76" s="76"/>
-      <c r="C76" s="77"/>
-      <c r="D76" s="68" t="s">
+      <c r="B76" s="61"/>
+      <c r="C76" s="64"/>
+      <c r="D76" s="55" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="77" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B77" s="76"/>
-      <c r="C77" s="77"/>
-      <c r="D77" s="68" t="s">
+      <c r="B77" s="61"/>
+      <c r="C77" s="64"/>
+      <c r="D77" s="55" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="78" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B78" s="76"/>
-      <c r="C78" s="77"/>
-      <c r="D78" s="68" t="s">
+      <c r="B78" s="61"/>
+      <c r="C78" s="64"/>
+      <c r="D78" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="79" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B79" s="76"/>
-      <c r="C79" s="77"/>
+      <c r="B79" s="61"/>
+      <c r="C79" s="64"/>
       <c r="D79" s="42" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="80" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B80" s="76"/>
-      <c r="C80" s="77"/>
+      <c r="B80" s="61"/>
+      <c r="C80" s="64"/>
       <c r="D80" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="81" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B81" s="78"/>
-      <c r="C81" s="79"/>
+      <c r="B81" s="62"/>
+      <c r="C81" s="65"/>
       <c r="D81" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="82" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B82" s="74">
+      <c r="B82" s="60">
         <v>46070</v>
       </c>
-      <c r="C82" s="75">
+      <c r="C82" s="63">
         <v>3</v>
       </c>
-      <c r="D82" s="67" t="s">
+      <c r="D82" s="54" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="83" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B83" s="76"/>
-      <c r="C83" s="77"/>
-      <c r="D83" s="68" t="s">
+      <c r="B83" s="61"/>
+      <c r="C83" s="64"/>
+      <c r="D83" s="55" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="84" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B84" s="76"/>
-      <c r="C84" s="77"/>
-      <c r="D84" s="68" t="s">
+      <c r="B84" s="61"/>
+      <c r="C84" s="64"/>
+      <c r="D84" s="55" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="85" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B85" s="76"/>
-      <c r="C85" s="77"/>
-      <c r="D85" s="68" t="s">
+      <c r="B85" s="61"/>
+      <c r="C85" s="64"/>
+      <c r="D85" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="86" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B86" s="76"/>
-      <c r="C86" s="77"/>
+      <c r="B86" s="61"/>
+      <c r="C86" s="64"/>
       <c r="D86" s="42" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="87" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B87" s="76"/>
-      <c r="C87" s="77"/>
+      <c r="B87" s="61"/>
+      <c r="C87" s="64"/>
       <c r="D87" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="88" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B88" s="78"/>
-      <c r="C88" s="79"/>
+      <c r="B88" s="62"/>
+      <c r="C88" s="65"/>
       <c r="D88" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="89" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B89" s="74">
+      <c r="B89" s="60">
         <v>46071</v>
       </c>
-      <c r="C89" s="75">
+      <c r="C89" s="63">
         <v>2</v>
       </c>
-      <c r="D89" s="67" t="s">
+      <c r="D89" s="54" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="90" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B90" s="76"/>
-      <c r="C90" s="77"/>
-      <c r="D90" s="68" t="s">
+      <c r="B90" s="61"/>
+      <c r="C90" s="64"/>
+      <c r="D90" s="55" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="91" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B91" s="76"/>
-      <c r="C91" s="77"/>
-      <c r="D91" s="68" t="s">
+      <c r="B91" s="61"/>
+      <c r="C91" s="64"/>
+      <c r="D91" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="92" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B92" s="76"/>
-      <c r="C92" s="77"/>
+      <c r="B92" s="61"/>
+      <c r="C92" s="64"/>
       <c r="D92" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="93" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B93" s="78"/>
-      <c r="C93" s="79"/>
+      <c r="B93" s="62"/>
+      <c r="C93" s="65"/>
       <c r="D93" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="94" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B94" s="74">
+      <c r="B94" s="60">
         <v>46074</v>
       </c>
-      <c r="C94" s="75">
+      <c r="C94" s="63">
         <v>3</v>
       </c>
-      <c r="D94" s="80" t="s">
+      <c r="D94" s="58" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="95" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B95" s="76"/>
-      <c r="C95" s="77"/>
-      <c r="D95" s="81" t="s">
+      <c r="B95" s="61"/>
+      <c r="C95" s="64"/>
+      <c r="D95" s="59" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="96" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B96" s="78"/>
-      <c r="C96" s="79"/>
+      <c r="B96" s="62"/>
+      <c r="C96" s="65"/>
       <c r="D96" s="46" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="97" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B97" s="74">
+      <c r="B97" s="60">
         <v>46075</v>
       </c>
-      <c r="C97" s="75">
+      <c r="C97" s="63">
         <v>3</v>
       </c>
-      <c r="D97" s="67" t="s">
+      <c r="D97" s="54" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="98" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B98" s="76"/>
-      <c r="C98" s="77"/>
-      <c r="D98" s="68" t="s">
+      <c r="B98" s="61"/>
+      <c r="C98" s="64"/>
+      <c r="D98" s="55" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="99" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B99" s="76"/>
-      <c r="C99" s="77"/>
-      <c r="D99" s="68" t="s">
+      <c r="B99" s="61"/>
+      <c r="C99" s="64"/>
+      <c r="D99" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="100" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B100" s="78"/>
-      <c r="C100" s="79"/>
+      <c r="B100" s="62"/>
+      <c r="C100" s="65"/>
       <c r="D100" s="46" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="101" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B101" s="73">
+    <row r="101" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B101" s="82">
         <v>46076</v>
       </c>
-      <c r="C101" s="71">
+      <c r="C101" s="83">
         <v>4</v>
       </c>
-      <c r="D101" s="67" t="s">
+      <c r="D101" s="84" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="102" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B102" s="32"/>
-      <c r="C102" s="32"/>
-      <c r="D102" s="33"/>
+      <c r="B102" s="57">
+        <v>46077</v>
+      </c>
+      <c r="C102" s="56">
+        <v>2</v>
+      </c>
+      <c r="D102" s="54" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="103" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B103" s="71"/>
-      <c r="C103" s="71"/>
-      <c r="D103" s="51"/>
+      <c r="B103" s="56"/>
+      <c r="C103" s="56"/>
+      <c r="D103" s="55" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="104" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B104" s="32"/>
       <c r="C104" s="32"/>
-      <c r="D104" s="33"/>
-    </row>
-    <row r="105" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="D104" s="55" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="105" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B105" s="32"/>
       <c r="C105" s="32"/>
-      <c r="D105" s="33"/>
-    </row>
-    <row r="106" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B106" s="71"/>
-      <c r="C106" s="71"/>
-      <c r="D106" s="51"/>
+      <c r="D105" s="42" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="106" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B106" s="56"/>
+      <c r="C106" s="56"/>
+      <c r="D106" s="46" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="107" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B107" s="32"/>
@@ -3270,8 +3318,8 @@
       <c r="D108" s="33"/>
     </row>
     <row r="109" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B109" s="71"/>
-      <c r="C109" s="71"/>
+      <c r="B109" s="56"/>
+      <c r="C109" s="56"/>
       <c r="D109" s="51"/>
     </row>
     <row r="110" spans="2:4" x14ac:dyDescent="0.3">
@@ -3285,8 +3333,8 @@
       <c r="D111" s="33"/>
     </row>
     <row r="112" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B112" s="71"/>
-      <c r="C112" s="71"/>
+      <c r="B112" s="56"/>
+      <c r="C112" s="56"/>
       <c r="D112" s="51"/>
     </row>
     <row r="113" spans="2:4" x14ac:dyDescent="0.3">
@@ -3300,8 +3348,8 @@
       <c r="D114" s="33"/>
     </row>
     <row r="115" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B115" s="71"/>
-      <c r="C115" s="71"/>
+      <c r="B115" s="56"/>
+      <c r="C115" s="56"/>
       <c r="D115" s="51"/>
     </row>
     <row r="116" spans="2:4" x14ac:dyDescent="0.3">
@@ -3315,8 +3363,8 @@
       <c r="D117" s="33"/>
     </row>
     <row r="118" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B118" s="71"/>
-      <c r="C118" s="71"/>
+      <c r="B118" s="56"/>
+      <c r="C118" s="56"/>
       <c r="D118" s="51"/>
     </row>
     <row r="119" spans="2:4" x14ac:dyDescent="0.3">
@@ -3330,8 +3378,8 @@
       <c r="D120" s="33"/>
     </row>
     <row r="121" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B121" s="71"/>
-      <c r="C121" s="71"/>
+      <c r="B121" s="56"/>
+      <c r="C121" s="56"/>
       <c r="D121" s="51"/>
     </row>
     <row r="122" spans="2:4" x14ac:dyDescent="0.3">
@@ -3345,8 +3393,8 @@
       <c r="D123" s="33"/>
     </row>
     <row r="124" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B124" s="71"/>
-      <c r="C124" s="71"/>
+      <c r="B124" s="56"/>
+      <c r="C124" s="56"/>
       <c r="D124" s="51"/>
     </row>
     <row r="125" spans="2:4" x14ac:dyDescent="0.3">
@@ -3360,8 +3408,8 @@
       <c r="D126" s="33"/>
     </row>
     <row r="127" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B127" s="71"/>
-      <c r="C127" s="71"/>
+      <c r="B127" s="56"/>
+      <c r="C127" s="56"/>
       <c r="D127" s="51"/>
     </row>
     <row r="128" spans="2:4" x14ac:dyDescent="0.3">
@@ -3375,8 +3423,8 @@
       <c r="D129" s="33"/>
     </row>
     <row r="130" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B130" s="71"/>
-      <c r="C130" s="71"/>
+      <c r="B130" s="56"/>
+      <c r="C130" s="56"/>
       <c r="D130" s="51"/>
     </row>
     <row r="131" spans="2:4" x14ac:dyDescent="0.3">
@@ -3390,8 +3438,8 @@
       <c r="D132" s="33"/>
     </row>
     <row r="133" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B133" s="71"/>
-      <c r="C133" s="71"/>
+      <c r="B133" s="56"/>
+      <c r="C133" s="56"/>
       <c r="D133" s="51"/>
     </row>
     <row r="134" spans="2:4" x14ac:dyDescent="0.3">
@@ -3405,8 +3453,8 @@
       <c r="D135" s="33"/>
     </row>
     <row r="136" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B136" s="71"/>
-      <c r="C136" s="71"/>
+      <c r="B136" s="56"/>
+      <c r="C136" s="56"/>
       <c r="D136" s="51"/>
     </row>
     <row r="137" spans="2:4" x14ac:dyDescent="0.3">
@@ -3420,8 +3468,8 @@
       <c r="D138" s="33"/>
     </row>
     <row r="139" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B139" s="71"/>
-      <c r="C139" s="71"/>
+      <c r="B139" s="56"/>
+      <c r="C139" s="56"/>
       <c r="D139" s="51"/>
     </row>
     <row r="140" spans="2:4" x14ac:dyDescent="0.3">
@@ -3436,34 +3484,6 @@
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="B97:B100"/>
-    <mergeCell ref="C97:C100"/>
-    <mergeCell ref="B82:B88"/>
-    <mergeCell ref="C82:C88"/>
-    <mergeCell ref="B89:B93"/>
-    <mergeCell ref="C89:C93"/>
-    <mergeCell ref="B94:B96"/>
-    <mergeCell ref="C94:C96"/>
-    <mergeCell ref="B64:B68"/>
-    <mergeCell ref="C64:C68"/>
-    <mergeCell ref="B69:B74"/>
-    <mergeCell ref="C69:C74"/>
-    <mergeCell ref="B75:B81"/>
-    <mergeCell ref="C75:C81"/>
-    <mergeCell ref="B55:B58"/>
-    <mergeCell ref="C55:C58"/>
-    <mergeCell ref="B59:B63"/>
-    <mergeCell ref="C59:C63"/>
-    <mergeCell ref="B45:B49"/>
-    <mergeCell ref="C45:C49"/>
-    <mergeCell ref="B50:B54"/>
-    <mergeCell ref="C50:C54"/>
-    <mergeCell ref="C31:C36"/>
-    <mergeCell ref="B31:B36"/>
-    <mergeCell ref="C37:C41"/>
-    <mergeCell ref="B37:B41"/>
-    <mergeCell ref="B42:B44"/>
-    <mergeCell ref="C42:C44"/>
     <mergeCell ref="C16:C26"/>
     <mergeCell ref="B16:B26"/>
     <mergeCell ref="C27:C30"/>
@@ -3474,6 +3494,34 @@
     <mergeCell ref="C7:C10"/>
     <mergeCell ref="B11:B15"/>
     <mergeCell ref="C11:C15"/>
+    <mergeCell ref="C31:C36"/>
+    <mergeCell ref="B31:B36"/>
+    <mergeCell ref="C37:C41"/>
+    <mergeCell ref="B37:B41"/>
+    <mergeCell ref="B42:B44"/>
+    <mergeCell ref="C42:C44"/>
+    <mergeCell ref="B55:B58"/>
+    <mergeCell ref="C55:C58"/>
+    <mergeCell ref="B59:B63"/>
+    <mergeCell ref="C59:C63"/>
+    <mergeCell ref="B45:B49"/>
+    <mergeCell ref="C45:C49"/>
+    <mergeCell ref="B50:B54"/>
+    <mergeCell ref="C50:C54"/>
+    <mergeCell ref="B64:B68"/>
+    <mergeCell ref="C64:C68"/>
+    <mergeCell ref="B69:B74"/>
+    <mergeCell ref="C69:C74"/>
+    <mergeCell ref="B75:B81"/>
+    <mergeCell ref="C75:C81"/>
+    <mergeCell ref="B97:B100"/>
+    <mergeCell ref="C97:C100"/>
+    <mergeCell ref="B82:B88"/>
+    <mergeCell ref="C82:C88"/>
+    <mergeCell ref="B89:B93"/>
+    <mergeCell ref="C89:C93"/>
+    <mergeCell ref="B94:B96"/>
+    <mergeCell ref="C94:C96"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3502,36 +3550,36 @@
       </c>
     </row>
     <row r="3" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D3" s="57" t="s">
+      <c r="D3" s="80" t="s">
         <v>8</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F3" s="54" t="s">
+      <c r="F3" s="77" t="s">
         <v>1</v>
       </c>
-      <c r="G3" s="55"/>
-      <c r="H3" s="55"/>
-      <c r="I3" s="56"/>
-      <c r="J3" s="54" t="s">
+      <c r="G3" s="78"/>
+      <c r="H3" s="78"/>
+      <c r="I3" s="79"/>
+      <c r="J3" s="77" t="s">
         <v>2</v>
       </c>
-      <c r="K3" s="55"/>
-      <c r="L3" s="55"/>
-      <c r="M3" s="56"/>
-      <c r="N3" s="54" t="s">
+      <c r="K3" s="78"/>
+      <c r="L3" s="78"/>
+      <c r="M3" s="79"/>
+      <c r="N3" s="77" t="s">
         <v>3</v>
       </c>
-      <c r="O3" s="55"/>
-      <c r="P3" s="55"/>
-      <c r="Q3" s="56"/>
+      <c r="O3" s="78"/>
+      <c r="P3" s="78"/>
+      <c r="Q3" s="79"/>
       <c r="R3" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="4:18" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D4" s="58"/>
+      <c r="D4" s="81"/>
       <c r="E4" s="4" t="s">
         <v>4</v>
       </c>
@@ -3702,36 +3750,36 @@
       </c>
     </row>
     <row r="15" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D15" s="57" t="s">
+      <c r="D15" s="80" t="s">
         <v>8</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F15" s="54" t="s">
+      <c r="F15" s="77" t="s">
         <v>1</v>
       </c>
-      <c r="G15" s="55"/>
-      <c r="H15" s="55"/>
-      <c r="I15" s="56"/>
-      <c r="J15" s="54" t="s">
+      <c r="G15" s="78"/>
+      <c r="H15" s="78"/>
+      <c r="I15" s="79"/>
+      <c r="J15" s="77" t="s">
         <v>2</v>
       </c>
-      <c r="K15" s="55"/>
-      <c r="L15" s="55"/>
-      <c r="M15" s="56"/>
-      <c r="N15" s="54" t="s">
+      <c r="K15" s="78"/>
+      <c r="L15" s="78"/>
+      <c r="M15" s="79"/>
+      <c r="N15" s="77" t="s">
         <v>3</v>
       </c>
-      <c r="O15" s="55"/>
-      <c r="P15" s="55"/>
-      <c r="Q15" s="56"/>
+      <c r="O15" s="78"/>
+      <c r="P15" s="78"/>
+      <c r="Q15" s="79"/>
       <c r="R15" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="16" spans="4:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D16" s="58"/>
+      <c r="D16" s="81"/>
       <c r="E16" s="4" t="s">
         <v>4</v>
       </c>

</xml_diff>

<commit_message>
connected SQL Server and PowerBI
</commit_message>
<xml_diff>
--- a/DocumentsAndReports/0. WorkLog_Charts.xlsx
+++ b/DocumentsAndReports/0. WorkLog_Charts.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qhung\Videos\CSIS4495 - Applied Research  Project\W26_4495_S2_HughT\DocumentsAndReports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33A14A7E-A6E3-4AC9-B75D-E2E3ACE017F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D156DDB-5858-4BC3-9E30-C02E7A40839D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E067A1E6-0DC4-42DD-AAF8-D95EFF7A112F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E067A1E6-0DC4-42DD-AAF8-D95EFF7A112F}"/>
   </bookViews>
   <sheets>
     <sheet name="Work_Log" sheetId="2" r:id="rId1"/>
     <sheet name="Timeline" sheetId="1" r:id="rId2"/>
+    <sheet name="Reference" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="134">
   <si>
     <t>January</t>
   </si>
@@ -365,12 +366,515 @@
   <si>
     <t>“how to do html navigation in fastApi?”</t>
   </si>
+  <si>
+    <t>- Chat GPT's prompts:</t>
+  </si>
+  <si>
+    <t>“why the connection fail?”</t>
+  </si>
+  <si>
+    <t>“how to fix?”</t>
+  </si>
+  <si>
+    <t>- Connected SQL server and PowerBI</t>
+  </si>
+  <si>
+    <t>“provide step by step for each option”</t>
+  </si>
+  <si>
+    <r>
+      <t>1.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">      </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11.5"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>tutorialspoint, Business Intelligence – Architecture</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.tutorialspoint.com/business-intelligence/business-intelligence-architecture.htm</t>
+  </si>
+  <si>
+    <r>
+      <t>2.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">      </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11.5"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>IBIMA Publishing, A five layered business intelligence architecture (2011)</t>
+    </r>
+  </si>
+  <si>
+    <t>chromeextension://efaidnbmnnnibpcajpcglclefindmkaj/https://ibimapublishing.com/articles/CIBIMA/2011/695619/695619.pdf</t>
+  </si>
+  <si>
+    <r>
+      <t>3.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">      </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11.5"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Kanerika Inc, A complete guide to business intelligence architecture (Jan 29, 2025)</t>
+    </r>
+  </si>
+  <si>
+    <t>https://medium.com/@kanerika/a-complete-guide-to-business-intelligence-architecture-25ce2896a097</t>
+  </si>
+  <si>
+    <r>
+      <t>4.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">      </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11.5"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>GeeksforGeeks, FastAPI Introduction (Sept 23, 2025)</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/python/fastapi-introduction/</t>
+  </si>
+  <si>
+    <r>
+      <t>5.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">      </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11.5"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Astera Analytics Team, A guide for Python to SQL Server integration  (Feb 14, 2025)</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.astera.com/knowledge-center/python-to-sql-server-integration/</t>
+  </si>
+  <si>
+    <r>
+      <t>6.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">      </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11.5"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Dr. Fatih Hattatoglu, How to connect between Python and SQL? (Dec 22, 2024)</t>
+    </r>
+  </si>
+  <si>
+    <t>https://medium.com/academy-team/how-to-connect-between-python-and-sql-5f0639ccce73</t>
+  </si>
+  <si>
+    <r>
+      <t>7.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">      </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11.5"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>BI Tricks, How to connect SQL Server in Power BI (Sept 19, 2023)</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=DGYbWBRxGGQ</t>
+  </si>
+  <si>
+    <r>
+      <t>8.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">      </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11.5"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Nestor Adrianzen, How to connect SQL Server to Power BI [AdventureWorks2022 Sample Database] (Jun 7, 2025)</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=DAhFcLHY0LY</t>
+  </si>
+  <si>
+    <r>
+      <t>9.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">      </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11.5"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>MAXQDA, What is a sentiment analysis?</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.maxqda.com/research-guides/sentiment-analysis?gad_source=1&amp;gad_campaignid=868754387&amp;gbraid=0AAAAAD-6Ox0Q7SJSayyvDBmq8U9RNL2p2&amp;gclid=Cj0KCQiAm9fLBhCQARIsAJoNOctmGzW2DXZZKTy1e9Z4isnCXpp6OHrsJIvNr3hjJH7md6PTAn_bI6YaAoe6EALw_wcB</t>
+  </si>
+  <si>
+    <r>
+      <t>10.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11.5"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>GeeksforGeeks, What is text analytics? (Jul 23, 2025)</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/data-science/what-is-text-analytics/</t>
+  </si>
+  <si>
+    <r>
+      <t>11.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11.5"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Dataquest, Using machine learning and natural language processing tools for text analysis (Feb 28, 2022)</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.dataquest.io/blog/using-machine-learning-and-natural-language-processing-tools-for-text-analysis/</t>
+  </si>
+  <si>
+    <r>
+      <t>12.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11.5"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>PyData, Sean P.Rogers – Introduction to machine learning for text analysis and classification with Python (Sept 3, 2024)</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=_ps6XQXA1lY</t>
+  </si>
+  <si>
+    <r>
+      <t>13.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11.5"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Christian Ofori-Boateng, How to publish Power BI reports: a step-by-step process                             (Apr 3, 2024)</t>
+    </r>
+  </si>
+  <si>
+    <t>https://go.christiansteven.com/bi-blog/how-to-publish-power-bi-reports-a-step-by-step-process?utm_term=power%20bi%20integrate&amp;utm_medium=ppc&amp;utm_campaign=1.+PBRS-Search+(US+)&amp;utm_source=adwords&amp;hsa_cam=19872567087&amp;hsa_acc=6168560490&amp;hsa_src=g&amp;hsa_ad=652240527744&amp;hsa_tgt=aud-932430925173:kwd-2128074850707&amp;hsa_ver=3&amp;hsa_grp=147377883036&amp;hsa_mt=p&amp;hsa_net=adwords&amp;hsa_kw=power%20bi%20integrate&amp;gad_source=1&amp;gad_campaignid=19872567087&amp;gbraid=0AAAAAD4FRWSHUNPJUsSOmAPnnKKQvNzl3&amp;gclid=Cj0KCQiAm9fLBhCQARIsAJoNOcviWEg5dO-r5LG0NKtGGwiSHf-uHZczQ9qDVqck_sd4LHoGN_YEv1MaAqmFEALw_wcB</t>
+  </si>
+  <si>
+    <r>
+      <t>14.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11.5"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Microsoft Learn, Add a Power BI report or dashboard to a web page</t>
+    </r>
+  </si>
+  <si>
+    <t>https://learn.microsoft.com/en-us/power-pages/configure/add-powerbi-report</t>
+  </si>
+  <si>
+    <r>
+      <t>15.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11.5"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>GreeksForGreeks, How to add Bootstrap in a project? (July 23, 2025)</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/bootstrap/how-to-add-bootstrap-in-a-project/</t>
+  </si>
+  <si>
+    <r>
+      <t>16.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11.5"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>GreeksForGreeks, How to create a progress bar using HTML and CSS? (July 15, 2025)</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/web-templates/how-to-create-a-progress-bar-using-html-and-css/</t>
+  </si>
+  <si>
+    <r>
+      <t>17.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="7"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11.5"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Fast API, Custom response – HTML, Stream, File, others</t>
+    </r>
+  </si>
+  <si>
+    <t>https://fastapi.tiangolo.com/advanced/custom-response/</t>
+  </si>
+  <si>
+    <t>https://learn.microsoft.com/en-us/power-bi/connect-data/service-gateway-sql-tutorial</t>
+  </si>
+  <si>
+    <t>18. Microsoft, Refresh data from an on-premises SQL Server database</t>
+  </si>
+  <si>
+    <t>19. Andy McDonald, Connect PowerBI to SQL Server: step-by-step guide (Dec 2, 2024)</t>
+  </si>
+  <si>
+    <t>https://sqlspreads.com/blog/connect-power-bi-to-sql-server-step-by-step-guide/</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -454,6 +958,36 @@
       <name val="Aptos"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11.5"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="7"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <i/>
+      <u/>
+      <sz val="12"/>
+      <color rgb="FF467886"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -931,10 +1465,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1063,6 +1598,48 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="34" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="37" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -1081,39 +1658,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="15" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="15" fontId="7" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="15" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="15" fontId="7" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1129,17 +1673,22 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="37" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="28" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2496,10 +3045,10 @@
       </c>
     </row>
     <row r="3" spans="2:4" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="76">
+      <c r="B3" s="64">
         <v>45683</v>
       </c>
-      <c r="C3" s="75">
+      <c r="C3" s="63">
         <v>2</v>
       </c>
       <c r="D3" s="35" t="s">
@@ -2507,31 +3056,31 @@
       </c>
     </row>
     <row r="4" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="76"/>
-      <c r="C4" s="75"/>
+      <c r="B4" s="64"/>
+      <c r="C4" s="63"/>
       <c r="D4" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="76"/>
-      <c r="C5" s="75"/>
+      <c r="B5" s="64"/>
+      <c r="C5" s="63"/>
       <c r="D5" s="41" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="76"/>
-      <c r="C6" s="75"/>
+      <c r="B6" s="64"/>
+      <c r="C6" s="63"/>
       <c r="D6" s="42" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="7" spans="2:4" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="76">
+      <c r="B7" s="64">
         <v>45684</v>
       </c>
-      <c r="C7" s="75">
+      <c r="C7" s="63">
         <v>1.5</v>
       </c>
       <c r="D7" s="36" t="s">
@@ -2539,31 +3088,31 @@
       </c>
     </row>
     <row r="8" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="76"/>
-      <c r="C8" s="75"/>
+      <c r="B8" s="64"/>
+      <c r="C8" s="63"/>
       <c r="D8" s="37" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="9" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="76"/>
-      <c r="C9" s="75"/>
+      <c r="B9" s="64"/>
+      <c r="C9" s="63"/>
       <c r="D9" s="43" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="10" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="76"/>
-      <c r="C10" s="75"/>
+      <c r="B10" s="64"/>
+      <c r="C10" s="63"/>
       <c r="D10" s="44" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="76">
+      <c r="B11" s="64">
         <v>45686</v>
       </c>
-      <c r="C11" s="75">
+      <c r="C11" s="63">
         <v>3</v>
       </c>
       <c r="D11" s="35" t="s">
@@ -2571,38 +3120,38 @@
       </c>
     </row>
     <row r="12" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="76"/>
-      <c r="C12" s="75"/>
+      <c r="B12" s="64"/>
+      <c r="C12" s="63"/>
       <c r="D12" s="35" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="76"/>
-      <c r="C13" s="75"/>
+      <c r="B13" s="64"/>
+      <c r="C13" s="63"/>
       <c r="D13" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="76"/>
-      <c r="C14" s="75"/>
+      <c r="B14" s="64"/>
+      <c r="C14" s="63"/>
       <c r="D14" s="45" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="76"/>
-      <c r="C15" s="75"/>
+      <c r="B15" s="64"/>
+      <c r="C15" s="63"/>
       <c r="D15" s="42" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="76">
+      <c r="B16" s="64">
         <v>46053</v>
       </c>
-      <c r="C16" s="75">
+      <c r="C16" s="63">
         <v>4</v>
       </c>
       <c r="D16" s="38" t="s">
@@ -2610,80 +3159,80 @@
       </c>
     </row>
     <row r="17" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="76"/>
-      <c r="C17" s="75"/>
+      <c r="B17" s="64"/>
+      <c r="C17" s="63"/>
       <c r="D17" s="35" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="76"/>
-      <c r="C18" s="75"/>
+      <c r="B18" s="64"/>
+      <c r="C18" s="63"/>
       <c r="D18" s="35" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="19" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="76"/>
-      <c r="C19" s="75"/>
+      <c r="B19" s="64"/>
+      <c r="C19" s="63"/>
       <c r="D19" s="35" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="20" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="76"/>
-      <c r="C20" s="75"/>
+      <c r="B20" s="64"/>
+      <c r="C20" s="63"/>
       <c r="D20" s="35" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="21" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="76"/>
-      <c r="C21" s="75"/>
+      <c r="B21" s="64"/>
+      <c r="C21" s="63"/>
       <c r="D21" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="76"/>
-      <c r="C22" s="75"/>
+      <c r="B22" s="64"/>
+      <c r="C22" s="63"/>
       <c r="D22" s="45" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="23" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="76"/>
-      <c r="C23" s="75"/>
+      <c r="B23" s="64"/>
+      <c r="C23" s="63"/>
       <c r="D23" s="41" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="24" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="76"/>
-      <c r="C24" s="75"/>
+      <c r="B24" s="64"/>
+      <c r="C24" s="63"/>
       <c r="D24" s="41" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="25" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="76"/>
-      <c r="C25" s="75"/>
+      <c r="B25" s="64"/>
+      <c r="C25" s="63"/>
       <c r="D25" s="41" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="26" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="76"/>
-      <c r="C26" s="75"/>
+      <c r="B26" s="64"/>
+      <c r="C26" s="63"/>
       <c r="D26" s="46" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="27" spans="2:4" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="76">
+      <c r="B27" s="64">
         <v>46054</v>
       </c>
-      <c r="C27" s="75">
+      <c r="C27" s="63">
         <v>1</v>
       </c>
       <c r="D27" s="35" t="s">
@@ -2691,31 +3240,31 @@
       </c>
     </row>
     <row r="28" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="76"/>
-      <c r="C28" s="75"/>
+      <c r="B28" s="64"/>
+      <c r="C28" s="63"/>
       <c r="D28" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="29" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="76"/>
-      <c r="C29" s="75"/>
+      <c r="B29" s="64"/>
+      <c r="C29" s="63"/>
       <c r="D29" s="41" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="30" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="76"/>
-      <c r="C30" s="75"/>
+      <c r="B30" s="64"/>
+      <c r="C30" s="63"/>
       <c r="D30" s="42" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="31" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B31" s="76">
+      <c r="B31" s="64">
         <v>46055</v>
       </c>
-      <c r="C31" s="75">
+      <c r="C31" s="63">
         <v>4</v>
       </c>
       <c r="D31" s="39" t="s">
@@ -2723,45 +3272,45 @@
       </c>
     </row>
     <row r="32" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B32" s="76"/>
-      <c r="C32" s="75"/>
+      <c r="B32" s="64"/>
+      <c r="C32" s="63"/>
       <c r="D32" s="40" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="33" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="76"/>
-      <c r="C33" s="75"/>
+      <c r="B33" s="64"/>
+      <c r="C33" s="63"/>
       <c r="D33" s="40" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="34" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B34" s="76"/>
-      <c r="C34" s="75"/>
+      <c r="B34" s="64"/>
+      <c r="C34" s="63"/>
       <c r="D34" s="40" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="35" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B35" s="76"/>
-      <c r="C35" s="75"/>
+      <c r="B35" s="64"/>
+      <c r="C35" s="63"/>
       <c r="D35" s="47" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="36" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B36" s="76"/>
-      <c r="C36" s="75"/>
+      <c r="B36" s="64"/>
+      <c r="C36" s="63"/>
       <c r="D36" s="48" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="37" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="76">
+      <c r="B37" s="64">
         <v>46056</v>
       </c>
-      <c r="C37" s="75">
+      <c r="C37" s="63">
         <v>3</v>
       </c>
       <c r="D37" s="35" t="s">
@@ -2769,38 +3318,38 @@
       </c>
     </row>
     <row r="38" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B38" s="76"/>
-      <c r="C38" s="75"/>
+      <c r="B38" s="64"/>
+      <c r="C38" s="63"/>
       <c r="D38" s="35" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="39" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B39" s="76"/>
-      <c r="C39" s="75"/>
+      <c r="B39" s="64"/>
+      <c r="C39" s="63"/>
       <c r="D39" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="40" spans="2:4" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B40" s="76"/>
-      <c r="C40" s="75"/>
+      <c r="B40" s="64"/>
+      <c r="C40" s="63"/>
       <c r="D40" s="41" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="41" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B41" s="76"/>
-      <c r="C41" s="75"/>
+      <c r="B41" s="64"/>
+      <c r="C41" s="63"/>
       <c r="D41" s="42" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="42" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B42" s="76">
+      <c r="B42" s="64">
         <v>46057</v>
       </c>
-      <c r="C42" s="75">
+      <c r="C42" s="63">
         <v>4</v>
       </c>
       <c r="D42" s="38" t="s">
@@ -2808,24 +3357,24 @@
       </c>
     </row>
     <row r="43" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B43" s="76"/>
-      <c r="C43" s="75"/>
+      <c r="B43" s="64"/>
+      <c r="C43" s="63"/>
       <c r="D43" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="44" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B44" s="76"/>
-      <c r="C44" s="75"/>
+      <c r="B44" s="64"/>
+      <c r="C44" s="63"/>
       <c r="D44" s="42" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="45" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B45" s="66">
+      <c r="B45" s="65">
         <v>46059</v>
       </c>
-      <c r="C45" s="69">
+      <c r="C45" s="68">
         <v>2</v>
       </c>
       <c r="D45" s="50" t="s">
@@ -2833,38 +3382,38 @@
       </c>
     </row>
     <row r="46" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B46" s="67"/>
-      <c r="C46" s="70"/>
+      <c r="B46" s="66"/>
+      <c r="C46" s="69"/>
       <c r="D46" s="49" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="47" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B47" s="67"/>
-      <c r="C47" s="70"/>
+      <c r="B47" s="66"/>
+      <c r="C47" s="69"/>
       <c r="D47" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="48" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B48" s="67"/>
-      <c r="C48" s="70"/>
+      <c r="B48" s="66"/>
+      <c r="C48" s="69"/>
       <c r="D48" s="42" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="49" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B49" s="68"/>
-      <c r="C49" s="71"/>
+      <c r="B49" s="67"/>
+      <c r="C49" s="70"/>
       <c r="D49" s="46" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="50" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B50" s="66">
+      <c r="B50" s="65">
         <v>46061</v>
       </c>
-      <c r="C50" s="69">
+      <c r="C50" s="68">
         <v>1.5</v>
       </c>
       <c r="D50" s="50" t="s">
@@ -2872,38 +3421,38 @@
       </c>
     </row>
     <row r="51" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B51" s="67"/>
-      <c r="C51" s="70"/>
+      <c r="B51" s="66"/>
+      <c r="C51" s="69"/>
       <c r="D51" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="52" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B52" s="67"/>
-      <c r="C52" s="70"/>
+      <c r="B52" s="66"/>
+      <c r="C52" s="69"/>
       <c r="D52" s="42" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="53" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B53" s="67"/>
-      <c r="C53" s="70"/>
+      <c r="B53" s="66"/>
+      <c r="C53" s="69"/>
       <c r="D53" s="42" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="54" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B54" s="68"/>
-      <c r="C54" s="71"/>
+      <c r="B54" s="67"/>
+      <c r="C54" s="70"/>
       <c r="D54" s="46" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="55" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="66">
+      <c r="B55" s="65">
         <v>46062</v>
       </c>
-      <c r="C55" s="69">
+      <c r="C55" s="68">
         <v>2</v>
       </c>
       <c r="D55" s="54" t="s">
@@ -2911,31 +3460,31 @@
       </c>
     </row>
     <row r="56" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B56" s="67"/>
-      <c r="C56" s="70"/>
+      <c r="B56" s="66"/>
+      <c r="C56" s="69"/>
       <c r="D56" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="57" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B57" s="67"/>
-      <c r="C57" s="70"/>
+      <c r="B57" s="66"/>
+      <c r="C57" s="69"/>
       <c r="D57" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="58" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B58" s="68"/>
-      <c r="C58" s="71"/>
+      <c r="B58" s="67"/>
+      <c r="C58" s="70"/>
       <c r="D58" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="59" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="66">
+      <c r="B59" s="65">
         <v>46063</v>
       </c>
-      <c r="C59" s="69">
+      <c r="C59" s="68">
         <v>3</v>
       </c>
       <c r="D59" s="54" t="s">
@@ -2943,38 +3492,38 @@
       </c>
     </row>
     <row r="60" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B60" s="67"/>
-      <c r="C60" s="70"/>
+      <c r="B60" s="66"/>
+      <c r="C60" s="69"/>
       <c r="D60" s="55" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="61" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B61" s="67"/>
-      <c r="C61" s="70"/>
+      <c r="B61" s="66"/>
+      <c r="C61" s="69"/>
       <c r="D61" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="62" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B62" s="67"/>
-      <c r="C62" s="70"/>
+      <c r="B62" s="66"/>
+      <c r="C62" s="69"/>
       <c r="D62" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="63" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B63" s="68"/>
-      <c r="C63" s="71"/>
+      <c r="B63" s="67"/>
+      <c r="C63" s="70"/>
       <c r="D63" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="64" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B64" s="66">
+      <c r="B64" s="65">
         <v>46064</v>
       </c>
-      <c r="C64" s="69">
+      <c r="C64" s="68">
         <v>3</v>
       </c>
       <c r="D64" s="54" t="s">
@@ -2982,38 +3531,38 @@
       </c>
     </row>
     <row r="65" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B65" s="67"/>
-      <c r="C65" s="70"/>
+      <c r="B65" s="66"/>
+      <c r="C65" s="69"/>
       <c r="D65" s="55" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="66" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B66" s="67"/>
-      <c r="C66" s="70"/>
+      <c r="B66" s="66"/>
+      <c r="C66" s="69"/>
       <c r="D66" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="67" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B67" s="67"/>
-      <c r="C67" s="70"/>
+      <c r="B67" s="66"/>
+      <c r="C67" s="69"/>
       <c r="D67" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="68" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B68" s="68"/>
-      <c r="C68" s="71"/>
+      <c r="B68" s="67"/>
+      <c r="C68" s="70"/>
       <c r="D68" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="69" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B69" s="72">
+      <c r="B69" s="71">
         <v>46066</v>
       </c>
-      <c r="C69" s="69">
+      <c r="C69" s="68">
         <v>2</v>
       </c>
       <c r="D69" s="54" t="s">
@@ -3021,45 +3570,45 @@
       </c>
     </row>
     <row r="70" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B70" s="73"/>
-      <c r="C70" s="70"/>
+      <c r="B70" s="72"/>
+      <c r="C70" s="69"/>
       <c r="D70" s="55" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="71" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B71" s="73"/>
-      <c r="C71" s="70"/>
+      <c r="B71" s="72"/>
+      <c r="C71" s="69"/>
       <c r="D71" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="72" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B72" s="73"/>
-      <c r="C72" s="70"/>
+      <c r="B72" s="72"/>
+      <c r="C72" s="69"/>
       <c r="D72" s="42" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="73" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B73" s="73"/>
-      <c r="C73" s="70"/>
+      <c r="B73" s="72"/>
+      <c r="C73" s="69"/>
       <c r="D73" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="74" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B74" s="74"/>
-      <c r="C74" s="71"/>
+      <c r="B74" s="73"/>
+      <c r="C74" s="70"/>
       <c r="D74" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="75" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B75" s="60">
+      <c r="B75" s="74">
         <v>46068</v>
       </c>
-      <c r="C75" s="63">
+      <c r="C75" s="77">
         <v>2.5</v>
       </c>
       <c r="D75" s="54" t="s">
@@ -3067,52 +3616,52 @@
       </c>
     </row>
     <row r="76" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B76" s="61"/>
-      <c r="C76" s="64"/>
+      <c r="B76" s="75"/>
+      <c r="C76" s="78"/>
       <c r="D76" s="55" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="77" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B77" s="61"/>
-      <c r="C77" s="64"/>
+      <c r="B77" s="75"/>
+      <c r="C77" s="78"/>
       <c r="D77" s="55" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="78" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B78" s="61"/>
-      <c r="C78" s="64"/>
+      <c r="B78" s="75"/>
+      <c r="C78" s="78"/>
       <c r="D78" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="79" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B79" s="61"/>
-      <c r="C79" s="64"/>
+      <c r="B79" s="75"/>
+      <c r="C79" s="78"/>
       <c r="D79" s="42" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="80" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B80" s="61"/>
-      <c r="C80" s="64"/>
+      <c r="B80" s="75"/>
+      <c r="C80" s="78"/>
       <c r="D80" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="81" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B81" s="62"/>
-      <c r="C81" s="65"/>
+      <c r="B81" s="76"/>
+      <c r="C81" s="79"/>
       <c r="D81" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="82" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B82" s="60">
+      <c r="B82" s="74">
         <v>46070</v>
       </c>
-      <c r="C82" s="63">
+      <c r="C82" s="77">
         <v>3</v>
       </c>
       <c r="D82" s="54" t="s">
@@ -3120,52 +3669,52 @@
       </c>
     </row>
     <row r="83" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B83" s="61"/>
-      <c r="C83" s="64"/>
+      <c r="B83" s="75"/>
+      <c r="C83" s="78"/>
       <c r="D83" s="55" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="84" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B84" s="61"/>
-      <c r="C84" s="64"/>
+      <c r="B84" s="75"/>
+      <c r="C84" s="78"/>
       <c r="D84" s="55" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="85" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B85" s="61"/>
-      <c r="C85" s="64"/>
+      <c r="B85" s="75"/>
+      <c r="C85" s="78"/>
       <c r="D85" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="86" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B86" s="61"/>
-      <c r="C86" s="64"/>
+      <c r="B86" s="75"/>
+      <c r="C86" s="78"/>
       <c r="D86" s="42" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="87" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B87" s="61"/>
-      <c r="C87" s="64"/>
+      <c r="B87" s="75"/>
+      <c r="C87" s="78"/>
       <c r="D87" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="88" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B88" s="62"/>
-      <c r="C88" s="65"/>
+      <c r="B88" s="76"/>
+      <c r="C88" s="79"/>
       <c r="D88" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="89" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B89" s="60">
+      <c r="B89" s="74">
         <v>46071</v>
       </c>
-      <c r="C89" s="63">
+      <c r="C89" s="77">
         <v>2</v>
       </c>
       <c r="D89" s="54" t="s">
@@ -3173,38 +3722,38 @@
       </c>
     </row>
     <row r="90" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B90" s="61"/>
-      <c r="C90" s="64"/>
+      <c r="B90" s="75"/>
+      <c r="C90" s="78"/>
       <c r="D90" s="55" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="91" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B91" s="61"/>
-      <c r="C91" s="64"/>
+      <c r="B91" s="75"/>
+      <c r="C91" s="78"/>
       <c r="D91" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="92" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B92" s="61"/>
-      <c r="C92" s="64"/>
+      <c r="B92" s="75"/>
+      <c r="C92" s="78"/>
       <c r="D92" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="93" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B93" s="62"/>
-      <c r="C93" s="65"/>
+      <c r="B93" s="76"/>
+      <c r="C93" s="79"/>
       <c r="D93" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="94" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B94" s="60">
+      <c r="B94" s="74">
         <v>46074</v>
       </c>
-      <c r="C94" s="63">
+      <c r="C94" s="77">
         <v>3</v>
       </c>
       <c r="D94" s="58" t="s">
@@ -3212,24 +3761,24 @@
       </c>
     </row>
     <row r="95" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B95" s="61"/>
-      <c r="C95" s="64"/>
+      <c r="B95" s="75"/>
+      <c r="C95" s="78"/>
       <c r="D95" s="59" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="96" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B96" s="62"/>
-      <c r="C96" s="65"/>
+      <c r="B96" s="76"/>
+      <c r="C96" s="79"/>
       <c r="D96" s="46" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="97" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B97" s="60">
+      <c r="B97" s="74">
         <v>46075</v>
       </c>
-      <c r="C97" s="63">
+      <c r="C97" s="77">
         <v>3</v>
       </c>
       <c r="D97" s="54" t="s">
@@ -3237,42 +3786,42 @@
       </c>
     </row>
     <row r="98" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B98" s="61"/>
-      <c r="C98" s="64"/>
+      <c r="B98" s="75"/>
+      <c r="C98" s="78"/>
       <c r="D98" s="55" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="99" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B99" s="61"/>
-      <c r="C99" s="64"/>
+      <c r="B99" s="75"/>
+      <c r="C99" s="78"/>
       <c r="D99" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="100" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B100" s="62"/>
-      <c r="C100" s="65"/>
+      <c r="B100" s="76"/>
+      <c r="C100" s="79"/>
       <c r="D100" s="46" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="101" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B101" s="82">
+      <c r="B101" s="60">
         <v>46076</v>
       </c>
-      <c r="C101" s="83">
+      <c r="C101" s="61">
         <v>4</v>
       </c>
-      <c r="D101" s="84" t="s">
+      <c r="D101" s="62" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="102" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B102" s="57">
+      <c r="B102" s="74">
         <v>46077</v>
       </c>
-      <c r="C102" s="56">
+      <c r="C102" s="77">
         <v>2</v>
       </c>
       <c r="D102" s="54" t="s">
@@ -3280,57 +3829,71 @@
       </c>
     </row>
     <row r="103" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B103" s="56"/>
-      <c r="C103" s="56"/>
+      <c r="B103" s="75"/>
+      <c r="C103" s="78"/>
       <c r="D103" s="55" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="104" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B104" s="32"/>
-      <c r="C104" s="32"/>
+      <c r="B104" s="75"/>
+      <c r="C104" s="78"/>
       <c r="D104" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="105" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B105" s="32"/>
-      <c r="C105" s="32"/>
+      <c r="B105" s="75"/>
+      <c r="C105" s="78"/>
       <c r="D105" s="42" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="106" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B106" s="56"/>
-      <c r="C106" s="56"/>
+      <c r="B106" s="76"/>
+      <c r="C106" s="79"/>
       <c r="D106" s="46" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="107" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B107" s="32"/>
-      <c r="C107" s="32"/>
-      <c r="D107" s="33"/>
+      <c r="B107" s="57">
+        <v>46078</v>
+      </c>
+      <c r="C107" s="56">
+        <v>1</v>
+      </c>
+      <c r="D107" s="88" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="108" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B108" s="32"/>
       <c r="C108" s="32"/>
-      <c r="D108" s="33"/>
-    </row>
-    <row r="109" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="D108" s="55" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="109" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B109" s="56"/>
       <c r="C109" s="56"/>
-      <c r="D109" s="51"/>
-    </row>
-    <row r="110" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="D109" s="42" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="110" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B110" s="32"/>
       <c r="C110" s="32"/>
-      <c r="D110" s="33"/>
-    </row>
-    <row r="111" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="D110" s="42" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="111" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B111" s="32"/>
       <c r="C111" s="32"/>
-      <c r="D111" s="33"/>
+      <c r="D111" s="89" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="112" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B112" s="56"/>
@@ -3483,7 +4046,37 @@
       <c r="D141" s="33"/>
     </row>
   </sheetData>
-  <mergeCells count="38">
+  <mergeCells count="40">
+    <mergeCell ref="B102:B106"/>
+    <mergeCell ref="C102:C106"/>
+    <mergeCell ref="B97:B100"/>
+    <mergeCell ref="C97:C100"/>
+    <mergeCell ref="B82:B88"/>
+    <mergeCell ref="C82:C88"/>
+    <mergeCell ref="B89:B93"/>
+    <mergeCell ref="C89:C93"/>
+    <mergeCell ref="B94:B96"/>
+    <mergeCell ref="C94:C96"/>
+    <mergeCell ref="B64:B68"/>
+    <mergeCell ref="C64:C68"/>
+    <mergeCell ref="B69:B74"/>
+    <mergeCell ref="C69:C74"/>
+    <mergeCell ref="B75:B81"/>
+    <mergeCell ref="C75:C81"/>
+    <mergeCell ref="B55:B58"/>
+    <mergeCell ref="C55:C58"/>
+    <mergeCell ref="B59:B63"/>
+    <mergeCell ref="C59:C63"/>
+    <mergeCell ref="B45:B49"/>
+    <mergeCell ref="C45:C49"/>
+    <mergeCell ref="B50:B54"/>
+    <mergeCell ref="C50:C54"/>
+    <mergeCell ref="C31:C36"/>
+    <mergeCell ref="B31:B36"/>
+    <mergeCell ref="C37:C41"/>
+    <mergeCell ref="B37:B41"/>
+    <mergeCell ref="B42:B44"/>
+    <mergeCell ref="C42:C44"/>
     <mergeCell ref="C16:C26"/>
     <mergeCell ref="B16:B26"/>
     <mergeCell ref="C27:C30"/>
@@ -3494,34 +4087,6 @@
     <mergeCell ref="C7:C10"/>
     <mergeCell ref="B11:B15"/>
     <mergeCell ref="C11:C15"/>
-    <mergeCell ref="C31:C36"/>
-    <mergeCell ref="B31:B36"/>
-    <mergeCell ref="C37:C41"/>
-    <mergeCell ref="B37:B41"/>
-    <mergeCell ref="B42:B44"/>
-    <mergeCell ref="C42:C44"/>
-    <mergeCell ref="B55:B58"/>
-    <mergeCell ref="C55:C58"/>
-    <mergeCell ref="B59:B63"/>
-    <mergeCell ref="C59:C63"/>
-    <mergeCell ref="B45:B49"/>
-    <mergeCell ref="C45:C49"/>
-    <mergeCell ref="B50:B54"/>
-    <mergeCell ref="C50:C54"/>
-    <mergeCell ref="B64:B68"/>
-    <mergeCell ref="C64:C68"/>
-    <mergeCell ref="B69:B74"/>
-    <mergeCell ref="C69:C74"/>
-    <mergeCell ref="B75:B81"/>
-    <mergeCell ref="C75:C81"/>
-    <mergeCell ref="B97:B100"/>
-    <mergeCell ref="C97:C100"/>
-    <mergeCell ref="B82:B88"/>
-    <mergeCell ref="C82:C88"/>
-    <mergeCell ref="B89:B93"/>
-    <mergeCell ref="C89:C93"/>
-    <mergeCell ref="B94:B96"/>
-    <mergeCell ref="C94:C96"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3550,36 +4115,36 @@
       </c>
     </row>
     <row r="3" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D3" s="80" t="s">
+      <c r="D3" s="83" t="s">
         <v>8</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F3" s="77" t="s">
+      <c r="F3" s="80" t="s">
         <v>1</v>
       </c>
-      <c r="G3" s="78"/>
-      <c r="H3" s="78"/>
-      <c r="I3" s="79"/>
-      <c r="J3" s="77" t="s">
+      <c r="G3" s="81"/>
+      <c r="H3" s="81"/>
+      <c r="I3" s="82"/>
+      <c r="J3" s="80" t="s">
         <v>2</v>
       </c>
-      <c r="K3" s="78"/>
-      <c r="L3" s="78"/>
-      <c r="M3" s="79"/>
-      <c r="N3" s="77" t="s">
+      <c r="K3" s="81"/>
+      <c r="L3" s="81"/>
+      <c r="M3" s="82"/>
+      <c r="N3" s="80" t="s">
         <v>3</v>
       </c>
-      <c r="O3" s="78"/>
-      <c r="P3" s="78"/>
-      <c r="Q3" s="79"/>
+      <c r="O3" s="81"/>
+      <c r="P3" s="81"/>
+      <c r="Q3" s="82"/>
       <c r="R3" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="4:18" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D4" s="81"/>
+      <c r="D4" s="84"/>
       <c r="E4" s="4" t="s">
         <v>4</v>
       </c>
@@ -3750,36 +4315,36 @@
       </c>
     </row>
     <row r="15" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D15" s="80" t="s">
+      <c r="D15" s="83" t="s">
         <v>8</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F15" s="77" t="s">
+      <c r="F15" s="80" t="s">
         <v>1</v>
       </c>
-      <c r="G15" s="78"/>
-      <c r="H15" s="78"/>
-      <c r="I15" s="79"/>
-      <c r="J15" s="77" t="s">
+      <c r="G15" s="81"/>
+      <c r="H15" s="81"/>
+      <c r="I15" s="82"/>
+      <c r="J15" s="80" t="s">
         <v>2</v>
       </c>
-      <c r="K15" s="78"/>
-      <c r="L15" s="78"/>
-      <c r="M15" s="79"/>
-      <c r="N15" s="77" t="s">
+      <c r="K15" s="81"/>
+      <c r="L15" s="81"/>
+      <c r="M15" s="82"/>
+      <c r="N15" s="80" t="s">
         <v>3</v>
       </c>
-      <c r="O15" s="78"/>
-      <c r="P15" s="78"/>
-      <c r="Q15" s="79"/>
+      <c r="O15" s="81"/>
+      <c r="P15" s="81"/>
+      <c r="Q15" s="82"/>
       <c r="R15" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="16" spans="4:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D16" s="81"/>
+      <c r="D16" s="84"/>
       <c r="E16" s="4" t="s">
         <v>4</v>
       </c>
@@ -3960,4 +4525,217 @@
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45547B32-EEB0-499C-B4DF-D4679D899AC7}">
+  <sheetPr>
+    <tabColor rgb="FF92D050"/>
+  </sheetPr>
+  <dimension ref="B2:B39"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="245.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="85" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="3" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="86" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="4" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="85" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="5" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="87" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="85" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="87" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="8" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="85" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="9" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="87" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="10" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="85" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="11" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="87" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="12" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="85" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="13" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="87" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="14" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="85" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="15" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="87" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="16" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="85" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="87" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="85" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="86" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="85" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="87" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="22" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="85" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="23" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="87" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="24" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="85" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="25" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="86" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="26" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="85" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="27" spans="2:2" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="B27" s="87" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="28" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="85" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="29" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="87" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="30" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="85" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="31" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B31" s="87" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="32" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="85" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="87" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="85" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="87" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="36" spans="2:2" ht="15" x14ac:dyDescent="0.3">
+      <c r="B36" s="85" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="37" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B37" s="87" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="38" spans="2:2" ht="15" x14ac:dyDescent="0.3">
+      <c r="B38" s="85" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="39" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B39" s="87" t="s">
+        <v>133</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B3" r:id="rId1" xr:uid="{A35CD954-7AB9-4926-9E8C-4A89F880BC35}"/>
+    <hyperlink ref="B19" r:id="rId2" xr:uid="{C2449309-6DBA-4085-87DC-4AAD46A37213}"/>
+    <hyperlink ref="B25" r:id="rId3" xr:uid="{201ECACC-0140-4555-B2A5-3873862F9FE5}"/>
+    <hyperlink ref="B37" r:id="rId4" xr:uid="{F3266E3B-CA49-451D-9077-A713C3165DF0}"/>
+    <hyperlink ref="B39" r:id="rId5" xr:uid="{CBD12324-3408-4DAF-B1DD-D30DBDA42E22}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
embeded PowerBBI report to dashboard.html
</commit_message>
<xml_diff>
--- a/DocumentsAndReports/0. WorkLog_Charts.xlsx
+++ b/DocumentsAndReports/0. WorkLog_Charts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qhung\Videos\CSIS4495 - Applied Research  Project\W26_4495_S2_HughT\DocumentsAndReports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D156DDB-5858-4BC3-9E30-C02E7A40839D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{085CCC51-433A-4200-8045-8D444ACF3AD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E067A1E6-0DC4-42DD-AAF8-D95EFF7A112F}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="139">
   <si>
     <t>January</t>
   </si>
@@ -868,6 +868,21 @@
   </si>
   <si>
     <t>https://sqlspreads.com/blog/connect-power-bi-to-sql-server-step-by-step-guide/</t>
+  </si>
+  <si>
+    <t>- Embeded PowerBI report to front-end</t>
+  </si>
+  <si>
+    <t>“i'm using school account, how can i switch to personal account then their is no need to ask admin permission?”</t>
+  </si>
+  <si>
+    <t>“not work with "Public to web(public)", can i use "website or portal" instead?”</t>
+  </si>
+  <si>
+    <t>20. Microsoft Learn, Publish to web from PowerBI</t>
+  </si>
+  <si>
+    <t>https://learn.microsoft.com/en-us/power-bi/collaborate-share/service-publish-to-web#enable-publish-to-web-as-an-administrator</t>
   </si>
 </sst>
 </file>
@@ -1607,57 +1622,69 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="37" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="28" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="15" fontId="7" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="15" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="15" fontId="7" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="15" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1673,19 +1700,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="28" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3028,7 +3043,7 @@
     <col min="1" max="1" width="8.88671875" style="2"/>
     <col min="2" max="2" width="18.21875" style="30" customWidth="1"/>
     <col min="3" max="3" width="17.33203125" style="30" customWidth="1"/>
-    <col min="4" max="4" width="94" style="2" customWidth="1"/>
+    <col min="4" max="4" width="112.109375" style="2" customWidth="1"/>
     <col min="5" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
@@ -3045,10 +3060,10 @@
       </c>
     </row>
     <row r="3" spans="2:4" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="64">
+      <c r="B3" s="83">
         <v>45683</v>
       </c>
-      <c r="C3" s="63">
+      <c r="C3" s="82">
         <v>2</v>
       </c>
       <c r="D3" s="35" t="s">
@@ -3056,31 +3071,31 @@
       </c>
     </row>
     <row r="4" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="64"/>
-      <c r="C4" s="63"/>
+      <c r="B4" s="83"/>
+      <c r="C4" s="82"/>
       <c r="D4" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="64"/>
-      <c r="C5" s="63"/>
+      <c r="B5" s="83"/>
+      <c r="C5" s="82"/>
       <c r="D5" s="41" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="64"/>
-      <c r="C6" s="63"/>
+      <c r="B6" s="83"/>
+      <c r="C6" s="82"/>
       <c r="D6" s="42" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="7" spans="2:4" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="64">
+      <c r="B7" s="83">
         <v>45684</v>
       </c>
-      <c r="C7" s="63">
+      <c r="C7" s="82">
         <v>1.5</v>
       </c>
       <c r="D7" s="36" t="s">
@@ -3088,31 +3103,31 @@
       </c>
     </row>
     <row r="8" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="64"/>
-      <c r="C8" s="63"/>
+      <c r="B8" s="83"/>
+      <c r="C8" s="82"/>
       <c r="D8" s="37" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="9" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="64"/>
-      <c r="C9" s="63"/>
+      <c r="B9" s="83"/>
+      <c r="C9" s="82"/>
       <c r="D9" s="43" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="10" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="64"/>
-      <c r="C10" s="63"/>
+      <c r="B10" s="83"/>
+      <c r="C10" s="82"/>
       <c r="D10" s="44" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="64">
+      <c r="B11" s="83">
         <v>45686</v>
       </c>
-      <c r="C11" s="63">
+      <c r="C11" s="82">
         <v>3</v>
       </c>
       <c r="D11" s="35" t="s">
@@ -3120,38 +3135,38 @@
       </c>
     </row>
     <row r="12" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="64"/>
-      <c r="C12" s="63"/>
+      <c r="B12" s="83"/>
+      <c r="C12" s="82"/>
       <c r="D12" s="35" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="64"/>
-      <c r="C13" s="63"/>
+      <c r="B13" s="83"/>
+      <c r="C13" s="82"/>
       <c r="D13" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="64"/>
-      <c r="C14" s="63"/>
+      <c r="B14" s="83"/>
+      <c r="C14" s="82"/>
       <c r="D14" s="45" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="64"/>
-      <c r="C15" s="63"/>
+      <c r="B15" s="83"/>
+      <c r="C15" s="82"/>
       <c r="D15" s="42" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="64">
+      <c r="B16" s="83">
         <v>46053</v>
       </c>
-      <c r="C16" s="63">
+      <c r="C16" s="82">
         <v>4</v>
       </c>
       <c r="D16" s="38" t="s">
@@ -3159,80 +3174,80 @@
       </c>
     </row>
     <row r="17" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="64"/>
-      <c r="C17" s="63"/>
+      <c r="B17" s="83"/>
+      <c r="C17" s="82"/>
       <c r="D17" s="35" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="64"/>
-      <c r="C18" s="63"/>
+      <c r="B18" s="83"/>
+      <c r="C18" s="82"/>
       <c r="D18" s="35" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="19" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="64"/>
-      <c r="C19" s="63"/>
+      <c r="B19" s="83"/>
+      <c r="C19" s="82"/>
       <c r="D19" s="35" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="20" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="64"/>
-      <c r="C20" s="63"/>
+      <c r="B20" s="83"/>
+      <c r="C20" s="82"/>
       <c r="D20" s="35" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="21" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="64"/>
-      <c r="C21" s="63"/>
+      <c r="B21" s="83"/>
+      <c r="C21" s="82"/>
       <c r="D21" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="64"/>
-      <c r="C22" s="63"/>
+      <c r="B22" s="83"/>
+      <c r="C22" s="82"/>
       <c r="D22" s="45" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="23" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="64"/>
-      <c r="C23" s="63"/>
+      <c r="B23" s="83"/>
+      <c r="C23" s="82"/>
       <c r="D23" s="41" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="24" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="64"/>
-      <c r="C24" s="63"/>
+      <c r="B24" s="83"/>
+      <c r="C24" s="82"/>
       <c r="D24" s="41" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="25" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="64"/>
-      <c r="C25" s="63"/>
+      <c r="B25" s="83"/>
+      <c r="C25" s="82"/>
       <c r="D25" s="41" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="26" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="64"/>
-      <c r="C26" s="63"/>
+      <c r="B26" s="83"/>
+      <c r="C26" s="82"/>
       <c r="D26" s="46" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="27" spans="2:4" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="64">
+      <c r="B27" s="83">
         <v>46054</v>
       </c>
-      <c r="C27" s="63">
+      <c r="C27" s="82">
         <v>1</v>
       </c>
       <c r="D27" s="35" t="s">
@@ -3240,31 +3255,31 @@
       </c>
     </row>
     <row r="28" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="64"/>
-      <c r="C28" s="63"/>
+      <c r="B28" s="83"/>
+      <c r="C28" s="82"/>
       <c r="D28" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="29" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="64"/>
-      <c r="C29" s="63"/>
+      <c r="B29" s="83"/>
+      <c r="C29" s="82"/>
       <c r="D29" s="41" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="30" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="64"/>
-      <c r="C30" s="63"/>
+      <c r="B30" s="83"/>
+      <c r="C30" s="82"/>
       <c r="D30" s="42" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="31" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B31" s="64">
+      <c r="B31" s="83">
         <v>46055</v>
       </c>
-      <c r="C31" s="63">
+      <c r="C31" s="82">
         <v>4</v>
       </c>
       <c r="D31" s="39" t="s">
@@ -3272,45 +3287,45 @@
       </c>
     </row>
     <row r="32" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B32" s="64"/>
-      <c r="C32" s="63"/>
+      <c r="B32" s="83"/>
+      <c r="C32" s="82"/>
       <c r="D32" s="40" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="33" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="64"/>
-      <c r="C33" s="63"/>
+      <c r="B33" s="83"/>
+      <c r="C33" s="82"/>
       <c r="D33" s="40" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="34" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B34" s="64"/>
-      <c r="C34" s="63"/>
+      <c r="B34" s="83"/>
+      <c r="C34" s="82"/>
       <c r="D34" s="40" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="35" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B35" s="64"/>
-      <c r="C35" s="63"/>
+      <c r="B35" s="83"/>
+      <c r="C35" s="82"/>
       <c r="D35" s="47" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="36" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B36" s="64"/>
-      <c r="C36" s="63"/>
+      <c r="B36" s="83"/>
+      <c r="C36" s="82"/>
       <c r="D36" s="48" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="37" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="64">
+      <c r="B37" s="83">
         <v>46056</v>
       </c>
-      <c r="C37" s="63">
+      <c r="C37" s="82">
         <v>3</v>
       </c>
       <c r="D37" s="35" t="s">
@@ -3318,38 +3333,38 @@
       </c>
     </row>
     <row r="38" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B38" s="64"/>
-      <c r="C38" s="63"/>
+      <c r="B38" s="83"/>
+      <c r="C38" s="82"/>
       <c r="D38" s="35" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="39" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B39" s="64"/>
-      <c r="C39" s="63"/>
+      <c r="B39" s="83"/>
+      <c r="C39" s="82"/>
       <c r="D39" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="40" spans="2:4" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B40" s="64"/>
-      <c r="C40" s="63"/>
+      <c r="B40" s="83"/>
+      <c r="C40" s="82"/>
       <c r="D40" s="41" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="41" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B41" s="64"/>
-      <c r="C41" s="63"/>
+      <c r="B41" s="83"/>
+      <c r="C41" s="82"/>
       <c r="D41" s="42" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="42" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B42" s="64">
+      <c r="B42" s="83">
         <v>46057</v>
       </c>
-      <c r="C42" s="63">
+      <c r="C42" s="82">
         <v>4</v>
       </c>
       <c r="D42" s="38" t="s">
@@ -3357,24 +3372,24 @@
       </c>
     </row>
     <row r="43" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B43" s="64"/>
-      <c r="C43" s="63"/>
+      <c r="B43" s="83"/>
+      <c r="C43" s="82"/>
       <c r="D43" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="44" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B44" s="64"/>
-      <c r="C44" s="63"/>
+      <c r="B44" s="83"/>
+      <c r="C44" s="82"/>
       <c r="D44" s="42" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="45" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B45" s="65">
+      <c r="B45" s="73">
         <v>46059</v>
       </c>
-      <c r="C45" s="68">
+      <c r="C45" s="76">
         <v>2</v>
       </c>
       <c r="D45" s="50" t="s">
@@ -3382,38 +3397,38 @@
       </c>
     </row>
     <row r="46" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B46" s="66"/>
-      <c r="C46" s="69"/>
+      <c r="B46" s="74"/>
+      <c r="C46" s="77"/>
       <c r="D46" s="49" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="47" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B47" s="66"/>
-      <c r="C47" s="69"/>
+      <c r="B47" s="74"/>
+      <c r="C47" s="77"/>
       <c r="D47" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="48" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B48" s="66"/>
-      <c r="C48" s="69"/>
+      <c r="B48" s="74"/>
+      <c r="C48" s="77"/>
       <c r="D48" s="42" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="49" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B49" s="67"/>
-      <c r="C49" s="70"/>
+      <c r="B49" s="75"/>
+      <c r="C49" s="78"/>
       <c r="D49" s="46" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="50" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B50" s="65">
+      <c r="B50" s="73">
         <v>46061</v>
       </c>
-      <c r="C50" s="68">
+      <c r="C50" s="76">
         <v>1.5</v>
       </c>
       <c r="D50" s="50" t="s">
@@ -3421,38 +3436,38 @@
       </c>
     </row>
     <row r="51" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B51" s="66"/>
-      <c r="C51" s="69"/>
+      <c r="B51" s="74"/>
+      <c r="C51" s="77"/>
       <c r="D51" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="52" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B52" s="66"/>
-      <c r="C52" s="69"/>
+      <c r="B52" s="74"/>
+      <c r="C52" s="77"/>
       <c r="D52" s="42" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="53" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B53" s="66"/>
-      <c r="C53" s="69"/>
+      <c r="B53" s="74"/>
+      <c r="C53" s="77"/>
       <c r="D53" s="42" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="54" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B54" s="67"/>
-      <c r="C54" s="70"/>
+      <c r="B54" s="75"/>
+      <c r="C54" s="78"/>
       <c r="D54" s="46" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="55" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="65">
+      <c r="B55" s="73">
         <v>46062</v>
       </c>
-      <c r="C55" s="68">
+      <c r="C55" s="76">
         <v>2</v>
       </c>
       <c r="D55" s="54" t="s">
@@ -3460,31 +3475,31 @@
       </c>
     </row>
     <row r="56" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B56" s="66"/>
-      <c r="C56" s="69"/>
+      <c r="B56" s="74"/>
+      <c r="C56" s="77"/>
       <c r="D56" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="57" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B57" s="66"/>
-      <c r="C57" s="69"/>
+      <c r="B57" s="74"/>
+      <c r="C57" s="77"/>
       <c r="D57" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="58" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B58" s="67"/>
-      <c r="C58" s="70"/>
+      <c r="B58" s="75"/>
+      <c r="C58" s="78"/>
       <c r="D58" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="59" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="65">
+      <c r="B59" s="73">
         <v>46063</v>
       </c>
-      <c r="C59" s="68">
+      <c r="C59" s="76">
         <v>3</v>
       </c>
       <c r="D59" s="54" t="s">
@@ -3492,38 +3507,38 @@
       </c>
     </row>
     <row r="60" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B60" s="66"/>
-      <c r="C60" s="69"/>
+      <c r="B60" s="74"/>
+      <c r="C60" s="77"/>
       <c r="D60" s="55" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="61" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B61" s="66"/>
-      <c r="C61" s="69"/>
+      <c r="B61" s="74"/>
+      <c r="C61" s="77"/>
       <c r="D61" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="62" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B62" s="66"/>
-      <c r="C62" s="69"/>
+      <c r="B62" s="74"/>
+      <c r="C62" s="77"/>
       <c r="D62" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="63" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B63" s="67"/>
-      <c r="C63" s="70"/>
+      <c r="B63" s="75"/>
+      <c r="C63" s="78"/>
       <c r="D63" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="64" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B64" s="65">
+      <c r="B64" s="73">
         <v>46064</v>
       </c>
-      <c r="C64" s="68">
+      <c r="C64" s="76">
         <v>3</v>
       </c>
       <c r="D64" s="54" t="s">
@@ -3531,38 +3546,38 @@
       </c>
     </row>
     <row r="65" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B65" s="66"/>
-      <c r="C65" s="69"/>
+      <c r="B65" s="74"/>
+      <c r="C65" s="77"/>
       <c r="D65" s="55" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="66" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B66" s="66"/>
-      <c r="C66" s="69"/>
+      <c r="B66" s="74"/>
+      <c r="C66" s="77"/>
       <c r="D66" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="67" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B67" s="66"/>
-      <c r="C67" s="69"/>
+      <c r="B67" s="74"/>
+      <c r="C67" s="77"/>
       <c r="D67" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="68" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B68" s="67"/>
-      <c r="C68" s="70"/>
+      <c r="B68" s="75"/>
+      <c r="C68" s="78"/>
       <c r="D68" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="69" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B69" s="71">
+      <c r="B69" s="79">
         <v>46066</v>
       </c>
-      <c r="C69" s="68">
+      <c r="C69" s="76">
         <v>2</v>
       </c>
       <c r="D69" s="54" t="s">
@@ -3570,45 +3585,45 @@
       </c>
     </row>
     <row r="70" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B70" s="72"/>
-      <c r="C70" s="69"/>
+      <c r="B70" s="80"/>
+      <c r="C70" s="77"/>
       <c r="D70" s="55" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="71" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B71" s="72"/>
-      <c r="C71" s="69"/>
+      <c r="B71" s="80"/>
+      <c r="C71" s="77"/>
       <c r="D71" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="72" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B72" s="72"/>
-      <c r="C72" s="69"/>
+      <c r="B72" s="80"/>
+      <c r="C72" s="77"/>
       <c r="D72" s="42" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="73" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B73" s="72"/>
-      <c r="C73" s="69"/>
+      <c r="B73" s="80"/>
+      <c r="C73" s="77"/>
       <c r="D73" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="74" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B74" s="73"/>
-      <c r="C74" s="70"/>
+      <c r="B74" s="81"/>
+      <c r="C74" s="78"/>
       <c r="D74" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="75" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B75" s="74">
+      <c r="B75" s="67">
         <v>46068</v>
       </c>
-      <c r="C75" s="77">
+      <c r="C75" s="70">
         <v>2.5</v>
       </c>
       <c r="D75" s="54" t="s">
@@ -3616,52 +3631,52 @@
       </c>
     </row>
     <row r="76" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B76" s="75"/>
-      <c r="C76" s="78"/>
+      <c r="B76" s="68"/>
+      <c r="C76" s="71"/>
       <c r="D76" s="55" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="77" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B77" s="75"/>
-      <c r="C77" s="78"/>
+      <c r="B77" s="68"/>
+      <c r="C77" s="71"/>
       <c r="D77" s="55" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="78" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B78" s="75"/>
-      <c r="C78" s="78"/>
+      <c r="B78" s="68"/>
+      <c r="C78" s="71"/>
       <c r="D78" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="79" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B79" s="75"/>
-      <c r="C79" s="78"/>
+      <c r="B79" s="68"/>
+      <c r="C79" s="71"/>
       <c r="D79" s="42" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="80" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B80" s="75"/>
-      <c r="C80" s="78"/>
+      <c r="B80" s="68"/>
+      <c r="C80" s="71"/>
       <c r="D80" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="81" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B81" s="76"/>
-      <c r="C81" s="79"/>
+      <c r="B81" s="69"/>
+      <c r="C81" s="72"/>
       <c r="D81" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="82" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B82" s="74">
+      <c r="B82" s="67">
         <v>46070</v>
       </c>
-      <c r="C82" s="77">
+      <c r="C82" s="70">
         <v>3</v>
       </c>
       <c r="D82" s="54" t="s">
@@ -3669,52 +3684,52 @@
       </c>
     </row>
     <row r="83" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B83" s="75"/>
-      <c r="C83" s="78"/>
+      <c r="B83" s="68"/>
+      <c r="C83" s="71"/>
       <c r="D83" s="55" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="84" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B84" s="75"/>
-      <c r="C84" s="78"/>
+      <c r="B84" s="68"/>
+      <c r="C84" s="71"/>
       <c r="D84" s="55" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="85" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B85" s="75"/>
-      <c r="C85" s="78"/>
+      <c r="B85" s="68"/>
+      <c r="C85" s="71"/>
       <c r="D85" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="86" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B86" s="75"/>
-      <c r="C86" s="78"/>
+      <c r="B86" s="68"/>
+      <c r="C86" s="71"/>
       <c r="D86" s="42" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="87" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B87" s="75"/>
-      <c r="C87" s="78"/>
+      <c r="B87" s="68"/>
+      <c r="C87" s="71"/>
       <c r="D87" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="88" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B88" s="76"/>
-      <c r="C88" s="79"/>
+      <c r="B88" s="69"/>
+      <c r="C88" s="72"/>
       <c r="D88" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="89" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B89" s="74">
+      <c r="B89" s="67">
         <v>46071</v>
       </c>
-      <c r="C89" s="77">
+      <c r="C89" s="70">
         <v>2</v>
       </c>
       <c r="D89" s="54" t="s">
@@ -3722,38 +3737,38 @@
       </c>
     </row>
     <row r="90" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B90" s="75"/>
-      <c r="C90" s="78"/>
+      <c r="B90" s="68"/>
+      <c r="C90" s="71"/>
       <c r="D90" s="55" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="91" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B91" s="75"/>
-      <c r="C91" s="78"/>
+      <c r="B91" s="68"/>
+      <c r="C91" s="71"/>
       <c r="D91" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="92" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B92" s="75"/>
-      <c r="C92" s="78"/>
+      <c r="B92" s="68"/>
+      <c r="C92" s="71"/>
       <c r="D92" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="93" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B93" s="76"/>
-      <c r="C93" s="79"/>
+      <c r="B93" s="69"/>
+      <c r="C93" s="72"/>
       <c r="D93" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="94" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B94" s="74">
+      <c r="B94" s="67">
         <v>46074</v>
       </c>
-      <c r="C94" s="77">
+      <c r="C94" s="70">
         <v>3</v>
       </c>
       <c r="D94" s="58" t="s">
@@ -3761,24 +3776,24 @@
       </c>
     </row>
     <row r="95" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B95" s="75"/>
-      <c r="C95" s="78"/>
+      <c r="B95" s="68"/>
+      <c r="C95" s="71"/>
       <c r="D95" s="59" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="96" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B96" s="76"/>
-      <c r="C96" s="79"/>
+      <c r="B96" s="69"/>
+      <c r="C96" s="72"/>
       <c r="D96" s="46" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="97" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B97" s="74">
+      <c r="B97" s="67">
         <v>46075</v>
       </c>
-      <c r="C97" s="77">
+      <c r="C97" s="70">
         <v>3</v>
       </c>
       <c r="D97" s="54" t="s">
@@ -3786,22 +3801,22 @@
       </c>
     </row>
     <row r="98" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B98" s="75"/>
-      <c r="C98" s="78"/>
+      <c r="B98" s="68"/>
+      <c r="C98" s="71"/>
       <c r="D98" s="55" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="99" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B99" s="75"/>
-      <c r="C99" s="78"/>
+      <c r="B99" s="68"/>
+      <c r="C99" s="71"/>
       <c r="D99" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="100" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B100" s="76"/>
-      <c r="C100" s="79"/>
+      <c r="B100" s="69"/>
+      <c r="C100" s="72"/>
       <c r="D100" s="46" t="s">
         <v>23</v>
       </c>
@@ -3818,10 +3833,10 @@
       </c>
     </row>
     <row r="102" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B102" s="74">
+      <c r="B102" s="67">
         <v>46077</v>
       </c>
-      <c r="C102" s="77">
+      <c r="C102" s="70">
         <v>2</v>
       </c>
       <c r="D102" s="54" t="s">
@@ -3829,91 +3844,103 @@
       </c>
     </row>
     <row r="103" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B103" s="75"/>
-      <c r="C103" s="78"/>
+      <c r="B103" s="68"/>
+      <c r="C103" s="71"/>
       <c r="D103" s="55" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="104" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B104" s="75"/>
-      <c r="C104" s="78"/>
+      <c r="B104" s="68"/>
+      <c r="C104" s="71"/>
       <c r="D104" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="105" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B105" s="75"/>
-      <c r="C105" s="78"/>
+      <c r="B105" s="68"/>
+      <c r="C105" s="71"/>
       <c r="D105" s="42" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="106" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B106" s="76"/>
-      <c r="C106" s="79"/>
+      <c r="B106" s="69"/>
+      <c r="C106" s="72"/>
       <c r="D106" s="46" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="107" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B107" s="57">
+      <c r="B107" s="67">
         <v>46078</v>
       </c>
-      <c r="C107" s="56">
+      <c r="C107" s="70">
         <v>1</v>
       </c>
-      <c r="D107" s="88" t="s">
+      <c r="D107" s="66" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="108" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B108" s="32"/>
-      <c r="C108" s="32"/>
+      <c r="B108" s="68"/>
+      <c r="C108" s="71"/>
       <c r="D108" s="55" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="109" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B109" s="56"/>
-      <c r="C109" s="56"/>
+      <c r="B109" s="68"/>
+      <c r="C109" s="71"/>
       <c r="D109" s="42" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="110" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B110" s="32"/>
-      <c r="C110" s="32"/>
+      <c r="B110" s="68"/>
+      <c r="C110" s="71"/>
       <c r="D110" s="42" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="111" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B111" s="32"/>
-      <c r="C111" s="32"/>
+    <row r="111" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B111" s="69"/>
+      <c r="C111" s="72"/>
       <c r="D111" s="89" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="112" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B112" s="56"/>
-      <c r="C112" s="56"/>
-      <c r="D112" s="51"/>
+      <c r="B112" s="57">
+        <v>46079</v>
+      </c>
+      <c r="C112" s="56">
+        <v>2</v>
+      </c>
+      <c r="D112" s="66" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="113" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B113" s="32"/>
       <c r="C113" s="32"/>
-      <c r="D113" s="33"/>
-    </row>
-    <row r="114" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="D113" s="55" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="114" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B114" s="32"/>
       <c r="C114" s="32"/>
-      <c r="D114" s="33"/>
-    </row>
-    <row r="115" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="D114" s="42" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="115" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B115" s="56"/>
       <c r="C115" s="56"/>
-      <c r="D115" s="51"/>
+      <c r="D115" s="42" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="116" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B116" s="32"/>
@@ -4046,7 +4073,39 @@
       <c r="D141" s="33"/>
     </row>
   </sheetData>
-  <mergeCells count="40">
+  <mergeCells count="42">
+    <mergeCell ref="B107:B111"/>
+    <mergeCell ref="C107:C111"/>
+    <mergeCell ref="C16:C26"/>
+    <mergeCell ref="B16:B26"/>
+    <mergeCell ref="C27:C30"/>
+    <mergeCell ref="B27:B30"/>
+    <mergeCell ref="B3:B6"/>
+    <mergeCell ref="C3:C6"/>
+    <mergeCell ref="B7:B10"/>
+    <mergeCell ref="C7:C10"/>
+    <mergeCell ref="B11:B15"/>
+    <mergeCell ref="C11:C15"/>
+    <mergeCell ref="C31:C36"/>
+    <mergeCell ref="B31:B36"/>
+    <mergeCell ref="C37:C41"/>
+    <mergeCell ref="B37:B41"/>
+    <mergeCell ref="B42:B44"/>
+    <mergeCell ref="C42:C44"/>
+    <mergeCell ref="B55:B58"/>
+    <mergeCell ref="C55:C58"/>
+    <mergeCell ref="B59:B63"/>
+    <mergeCell ref="C59:C63"/>
+    <mergeCell ref="B45:B49"/>
+    <mergeCell ref="C45:C49"/>
+    <mergeCell ref="B50:B54"/>
+    <mergeCell ref="C50:C54"/>
+    <mergeCell ref="B64:B68"/>
+    <mergeCell ref="C64:C68"/>
+    <mergeCell ref="B69:B74"/>
+    <mergeCell ref="C69:C74"/>
+    <mergeCell ref="B75:B81"/>
+    <mergeCell ref="C75:C81"/>
     <mergeCell ref="B102:B106"/>
     <mergeCell ref="C102:C106"/>
     <mergeCell ref="B97:B100"/>
@@ -4057,36 +4116,6 @@
     <mergeCell ref="C89:C93"/>
     <mergeCell ref="B94:B96"/>
     <mergeCell ref="C94:C96"/>
-    <mergeCell ref="B64:B68"/>
-    <mergeCell ref="C64:C68"/>
-    <mergeCell ref="B69:B74"/>
-    <mergeCell ref="C69:C74"/>
-    <mergeCell ref="B75:B81"/>
-    <mergeCell ref="C75:C81"/>
-    <mergeCell ref="B55:B58"/>
-    <mergeCell ref="C55:C58"/>
-    <mergeCell ref="B59:B63"/>
-    <mergeCell ref="C59:C63"/>
-    <mergeCell ref="B45:B49"/>
-    <mergeCell ref="C45:C49"/>
-    <mergeCell ref="B50:B54"/>
-    <mergeCell ref="C50:C54"/>
-    <mergeCell ref="C31:C36"/>
-    <mergeCell ref="B31:B36"/>
-    <mergeCell ref="C37:C41"/>
-    <mergeCell ref="B37:B41"/>
-    <mergeCell ref="B42:B44"/>
-    <mergeCell ref="C42:C44"/>
-    <mergeCell ref="C16:C26"/>
-    <mergeCell ref="B16:B26"/>
-    <mergeCell ref="C27:C30"/>
-    <mergeCell ref="B27:B30"/>
-    <mergeCell ref="B3:B6"/>
-    <mergeCell ref="C3:C6"/>
-    <mergeCell ref="B7:B10"/>
-    <mergeCell ref="C7:C10"/>
-    <mergeCell ref="B11:B15"/>
-    <mergeCell ref="C11:C15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4115,36 +4144,36 @@
       </c>
     </row>
     <row r="3" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D3" s="83" t="s">
+      <c r="D3" s="87" t="s">
         <v>8</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F3" s="80" t="s">
+      <c r="F3" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="G3" s="81"/>
-      <c r="H3" s="81"/>
-      <c r="I3" s="82"/>
-      <c r="J3" s="80" t="s">
+      <c r="G3" s="85"/>
+      <c r="H3" s="85"/>
+      <c r="I3" s="86"/>
+      <c r="J3" s="84" t="s">
         <v>2</v>
       </c>
-      <c r="K3" s="81"/>
-      <c r="L3" s="81"/>
-      <c r="M3" s="82"/>
-      <c r="N3" s="80" t="s">
+      <c r="K3" s="85"/>
+      <c r="L3" s="85"/>
+      <c r="M3" s="86"/>
+      <c r="N3" s="84" t="s">
         <v>3</v>
       </c>
-      <c r="O3" s="81"/>
-      <c r="P3" s="81"/>
-      <c r="Q3" s="82"/>
+      <c r="O3" s="85"/>
+      <c r="P3" s="85"/>
+      <c r="Q3" s="86"/>
       <c r="R3" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="4:18" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D4" s="84"/>
+      <c r="D4" s="88"/>
       <c r="E4" s="4" t="s">
         <v>4</v>
       </c>
@@ -4315,36 +4344,36 @@
       </c>
     </row>
     <row r="15" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D15" s="83" t="s">
+      <c r="D15" s="87" t="s">
         <v>8</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F15" s="80" t="s">
+      <c r="F15" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="G15" s="81"/>
-      <c r="H15" s="81"/>
-      <c r="I15" s="82"/>
-      <c r="J15" s="80" t="s">
+      <c r="G15" s="85"/>
+      <c r="H15" s="85"/>
+      <c r="I15" s="86"/>
+      <c r="J15" s="84" t="s">
         <v>2</v>
       </c>
-      <c r="K15" s="81"/>
-      <c r="L15" s="81"/>
-      <c r="M15" s="82"/>
-      <c r="N15" s="80" t="s">
+      <c r="K15" s="85"/>
+      <c r="L15" s="85"/>
+      <c r="M15" s="86"/>
+      <c r="N15" s="84" t="s">
         <v>3</v>
       </c>
-      <c r="O15" s="81"/>
-      <c r="P15" s="81"/>
-      <c r="Q15" s="82"/>
+      <c r="O15" s="85"/>
+      <c r="P15" s="85"/>
+      <c r="Q15" s="86"/>
       <c r="R15" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="16" spans="4:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D16" s="84"/>
+      <c r="D16" s="88"/>
       <c r="E16" s="4" t="s">
         <v>4</v>
       </c>
@@ -4532,200 +4561,210 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="B2:B39"/>
+  <dimension ref="B2:B41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="245.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="85" t="s">
+      <c r="B2" s="63" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="3" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="86" t="s">
+      <c r="B3" s="64" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="4" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="85" t="s">
+      <c r="B4" s="63" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="5" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="87" t="s">
+      <c r="B5" s="65" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="6" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="85" t="s">
+      <c r="B6" s="63" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="7" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="87" t="s">
+      <c r="B7" s="65" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="8" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="85" t="s">
+      <c r="B8" s="63" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="9" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="87" t="s">
+      <c r="B9" s="65" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="10" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="85" t="s">
+      <c r="B10" s="63" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="11" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="87" t="s">
+      <c r="B11" s="65" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="12" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="85" t="s">
+      <c r="B12" s="63" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="13" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="87" t="s">
+      <c r="B13" s="65" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="14" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="85" t="s">
+      <c r="B14" s="63" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="15" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="87" t="s">
+      <c r="B15" s="65" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="16" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="85" t="s">
+      <c r="B16" s="63" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="17" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="87" t="s">
+      <c r="B17" s="65" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="18" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="85" t="s">
+      <c r="B18" s="63" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="19" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="86" t="s">
+      <c r="B19" s="64" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="20" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="85" t="s">
+      <c r="B20" s="63" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="21" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="87" t="s">
+      <c r="B21" s="65" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="22" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="85" t="s">
+      <c r="B22" s="63" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="23" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="87" t="s">
+      <c r="B23" s="65" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="24" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="85" t="s">
+      <c r="B24" s="63" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="25" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="86" t="s">
+      <c r="B25" s="64" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="26" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="85" t="s">
+      <c r="B26" s="63" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="27" spans="2:2" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="B27" s="87" t="s">
+      <c r="B27" s="65" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="28" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="85" t="s">
+      <c r="B28" s="63" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="29" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="87" t="s">
+      <c r="B29" s="65" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="30" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="85" t="s">
+      <c r="B30" s="63" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="31" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="87" t="s">
+      <c r="B31" s="65" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="32" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="85" t="s">
+      <c r="B32" s="63" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="33" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="87" t="s">
+      <c r="B33" s="65" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="34" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="63" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="35" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="87" t="s">
+      <c r="B35" s="65" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="36" spans="2:2" ht="15" x14ac:dyDescent="0.3">
-      <c r="B36" s="85" t="s">
+      <c r="B36" s="63" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="37" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B37" s="87" t="s">
+      <c r="B37" s="65" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="38" spans="2:2" ht="15" x14ac:dyDescent="0.3">
-      <c r="B38" s="85" t="s">
+      <c r="B38" s="63" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="39" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B39" s="87" t="s">
+      <c r="B39" s="65" t="s">
         <v>133</v>
+      </c>
+    </row>
+    <row r="40" spans="2:2" ht="15" x14ac:dyDescent="0.3">
+      <c r="B40" s="63" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="41" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B41" s="65" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -4735,6 +4774,7 @@
     <hyperlink ref="B25" r:id="rId3" xr:uid="{201ECACC-0140-4555-B2A5-3873862F9FE5}"/>
     <hyperlink ref="B37" r:id="rId4" xr:uid="{F3266E3B-CA49-451D-9077-A713C3165DF0}"/>
     <hyperlink ref="B39" r:id="rId5" xr:uid="{CBD12324-3408-4DAF-B1DD-D30DBDA42E22}"/>
+    <hyperlink ref="B41" r:id="rId6" location="enable-publish-to-web-as-an-administrator" xr:uid="{929E3321-EF11-4327-9F10-293942C70B36}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
submimt the progress report 2
</commit_message>
<xml_diff>
--- a/DocumentsAndReports/0. WorkLog_Charts.xlsx
+++ b/DocumentsAndReports/0. WorkLog_Charts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qhung\Videos\CSIS4495 - Applied Research  Project\W26_4495_S2_HughT\DocumentsAndReports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{085CCC51-433A-4200-8045-8D444ACF3AD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CD54478-46F9-4CCB-A6FF-316A0AC32296}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E067A1E6-0DC4-42DD-AAF8-D95EFF7A112F}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="151">
   <si>
     <t>January</t>
   </si>
@@ -350,9 +350,6 @@
   </si>
   <si>
     <t>- Made the video, finalized the midterm report</t>
-  </si>
-  <si>
-    <t>THE ADJUSTED PLAN</t>
   </si>
   <si>
     <t>- Build front-end for dashboard</t>
@@ -883,6 +880,45 @@
   </si>
   <si>
     <t>https://learn.microsoft.com/en-us/power-bi/collaborate-share/service-publish-to-web#enable-publish-to-web-as-an-administrator</t>
+  </si>
+  <si>
+    <t>https://www.netsuite.com/portal/resource/articles/accounting/sales-kpis.shtml</t>
+  </si>
+  <si>
+    <t>22. Tableau, Great Examples &amp; Templates of Sales Dashboards</t>
+  </si>
+  <si>
+    <t>https://www.tableau.com/dashboard/sales-dashboard-examples-and-templates</t>
+  </si>
+  <si>
+    <t>21. Austin Caldwell , 21 Sales KPIs for Sales Teams to Track in 2023 (Jan 26, 2023)</t>
+  </si>
+  <si>
+    <t>23. Spider Strategies, Sales KPIs</t>
+  </si>
+  <si>
+    <t>https://www.spiderstrategies.com/kpi/department/sales/</t>
+  </si>
+  <si>
+    <t>24. Orisha, 12 Sales KPIs to measures performance and customer satisfaction (Sept 16, 2025)</t>
+  </si>
+  <si>
+    <t>https://commerce.orisha.com/blog/kpi-sale-store/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Researched sales KPIs for business </t>
+  </si>
+  <si>
+    <t>- Wrote progress report 2</t>
+  </si>
+  <si>
+    <t>-  Chat GPT's prompts:</t>
+  </si>
+  <si>
+    <t>THE ADJUSTED PLAN AT MIDTERM REPORT</t>
+  </si>
+  <si>
+    <t>THE ADJUSTED PLAN AT PROGRESS REPORT 2</t>
   </si>
 </sst>
 </file>
@@ -1484,7 +1520,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1604,9 +1640,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="33" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
@@ -1634,6 +1667,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="28" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -1652,6 +1686,12 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="15" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -1679,12 +1719,6 @@
     <xf numFmtId="14" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="15" fontId="7" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1700,7 +1734,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2679,6 +2712,570 @@
             <a:lumMod val="40000"/>
             <a:lumOff val="60000"/>
           </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent6">
+              <a:lumMod val="40000"/>
+              <a:lumOff val="60000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent2"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>30480</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>59057</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>592455</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>209550</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="16" name="Rectangle: Rounded Corners 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4F9B035D-9BE2-47B4-AD4B-8F42ED6FB9AB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3931920" y="3838577"/>
+          <a:ext cx="1171575" cy="150493"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent2"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent6">
+              <a:lumMod val="40000"/>
+              <a:lumOff val="60000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent2"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>59054</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>590550</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>219075</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="17" name="Rectangle: Rounded Corners 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F982C586-C91B-472F-BD6A-FAC701D8B4FD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4530090" y="4105274"/>
+          <a:ext cx="571500" cy="160021"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent2"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent6">
+              <a:lumMod val="40000"/>
+              <a:lumOff val="60000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent2"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>26671</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>55246</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>592455</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>209550</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="18" name="Rectangle: Rounded Corners 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B6FC15CA-15F9-4106-9262-3954F38E3CD0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5147311" y="4368166"/>
+          <a:ext cx="1175384" cy="154304"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent2"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent6">
+              <a:lumMod val="40000"/>
+              <a:lumOff val="60000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent2"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>28574</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>53341</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>569595</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>205740</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="19" name="Rectangle: Rounded Corners 18">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{87DBF415-3022-406D-B7CA-9F99916A2FF3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5758814" y="4632961"/>
+          <a:ext cx="1760221" cy="152399"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent6">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent6">
+              <a:lumMod val="40000"/>
+              <a:lumOff val="60000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent2"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>30480</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>57149</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>592454</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="20" name="Rectangle: Rounded Corners 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0C7F4CFD-8998-4A17-824C-31CD4CBCB6FB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6979920" y="7364729"/>
+          <a:ext cx="1781174" cy="133351"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent6">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent6">
+              <a:lumMod val="40000"/>
+              <a:lumOff val="60000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent2"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>55246</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>573405</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>209550</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="21" name="Rectangle: Rounded Corners 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8F83CD28-EA6D-4B69-A6E2-BC0B8AEC89E5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7578090" y="5168266"/>
+          <a:ext cx="1773555" cy="154304"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent6">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent6">
+              <a:lumMod val="40000"/>
+              <a:lumOff val="60000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent2"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>30481</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>55244</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>579120</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>201929</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="22" name="Rectangle: Rounded Corners 21">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7E73BE93-C7B8-43A1-86D2-18D30485E7FC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9418321" y="5434964"/>
+          <a:ext cx="548639" cy="146685"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent6">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent6">
+              <a:lumMod val="40000"/>
+              <a:lumOff val="60000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent2"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>26670</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>609599</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>194310</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="23" name="Rectangle: Rounded Corners 22">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9A945971-56D6-4557-AD74-6EF7B51BC9C7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5756910" y="7520940"/>
+          <a:ext cx="1192529" cy="148590"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent2"/>
         </a:solidFill>
         <a:ln>
           <a:solidFill>
@@ -3059,11 +3656,11 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="83">
+    <row r="3" spans="2:4" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="74">
         <v>45683</v>
       </c>
-      <c r="C3" s="82">
+      <c r="C3" s="73">
         <v>2</v>
       </c>
       <c r="D3" s="35" t="s">
@@ -3071,31 +3668,31 @@
       </c>
     </row>
     <row r="4" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="83"/>
-      <c r="C4" s="82"/>
+      <c r="B4" s="74"/>
+      <c r="C4" s="73"/>
       <c r="D4" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="83"/>
-      <c r="C5" s="82"/>
+      <c r="B5" s="74"/>
+      <c r="C5" s="73"/>
       <c r="D5" s="41" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="83"/>
-      <c r="C6" s="82"/>
+      <c r="B6" s="74"/>
+      <c r="C6" s="73"/>
       <c r="D6" s="42" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="83">
+    <row r="7" spans="2:4" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="74">
         <v>45684</v>
       </c>
-      <c r="C7" s="82">
+      <c r="C7" s="73">
         <v>1.5</v>
       </c>
       <c r="D7" s="36" t="s">
@@ -3103,31 +3700,31 @@
       </c>
     </row>
     <row r="8" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="83"/>
-      <c r="C8" s="82"/>
+      <c r="B8" s="74"/>
+      <c r="C8" s="73"/>
       <c r="D8" s="37" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="9" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="83"/>
-      <c r="C9" s="82"/>
+      <c r="B9" s="74"/>
+      <c r="C9" s="73"/>
       <c r="D9" s="43" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="10" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="83"/>
-      <c r="C10" s="82"/>
+      <c r="B10" s="74"/>
+      <c r="C10" s="73"/>
       <c r="D10" s="44" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="83">
+      <c r="B11" s="74">
         <v>45686</v>
       </c>
-      <c r="C11" s="82">
+      <c r="C11" s="73">
         <v>3</v>
       </c>
       <c r="D11" s="35" t="s">
@@ -3135,38 +3732,38 @@
       </c>
     </row>
     <row r="12" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="83"/>
-      <c r="C12" s="82"/>
+      <c r="B12" s="74"/>
+      <c r="C12" s="73"/>
       <c r="D12" s="35" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="83"/>
-      <c r="C13" s="82"/>
+      <c r="B13" s="74"/>
+      <c r="C13" s="73"/>
       <c r="D13" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="83"/>
-      <c r="C14" s="82"/>
+      <c r="B14" s="74"/>
+      <c r="C14" s="73"/>
       <c r="D14" s="45" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="83"/>
-      <c r="C15" s="82"/>
+      <c r="B15" s="74"/>
+      <c r="C15" s="73"/>
       <c r="D15" s="42" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="83">
+      <c r="B16" s="74">
         <v>46053</v>
       </c>
-      <c r="C16" s="82">
+      <c r="C16" s="73">
         <v>4</v>
       </c>
       <c r="D16" s="38" t="s">
@@ -3174,80 +3771,80 @@
       </c>
     </row>
     <row r="17" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="83"/>
-      <c r="C17" s="82"/>
+      <c r="B17" s="74"/>
+      <c r="C17" s="73"/>
       <c r="D17" s="35" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="83"/>
-      <c r="C18" s="82"/>
+      <c r="B18" s="74"/>
+      <c r="C18" s="73"/>
       <c r="D18" s="35" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="19" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="83"/>
-      <c r="C19" s="82"/>
+      <c r="B19" s="74"/>
+      <c r="C19" s="73"/>
       <c r="D19" s="35" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="20" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="83"/>
-      <c r="C20" s="82"/>
+      <c r="B20" s="74"/>
+      <c r="C20" s="73"/>
       <c r="D20" s="35" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="21" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="83"/>
-      <c r="C21" s="82"/>
+      <c r="B21" s="74"/>
+      <c r="C21" s="73"/>
       <c r="D21" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="83"/>
-      <c r="C22" s="82"/>
+      <c r="B22" s="74"/>
+      <c r="C22" s="73"/>
       <c r="D22" s="45" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="23" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="83"/>
-      <c r="C23" s="82"/>
+      <c r="B23" s="74"/>
+      <c r="C23" s="73"/>
       <c r="D23" s="41" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="24" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="83"/>
-      <c r="C24" s="82"/>
+      <c r="B24" s="74"/>
+      <c r="C24" s="73"/>
       <c r="D24" s="41" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="25" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="83"/>
-      <c r="C25" s="82"/>
+      <c r="B25" s="74"/>
+      <c r="C25" s="73"/>
       <c r="D25" s="41" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="26" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="83"/>
-      <c r="C26" s="82"/>
+      <c r="B26" s="74"/>
+      <c r="C26" s="73"/>
       <c r="D26" s="46" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="27" spans="2:4" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="83">
+      <c r="B27" s="74">
         <v>46054</v>
       </c>
-      <c r="C27" s="82">
+      <c r="C27" s="73">
         <v>1</v>
       </c>
       <c r="D27" s="35" t="s">
@@ -3255,31 +3852,31 @@
       </c>
     </row>
     <row r="28" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="83"/>
-      <c r="C28" s="82"/>
+      <c r="B28" s="74"/>
+      <c r="C28" s="73"/>
       <c r="D28" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="29" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="83"/>
-      <c r="C29" s="82"/>
+      <c r="B29" s="74"/>
+      <c r="C29" s="73"/>
       <c r="D29" s="41" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="30" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="83"/>
-      <c r="C30" s="82"/>
+      <c r="B30" s="74"/>
+      <c r="C30" s="73"/>
       <c r="D30" s="42" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="31" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B31" s="83">
+      <c r="B31" s="74">
         <v>46055</v>
       </c>
-      <c r="C31" s="82">
+      <c r="C31" s="73">
         <v>4</v>
       </c>
       <c r="D31" s="39" t="s">
@@ -3287,45 +3884,45 @@
       </c>
     </row>
     <row r="32" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B32" s="83"/>
-      <c r="C32" s="82"/>
+      <c r="B32" s="74"/>
+      <c r="C32" s="73"/>
       <c r="D32" s="40" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="33" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="83"/>
-      <c r="C33" s="82"/>
+      <c r="B33" s="74"/>
+      <c r="C33" s="73"/>
       <c r="D33" s="40" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="34" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B34" s="83"/>
-      <c r="C34" s="82"/>
+      <c r="B34" s="74"/>
+      <c r="C34" s="73"/>
       <c r="D34" s="40" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="35" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B35" s="83"/>
-      <c r="C35" s="82"/>
+      <c r="B35" s="74"/>
+      <c r="C35" s="73"/>
       <c r="D35" s="47" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="36" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B36" s="83"/>
-      <c r="C36" s="82"/>
+      <c r="B36" s="74"/>
+      <c r="C36" s="73"/>
       <c r="D36" s="48" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="37" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="83">
+      <c r="B37" s="74">
         <v>46056</v>
       </c>
-      <c r="C37" s="82">
+      <c r="C37" s="73">
         <v>3</v>
       </c>
       <c r="D37" s="35" t="s">
@@ -3333,38 +3930,38 @@
       </c>
     </row>
     <row r="38" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B38" s="83"/>
-      <c r="C38" s="82"/>
+      <c r="B38" s="74"/>
+      <c r="C38" s="73"/>
       <c r="D38" s="35" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="39" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B39" s="83"/>
-      <c r="C39" s="82"/>
+      <c r="B39" s="74"/>
+      <c r="C39" s="73"/>
       <c r="D39" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="40" spans="2:4" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B40" s="83"/>
-      <c r="C40" s="82"/>
+      <c r="B40" s="74"/>
+      <c r="C40" s="73"/>
       <c r="D40" s="41" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="41" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B41" s="83"/>
-      <c r="C41" s="82"/>
+      <c r="B41" s="74"/>
+      <c r="C41" s="73"/>
       <c r="D41" s="42" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="42" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B42" s="83">
+      <c r="B42" s="74">
         <v>46057</v>
       </c>
-      <c r="C42" s="82">
+      <c r="C42" s="73">
         <v>4</v>
       </c>
       <c r="D42" s="38" t="s">
@@ -3372,24 +3969,24 @@
       </c>
     </row>
     <row r="43" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B43" s="83"/>
-      <c r="C43" s="82"/>
+      <c r="B43" s="74"/>
+      <c r="C43" s="73"/>
       <c r="D43" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="44" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B44" s="83"/>
-      <c r="C44" s="82"/>
+      <c r="B44" s="74"/>
+      <c r="C44" s="73"/>
       <c r="D44" s="42" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="45" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B45" s="73">
+      <c r="B45" s="75">
         <v>46059</v>
       </c>
-      <c r="C45" s="76">
+      <c r="C45" s="78">
         <v>2</v>
       </c>
       <c r="D45" s="50" t="s">
@@ -3397,38 +3994,38 @@
       </c>
     </row>
     <row r="46" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B46" s="74"/>
-      <c r="C46" s="77"/>
+      <c r="B46" s="76"/>
+      <c r="C46" s="79"/>
       <c r="D46" s="49" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="47" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B47" s="74"/>
-      <c r="C47" s="77"/>
+      <c r="B47" s="76"/>
+      <c r="C47" s="79"/>
       <c r="D47" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="48" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B48" s="74"/>
-      <c r="C48" s="77"/>
+      <c r="B48" s="76"/>
+      <c r="C48" s="79"/>
       <c r="D48" s="42" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="49" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B49" s="75"/>
-      <c r="C49" s="78"/>
+      <c r="B49" s="77"/>
+      <c r="C49" s="80"/>
       <c r="D49" s="46" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="50" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B50" s="73">
+      <c r="B50" s="75">
         <v>46061</v>
       </c>
-      <c r="C50" s="76">
+      <c r="C50" s="78">
         <v>1.5</v>
       </c>
       <c r="D50" s="50" t="s">
@@ -3436,38 +4033,38 @@
       </c>
     </row>
     <row r="51" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B51" s="74"/>
-      <c r="C51" s="77"/>
+      <c r="B51" s="76"/>
+      <c r="C51" s="79"/>
       <c r="D51" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="52" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B52" s="74"/>
-      <c r="C52" s="77"/>
+      <c r="B52" s="76"/>
+      <c r="C52" s="79"/>
       <c r="D52" s="42" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="53" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B53" s="74"/>
-      <c r="C53" s="77"/>
+      <c r="B53" s="76"/>
+      <c r="C53" s="79"/>
       <c r="D53" s="42" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="54" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B54" s="75"/>
-      <c r="C54" s="78"/>
+      <c r="B54" s="77"/>
+      <c r="C54" s="80"/>
       <c r="D54" s="46" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="55" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="73">
+      <c r="B55" s="75">
         <v>46062</v>
       </c>
-      <c r="C55" s="76">
+      <c r="C55" s="78">
         <v>2</v>
       </c>
       <c r="D55" s="54" t="s">
@@ -3475,31 +4072,31 @@
       </c>
     </row>
     <row r="56" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B56" s="74"/>
-      <c r="C56" s="77"/>
+      <c r="B56" s="76"/>
+      <c r="C56" s="79"/>
       <c r="D56" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="57" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B57" s="74"/>
-      <c r="C57" s="77"/>
+      <c r="B57" s="76"/>
+      <c r="C57" s="79"/>
       <c r="D57" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="58" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B58" s="75"/>
-      <c r="C58" s="78"/>
+      <c r="B58" s="77"/>
+      <c r="C58" s="80"/>
       <c r="D58" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="59" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="73">
+      <c r="B59" s="75">
         <v>46063</v>
       </c>
-      <c r="C59" s="76">
+      <c r="C59" s="78">
         <v>3</v>
       </c>
       <c r="D59" s="54" t="s">
@@ -3507,38 +4104,38 @@
       </c>
     </row>
     <row r="60" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B60" s="74"/>
-      <c r="C60" s="77"/>
+      <c r="B60" s="76"/>
+      <c r="C60" s="79"/>
       <c r="D60" s="55" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="61" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B61" s="74"/>
-      <c r="C61" s="77"/>
+      <c r="B61" s="76"/>
+      <c r="C61" s="79"/>
       <c r="D61" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="62" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B62" s="74"/>
-      <c r="C62" s="77"/>
+      <c r="B62" s="76"/>
+      <c r="C62" s="79"/>
       <c r="D62" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="63" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B63" s="75"/>
-      <c r="C63" s="78"/>
+      <c r="B63" s="77"/>
+      <c r="C63" s="80"/>
       <c r="D63" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="64" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B64" s="73">
+      <c r="B64" s="75">
         <v>46064</v>
       </c>
-      <c r="C64" s="76">
+      <c r="C64" s="78">
         <v>3</v>
       </c>
       <c r="D64" s="54" t="s">
@@ -3546,75 +4143,75 @@
       </c>
     </row>
     <row r="65" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B65" s="74"/>
-      <c r="C65" s="77"/>
+      <c r="B65" s="76"/>
+      <c r="C65" s="79"/>
       <c r="D65" s="55" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="66" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B66" s="74"/>
-      <c r="C66" s="77"/>
+      <c r="B66" s="76"/>
+      <c r="C66" s="79"/>
       <c r="D66" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="67" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B67" s="74"/>
-      <c r="C67" s="77"/>
+      <c r="B67" s="76"/>
+      <c r="C67" s="79"/>
       <c r="D67" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="68" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B68" s="75"/>
-      <c r="C68" s="78"/>
+      <c r="B68" s="77"/>
+      <c r="C68" s="80"/>
       <c r="D68" s="46" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="69" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B69" s="79">
+    <row r="69" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B69" s="81">
         <v>46066</v>
       </c>
-      <c r="C69" s="76">
+      <c r="C69" s="78">
         <v>2</v>
       </c>
       <c r="D69" s="54" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="70" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B70" s="80"/>
-      <c r="C70" s="77"/>
+    <row r="70" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B70" s="82"/>
+      <c r="C70" s="79"/>
       <c r="D70" s="55" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="71" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B71" s="80"/>
-      <c r="C71" s="77"/>
+    <row r="71" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B71" s="82"/>
+      <c r="C71" s="79"/>
       <c r="D71" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="72" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B72" s="80"/>
-      <c r="C72" s="77"/>
+      <c r="B72" s="82"/>
+      <c r="C72" s="79"/>
       <c r="D72" s="42" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="73" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B73" s="80"/>
-      <c r="C73" s="77"/>
+      <c r="B73" s="82"/>
+      <c r="C73" s="79"/>
       <c r="D73" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="74" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B74" s="81"/>
-      <c r="C74" s="78"/>
+      <c r="B74" s="83"/>
+      <c r="C74" s="80"/>
       <c r="D74" s="46" t="s">
         <v>21</v>
       </c>
@@ -3771,14 +4368,14 @@
       <c r="C94" s="70">
         <v>3</v>
       </c>
-      <c r="D94" s="58" t="s">
+      <c r="D94" s="57" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="95" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B95" s="68"/>
       <c r="C95" s="71"/>
-      <c r="D95" s="59" t="s">
+      <c r="D95" s="58" t="s">
         <v>66</v>
       </c>
     </row>
@@ -3822,13 +4419,13 @@
       </c>
     </row>
     <row r="101" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B101" s="60">
+      <c r="B101" s="59">
         <v>46076</v>
       </c>
-      <c r="C101" s="61">
+      <c r="C101" s="60">
         <v>4</v>
       </c>
-      <c r="D101" s="62" t="s">
+      <c r="D101" s="61" t="s">
         <v>85</v>
       </c>
     </row>
@@ -3840,14 +4437,14 @@
         <v>2</v>
       </c>
       <c r="D102" s="54" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="103" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B103" s="68"/>
       <c r="C103" s="71"/>
       <c r="D103" s="55" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="104" spans="2:4" x14ac:dyDescent="0.3">
@@ -3861,14 +4458,14 @@
       <c r="B105" s="68"/>
       <c r="C105" s="71"/>
       <c r="D105" s="42" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="106" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B106" s="69"/>
       <c r="C106" s="72"/>
       <c r="D106" s="46" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="107" spans="2:4" x14ac:dyDescent="0.3">
@@ -3878,94 +4475,106 @@
       <c r="C107" s="70">
         <v>1</v>
       </c>
-      <c r="D107" s="66" t="s">
-        <v>94</v>
+      <c r="D107" s="65" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="108" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B108" s="68"/>
       <c r="C108" s="71"/>
       <c r="D108" s="55" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="109" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B109" s="68"/>
       <c r="C109" s="71"/>
       <c r="D109" s="42" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="110" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B110" s="68"/>
       <c r="C110" s="71"/>
       <c r="D110" s="42" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="111" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B111" s="69"/>
       <c r="C111" s="72"/>
-      <c r="D111" s="89" t="s">
-        <v>95</v>
+      <c r="D111" s="66" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="112" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B112" s="57">
+      <c r="B112" s="67">
         <v>46079</v>
       </c>
-      <c r="C112" s="56">
+      <c r="C112" s="70">
         <v>2</v>
       </c>
-      <c r="D112" s="66" t="s">
+      <c r="D112" s="65" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="113" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B113" s="68"/>
+      <c r="C113" s="71"/>
+      <c r="D113" s="55" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="114" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B114" s="68"/>
+      <c r="C114" s="71"/>
+      <c r="D114" s="42" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="113" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B113" s="32"/>
-      <c r="C113" s="32"/>
-      <c r="D113" s="55" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="114" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B114" s="32"/>
-      <c r="C114" s="32"/>
-      <c r="D114" s="42" t="s">
+    <row r="115" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B115" s="69"/>
+      <c r="C115" s="72"/>
+      <c r="D115" s="46" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="115" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B115" s="56"/>
-      <c r="C115" s="56"/>
-      <c r="D115" s="42" t="s">
-        <v>136</v>
-      </c>
-    </row>
     <row r="116" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B116" s="32"/>
-      <c r="C116" s="32"/>
-      <c r="D116" s="33"/>
+      <c r="B116" s="67">
+        <v>46083</v>
+      </c>
+      <c r="C116" s="70">
+        <v>3</v>
+      </c>
+      <c r="D116" s="65" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="117" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B117" s="32"/>
-      <c r="C117" s="32"/>
-      <c r="D117" s="33"/>
+      <c r="B117" s="68"/>
+      <c r="C117" s="71"/>
+      <c r="D117" s="55" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="118" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B118" s="56"/>
-      <c r="C118" s="56"/>
-      <c r="D118" s="51"/>
-    </row>
-    <row r="119" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B119" s="32"/>
-      <c r="C119" s="32"/>
-      <c r="D119" s="33"/>
+      <c r="B118" s="68"/>
+      <c r="C118" s="71"/>
+      <c r="D118" s="55" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="119" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B119" s="69"/>
+      <c r="C119" s="72"/>
+      <c r="D119" s="46" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="120" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B120" s="32"/>
-      <c r="C120" s="32"/>
-      <c r="D120" s="33"/>
+      <c r="B120" s="56"/>
+      <c r="C120" s="56"/>
+      <c r="D120" s="51"/>
     </row>
     <row r="121" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B121" s="56"/>
@@ -4073,35 +4682,11 @@
       <c r="D141" s="33"/>
     </row>
   </sheetData>
-  <mergeCells count="42">
-    <mergeCell ref="B107:B111"/>
-    <mergeCell ref="C107:C111"/>
-    <mergeCell ref="C16:C26"/>
-    <mergeCell ref="B16:B26"/>
-    <mergeCell ref="C27:C30"/>
-    <mergeCell ref="B27:B30"/>
-    <mergeCell ref="B3:B6"/>
-    <mergeCell ref="C3:C6"/>
-    <mergeCell ref="B7:B10"/>
-    <mergeCell ref="C7:C10"/>
-    <mergeCell ref="B11:B15"/>
-    <mergeCell ref="C11:C15"/>
-    <mergeCell ref="C31:C36"/>
-    <mergeCell ref="B31:B36"/>
-    <mergeCell ref="C37:C41"/>
-    <mergeCell ref="B37:B41"/>
-    <mergeCell ref="B42:B44"/>
-    <mergeCell ref="C42:C44"/>
-    <mergeCell ref="B55:B58"/>
-    <mergeCell ref="C55:C58"/>
-    <mergeCell ref="B59:B63"/>
-    <mergeCell ref="C59:C63"/>
-    <mergeCell ref="B45:B49"/>
-    <mergeCell ref="C45:C49"/>
-    <mergeCell ref="B50:B54"/>
-    <mergeCell ref="C50:C54"/>
-    <mergeCell ref="B64:B68"/>
-    <mergeCell ref="C64:C68"/>
+  <mergeCells count="46">
+    <mergeCell ref="B112:B115"/>
+    <mergeCell ref="C112:C115"/>
+    <mergeCell ref="B116:B119"/>
+    <mergeCell ref="C116:C119"/>
     <mergeCell ref="B69:B74"/>
     <mergeCell ref="C69:C74"/>
     <mergeCell ref="B75:B81"/>
@@ -4116,6 +4701,34 @@
     <mergeCell ref="C89:C93"/>
     <mergeCell ref="B94:B96"/>
     <mergeCell ref="C94:C96"/>
+    <mergeCell ref="B45:B49"/>
+    <mergeCell ref="C45:C49"/>
+    <mergeCell ref="B50:B54"/>
+    <mergeCell ref="C50:C54"/>
+    <mergeCell ref="B64:B68"/>
+    <mergeCell ref="C64:C68"/>
+    <mergeCell ref="B3:B6"/>
+    <mergeCell ref="C3:C6"/>
+    <mergeCell ref="B7:B10"/>
+    <mergeCell ref="C7:C10"/>
+    <mergeCell ref="B11:B15"/>
+    <mergeCell ref="C11:C15"/>
+    <mergeCell ref="B107:B111"/>
+    <mergeCell ref="C107:C111"/>
+    <mergeCell ref="C16:C26"/>
+    <mergeCell ref="B16:B26"/>
+    <mergeCell ref="C27:C30"/>
+    <mergeCell ref="B27:B30"/>
+    <mergeCell ref="C31:C36"/>
+    <mergeCell ref="B31:B36"/>
+    <mergeCell ref="C37:C41"/>
+    <mergeCell ref="B37:B41"/>
+    <mergeCell ref="B42:B44"/>
+    <mergeCell ref="C42:C44"/>
+    <mergeCell ref="B55:B58"/>
+    <mergeCell ref="C55:C58"/>
+    <mergeCell ref="B59:B63"/>
+    <mergeCell ref="C59:C63"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4126,7 +4739,7 @@
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
   </sheetPr>
-  <dimension ref="D2:R23"/>
+  <dimension ref="D2:R35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="8.88671875" style="2"/>
@@ -4340,7 +4953,7 @@
     </row>
     <row r="14" spans="4:18" s="53" customFormat="1" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D14" s="52" t="s">
-        <v>86</v>
+        <v>149</v>
       </c>
     </row>
     <row r="15" spans="4:18" x14ac:dyDescent="0.3">
@@ -4538,8 +5151,226 @@
       <c r="Q23" s="14"/>
       <c r="R23" s="11"/>
     </row>
+    <row r="26" spans="4:18" ht="33.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D26" s="52" t="s">
+        <v>150</v>
+      </c>
+      <c r="E26" s="53"/>
+      <c r="F26" s="53"/>
+      <c r="G26" s="53"/>
+      <c r="H26" s="53"/>
+      <c r="I26" s="53"/>
+      <c r="J26" s="53"/>
+      <c r="K26" s="53"/>
+      <c r="L26" s="53"/>
+      <c r="M26" s="53"/>
+      <c r="N26" s="53"/>
+      <c r="O26" s="53"/>
+      <c r="P26" s="53"/>
+      <c r="Q26" s="53"/>
+      <c r="R26" s="53"/>
+    </row>
+    <row r="27" spans="4:18" x14ac:dyDescent="0.3">
+      <c r="D27" s="87" t="s">
+        <v>8</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="F27" s="84" t="s">
+        <v>1</v>
+      </c>
+      <c r="G27" s="85"/>
+      <c r="H27" s="85"/>
+      <c r="I27" s="86"/>
+      <c r="J27" s="84" t="s">
+        <v>2</v>
+      </c>
+      <c r="K27" s="85"/>
+      <c r="L27" s="85"/>
+      <c r="M27" s="86"/>
+      <c r="N27" s="84" t="s">
+        <v>3</v>
+      </c>
+      <c r="O27" s="85"/>
+      <c r="P27" s="85"/>
+      <c r="Q27" s="86"/>
+      <c r="R27" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="4:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D28" s="88"/>
+      <c r="E28" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="I28" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="J28" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="K28" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="L28" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M28" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="N28" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="O28" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="P28" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q28" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="R28" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="4:18" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D29" s="27" t="s">
+        <v>9</v>
+      </c>
+      <c r="E29" s="8"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="16"/>
+      <c r="H29" s="16"/>
+      <c r="I29" s="17"/>
+      <c r="J29" s="24"/>
+      <c r="K29" s="16"/>
+      <c r="L29" s="16"/>
+      <c r="M29" s="17"/>
+      <c r="N29" s="9"/>
+      <c r="Q29" s="10"/>
+      <c r="R29" s="8"/>
+    </row>
+    <row r="30" spans="4:18" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D30" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="E30" s="8"/>
+      <c r="F30" s="18"/>
+      <c r="G30" s="19"/>
+      <c r="H30" s="19"/>
+      <c r="I30" s="20"/>
+      <c r="J30" s="25"/>
+      <c r="K30" s="19"/>
+      <c r="L30" s="19"/>
+      <c r="M30" s="20"/>
+      <c r="N30" s="9"/>
+      <c r="Q30" s="10"/>
+      <c r="R30" s="8"/>
+    </row>
+    <row r="31" spans="4:18" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D31" s="28" t="s">
+        <v>11</v>
+      </c>
+      <c r="E31" s="8"/>
+      <c r="F31" s="18"/>
+      <c r="G31" s="19"/>
+      <c r="H31" s="19"/>
+      <c r="I31" s="20"/>
+      <c r="J31" s="25"/>
+      <c r="K31" s="19"/>
+      <c r="L31" s="19"/>
+      <c r="M31" s="20"/>
+      <c r="N31" s="9"/>
+      <c r="Q31" s="10"/>
+      <c r="R31" s="8"/>
+    </row>
+    <row r="32" spans="4:18" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D32" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="E32" s="8"/>
+      <c r="F32" s="18"/>
+      <c r="G32" s="19"/>
+      <c r="H32" s="19"/>
+      <c r="I32" s="20"/>
+      <c r="J32" s="25"/>
+      <c r="K32" s="19"/>
+      <c r="L32" s="19"/>
+      <c r="M32" s="20"/>
+      <c r="N32" s="9"/>
+      <c r="Q32" s="10"/>
+      <c r="R32" s="8"/>
+    </row>
+    <row r="33" spans="4:18" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D33" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="E33" s="8"/>
+      <c r="F33" s="18"/>
+      <c r="G33" s="19"/>
+      <c r="H33" s="19"/>
+      <c r="I33" s="20"/>
+      <c r="J33" s="25"/>
+      <c r="K33" s="19"/>
+      <c r="L33" s="19"/>
+      <c r="M33" s="20"/>
+      <c r="N33" s="9"/>
+      <c r="Q33" s="10"/>
+      <c r="R33" s="8"/>
+    </row>
+    <row r="34" spans="4:18" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D34" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="E34" s="8"/>
+      <c r="F34" s="18"/>
+      <c r="G34" s="19"/>
+      <c r="H34" s="19"/>
+      <c r="I34" s="20"/>
+      <c r="J34" s="25"/>
+      <c r="K34" s="19"/>
+      <c r="L34" s="19"/>
+      <c r="M34" s="20"/>
+      <c r="N34" s="9"/>
+      <c r="Q34" s="10"/>
+      <c r="R34" s="8"/>
+    </row>
+    <row r="35" spans="4:18" ht="19.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D35" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="E35" s="11"/>
+      <c r="F35" s="21"/>
+      <c r="G35" s="22"/>
+      <c r="H35" s="22"/>
+      <c r="I35" s="23"/>
+      <c r="J35" s="26"/>
+      <c r="K35" s="22"/>
+      <c r="L35" s="22"/>
+      <c r="M35" s="23"/>
+      <c r="N35" s="12"/>
+      <c r="O35" s="13"/>
+      <c r="P35" s="13"/>
+      <c r="Q35" s="14"/>
+      <c r="R35" s="11"/>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="12">
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="F27:I27"/>
+    <mergeCell ref="J27:M27"/>
+    <mergeCell ref="N27:Q27"/>
     <mergeCell ref="F3:I3"/>
     <mergeCell ref="J3:M3"/>
     <mergeCell ref="N3:Q3"/>
@@ -4561,210 +5392,250 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="B2:B41"/>
+  <dimension ref="B2:B49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="245.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="63" t="s">
+      <c r="B2" s="62" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="3" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="63" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="3" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="64" t="s">
+    <row r="4" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="62" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="4" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="63" t="s">
+    <row r="5" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="64" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="5" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="65" t="s">
+    <row r="6" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="62" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="6" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="63" t="s">
+    <row r="7" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="64" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="65" t="s">
+    <row r="8" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="62" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="8" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="63" t="s">
+    <row r="9" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="64" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="9" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="65" t="s">
+    <row r="10" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="62" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="10" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="63" t="s">
+    <row r="11" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="64" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="11" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="65" t="s">
+    <row r="12" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="62" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="12" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="63" t="s">
+    <row r="13" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="64" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="13" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="65" t="s">
+    <row r="14" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="62" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="14" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="63" t="s">
+    <row r="15" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="64" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="15" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="65" t="s">
+    <row r="16" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="62" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="16" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="63" t="s">
+    <row r="17" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="64" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="17" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="65" t="s">
+    <row r="18" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="62" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="18" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="63" t="s">
+    <row r="19" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="63" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="19" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="64" t="s">
+    <row r="20" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="62" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="20" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="63" t="s">
+    <row r="21" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="64" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="21" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="65" t="s">
+    <row r="22" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="62" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="22" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="63" t="s">
+    <row r="23" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="64" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="23" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="65" t="s">
+    <row r="24" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="62" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="24" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="63" t="s">
+    <row r="25" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="63" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="25" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="64" t="s">
+    <row r="26" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="62" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="26" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="63" t="s">
+    <row r="27" spans="2:2" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="B27" s="64" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="27" spans="2:2" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="B27" s="65" t="s">
+    <row r="28" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="62" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="28" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="63" t="s">
+    <row r="29" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="64" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="29" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="65" t="s">
+    <row r="30" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="62" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="30" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="63" t="s">
+    <row r="31" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B31" s="64" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="31" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="65" t="s">
+    <row r="32" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="62" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="32" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="63" t="s">
+    <row r="33" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="64" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="33" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="65" t="s">
+    <row r="34" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="62" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="34" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="63" t="s">
+    <row r="35" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="64" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="35" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="65" t="s">
+    <row r="36" spans="2:2" ht="15" x14ac:dyDescent="0.3">
+      <c r="B36" s="62" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="37" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B37" s="64" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="36" spans="2:2" ht="15" x14ac:dyDescent="0.3">
-      <c r="B36" s="63" t="s">
+    <row r="38" spans="2:2" ht="15" x14ac:dyDescent="0.3">
+      <c r="B38" s="62" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="37" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B37" s="65" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="38" spans="2:2" ht="15" x14ac:dyDescent="0.3">
-      <c r="B38" s="63" t="s">
+    <row r="39" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B39" s="64" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="39" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B39" s="65" t="s">
-        <v>133</v>
-      </c>
-    </row>
     <row r="40" spans="2:2" ht="15" x14ac:dyDescent="0.3">
-      <c r="B40" s="63" t="s">
+      <c r="B40" s="62" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="41" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B41" s="64" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="41" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B41" s="65" t="s">
+    <row r="42" spans="2:2" ht="15" x14ac:dyDescent="0.3">
+      <c r="B42" s="62" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="43" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B43" s="64" t="s">
         <v>138</v>
+      </c>
+    </row>
+    <row r="44" spans="2:2" ht="15" x14ac:dyDescent="0.3">
+      <c r="B44" s="62" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="45" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B45" s="64" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="46" spans="2:2" ht="15" x14ac:dyDescent="0.3">
+      <c r="B46" s="62" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="47" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B47" s="64" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="48" spans="2:2" ht="15" x14ac:dyDescent="0.3">
+      <c r="B48" s="62" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="49" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B49" s="64" t="s">
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -4775,6 +5646,9 @@
     <hyperlink ref="B37" r:id="rId4" xr:uid="{F3266E3B-CA49-451D-9077-A713C3165DF0}"/>
     <hyperlink ref="B39" r:id="rId5" xr:uid="{CBD12324-3408-4DAF-B1DD-D30DBDA42E22}"/>
     <hyperlink ref="B41" r:id="rId6" location="enable-publish-to-web-as-an-administrator" xr:uid="{929E3321-EF11-4327-9F10-293942C70B36}"/>
+    <hyperlink ref="B43" r:id="rId7" xr:uid="{4EFC952B-9A09-44AD-AF56-146B4F568623}"/>
+    <hyperlink ref="B47" r:id="rId8" xr:uid="{BFE14320-69A1-490D-AB67-F9FA78E446C6}"/>
+    <hyperlink ref="B49" r:id="rId9" xr:uid="{7818186A-BA4A-4BB4-91D9-A4C948B644CE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
changed dataset, modified database
</commit_message>
<xml_diff>
--- a/DocumentsAndReports/0. WorkLog_Charts.xlsx
+++ b/DocumentsAndReports/0. WorkLog_Charts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qhung\Videos\CSIS4495 - Applied Research  Project\W26_4495_S2_HughT\DocumentsAndReports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CD54478-46F9-4CCB-A6FF-316A0AC32296}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF6898F5-01EE-4F15-9597-91B58E6B8A33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E067A1E6-0DC4-42DD-AAF8-D95EFF7A112F}"/>
+    <workbookView xWindow="1080" yWindow="708" windowWidth="21600" windowHeight="11232" xr2:uid="{E067A1E6-0DC4-42DD-AAF8-D95EFF7A112F}"/>
   </bookViews>
   <sheets>
     <sheet name="Work_Log" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="155">
   <si>
     <t>January</t>
   </si>
@@ -919,6 +919,18 @@
   </si>
   <si>
     <t>THE ADJUSTED PLAN AT PROGRESS REPORT 2</t>
+  </si>
+  <si>
+    <t>- Researched another dataset</t>
+  </si>
+  <si>
+    <t>25. Design Gurus, What is the difference between a table and a schema?</t>
+  </si>
+  <si>
+    <t>https://www.designgurus.io/answers/detail/what-is-the-difference-between-a-table-and-a-schema</t>
+  </si>
+  <si>
+    <t>- Modified database based on the new dataset</t>
   </si>
 </sst>
 </file>
@@ -1060,7 +1072,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="38">
+  <borders count="39">
     <border>
       <left/>
       <right/>
@@ -1515,12 +1527,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1719,6 +1742,12 @@
     <xf numFmtId="14" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1728,11 +1757,8 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="38" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -4572,24 +4598,34 @@
       </c>
     </row>
     <row r="120" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B120" s="56"/>
-      <c r="C120" s="56"/>
-      <c r="D120" s="51"/>
+      <c r="B120" s="67">
+        <v>411326</v>
+      </c>
+      <c r="C120" s="70">
+        <v>5</v>
+      </c>
+      <c r="D120" s="65" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="121" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B121" s="56"/>
-      <c r="C121" s="56"/>
-      <c r="D121" s="51"/>
-    </row>
-    <row r="122" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B122" s="32"/>
-      <c r="C122" s="32"/>
-      <c r="D122" s="33"/>
+      <c r="B121" s="68"/>
+      <c r="C121" s="71"/>
+      <c r="D121" s="55" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="122" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B122" s="69"/>
+      <c r="C122" s="72"/>
+      <c r="D122" s="89" t="s">
+        <v>154</v>
+      </c>
     </row>
     <row r="123" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B123" s="32"/>
-      <c r="C123" s="32"/>
-      <c r="D123" s="33"/>
+      <c r="B123" s="56"/>
+      <c r="C123" s="56"/>
+      <c r="D123" s="51"/>
     </row>
     <row r="124" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B124" s="56"/>
@@ -4682,7 +4718,9 @@
       <c r="D141" s="33"/>
     </row>
   </sheetData>
-  <mergeCells count="46">
+  <mergeCells count="48">
+    <mergeCell ref="B120:B122"/>
+    <mergeCell ref="C120:C122"/>
     <mergeCell ref="B112:B115"/>
     <mergeCell ref="C112:C115"/>
     <mergeCell ref="B116:B119"/>
@@ -4757,36 +4795,36 @@
       </c>
     </row>
     <row r="3" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D3" s="87" t="s">
+      <c r="D3" s="84" t="s">
         <v>8</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F3" s="84" t="s">
+      <c r="F3" s="86" t="s">
         <v>1</v>
       </c>
-      <c r="G3" s="85"/>
-      <c r="H3" s="85"/>
-      <c r="I3" s="86"/>
-      <c r="J3" s="84" t="s">
+      <c r="G3" s="87"/>
+      <c r="H3" s="87"/>
+      <c r="I3" s="88"/>
+      <c r="J3" s="86" t="s">
         <v>2</v>
       </c>
-      <c r="K3" s="85"/>
-      <c r="L3" s="85"/>
-      <c r="M3" s="86"/>
-      <c r="N3" s="84" t="s">
+      <c r="K3" s="87"/>
+      <c r="L3" s="87"/>
+      <c r="M3" s="88"/>
+      <c r="N3" s="86" t="s">
         <v>3</v>
       </c>
-      <c r="O3" s="85"/>
-      <c r="P3" s="85"/>
-      <c r="Q3" s="86"/>
+      <c r="O3" s="87"/>
+      <c r="P3" s="87"/>
+      <c r="Q3" s="88"/>
       <c r="R3" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="4:18" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D4" s="88"/>
+      <c r="D4" s="85"/>
       <c r="E4" s="4" t="s">
         <v>4</v>
       </c>
@@ -4957,36 +4995,36 @@
       </c>
     </row>
     <row r="15" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D15" s="87" t="s">
+      <c r="D15" s="84" t="s">
         <v>8</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F15" s="84" t="s">
+      <c r="F15" s="86" t="s">
         <v>1</v>
       </c>
-      <c r="G15" s="85"/>
-      <c r="H15" s="85"/>
-      <c r="I15" s="86"/>
-      <c r="J15" s="84" t="s">
+      <c r="G15" s="87"/>
+      <c r="H15" s="87"/>
+      <c r="I15" s="88"/>
+      <c r="J15" s="86" t="s">
         <v>2</v>
       </c>
-      <c r="K15" s="85"/>
-      <c r="L15" s="85"/>
-      <c r="M15" s="86"/>
-      <c r="N15" s="84" t="s">
+      <c r="K15" s="87"/>
+      <c r="L15" s="87"/>
+      <c r="M15" s="88"/>
+      <c r="N15" s="86" t="s">
         <v>3</v>
       </c>
-      <c r="O15" s="85"/>
-      <c r="P15" s="85"/>
-      <c r="Q15" s="86"/>
+      <c r="O15" s="87"/>
+      <c r="P15" s="87"/>
+      <c r="Q15" s="88"/>
       <c r="R15" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="16" spans="4:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D16" s="88"/>
+      <c r="D16" s="85"/>
       <c r="E16" s="4" t="s">
         <v>4</v>
       </c>
@@ -5171,36 +5209,36 @@
       <c r="R26" s="53"/>
     </row>
     <row r="27" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D27" s="87" t="s">
+      <c r="D27" s="84" t="s">
         <v>8</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F27" s="84" t="s">
+      <c r="F27" s="86" t="s">
         <v>1</v>
       </c>
-      <c r="G27" s="85"/>
-      <c r="H27" s="85"/>
-      <c r="I27" s="86"/>
-      <c r="J27" s="84" t="s">
+      <c r="G27" s="87"/>
+      <c r="H27" s="87"/>
+      <c r="I27" s="88"/>
+      <c r="J27" s="86" t="s">
         <v>2</v>
       </c>
-      <c r="K27" s="85"/>
-      <c r="L27" s="85"/>
-      <c r="M27" s="86"/>
-      <c r="N27" s="84" t="s">
+      <c r="K27" s="87"/>
+      <c r="L27" s="87"/>
+      <c r="M27" s="88"/>
+      <c r="N27" s="86" t="s">
         <v>3</v>
       </c>
-      <c r="O27" s="85"/>
-      <c r="P27" s="85"/>
-      <c r="Q27" s="86"/>
+      <c r="O27" s="87"/>
+      <c r="P27" s="87"/>
+      <c r="Q27" s="88"/>
       <c r="R27" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="28" spans="4:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D28" s="88"/>
+      <c r="D28" s="85"/>
       <c r="E28" s="4" t="s">
         <v>4</v>
       </c>
@@ -5392,7 +5430,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="B2:B49"/>
+  <dimension ref="B2:B51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="245.33203125" customWidth="1"/>
@@ -5636,6 +5674,16 @@
     <row r="49" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B49" s="64" t="s">
         <v>145</v>
+      </c>
+    </row>
+    <row r="50" spans="2:2" ht="15" x14ac:dyDescent="0.3">
+      <c r="B50" s="62" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="51" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B51" s="64" t="s">
+        <v>153</v>
       </c>
     </row>
   </sheetData>
@@ -5649,6 +5697,7 @@
     <hyperlink ref="B43" r:id="rId7" xr:uid="{4EFC952B-9A09-44AD-AF56-146B4F568623}"/>
     <hyperlink ref="B47" r:id="rId8" xr:uid="{BFE14320-69A1-490D-AB67-F9FA78E446C6}"/>
     <hyperlink ref="B49" r:id="rId9" xr:uid="{7818186A-BA4A-4BB4-91D9-A4C948B644CE}"/>
+    <hyperlink ref="B51" r:id="rId10" xr:uid="{DCC352E9-F585-47DE-BCF7-0C1F3F51E01B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
finalized KPI metric, created SQL queries
</commit_message>
<xml_diff>
--- a/DocumentsAndReports/0. WorkLog_Charts.xlsx
+++ b/DocumentsAndReports/0. WorkLog_Charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qhung\Videos\CSIS4495 - Applied Research  Project\W26_4495_S2_HughT\DocumentsAndReports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF6898F5-01EE-4F15-9597-91B58E6B8A33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{993C92A9-B969-4B34-9BFF-CBE6F2F8407F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="708" windowWidth="21600" windowHeight="11232" xr2:uid="{E067A1E6-0DC4-42DD-AAF8-D95EFF7A112F}"/>
+    <workbookView xWindow="0" yWindow="720" windowWidth="21600" windowHeight="11232" xr2:uid="{E067A1E6-0DC4-42DD-AAF8-D95EFF7A112F}"/>
   </bookViews>
   <sheets>
     <sheet name="Work_Log" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="161">
   <si>
     <t>January</t>
   </si>
@@ -931,6 +931,24 @@
   </si>
   <si>
     <t>- Modified database based on the new dataset</t>
+  </si>
+  <si>
+    <t>26. Star Jacobs, What is Monthly Recurring Revenue (MRR) and How can it help you understand business health? (May 20, 2024)</t>
+  </si>
+  <si>
+    <t>https://www.salesforce.com/blog/monthly-recurring-revenue/#h-what-is-monthly-recurring-revenue-mrr</t>
+  </si>
+  <si>
+    <t>- Finalized KPI metrics to be used for small business</t>
+  </si>
+  <si>
+    <t>“give an example of monthly recuring revenue”</t>
+  </si>
+  <si>
+    <t>"so the MRR is suitable for SaaS, how's about small business like a grocery store?"</t>
+  </si>
+  <si>
+    <t>- Created SQL queries for the KPI metrics</t>
   </si>
 </sst>
 </file>
@@ -1543,7 +1561,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1691,6 +1709,12 @@
       <alignment horizontal="justify" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="38" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -1756,9 +1780,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="38" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3660,7 +3681,7 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="B1:D141"/>
+  <dimension ref="B1:D140"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="2"/>
@@ -3683,10 +3704,10 @@
       </c>
     </row>
     <row r="3" spans="2:4" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="74">
+      <c r="B3" s="76">
         <v>45683</v>
       </c>
-      <c r="C3" s="73">
+      <c r="C3" s="75">
         <v>2</v>
       </c>
       <c r="D3" s="35" t="s">
@@ -3694,31 +3715,31 @@
       </c>
     </row>
     <row r="4" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="74"/>
-      <c r="C4" s="73"/>
+      <c r="B4" s="76"/>
+      <c r="C4" s="75"/>
       <c r="D4" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="74"/>
-      <c r="C5" s="73"/>
+      <c r="B5" s="76"/>
+      <c r="C5" s="75"/>
       <c r="D5" s="41" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="74"/>
-      <c r="C6" s="73"/>
+      <c r="B6" s="76"/>
+      <c r="C6" s="75"/>
       <c r="D6" s="42" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="7" spans="2:4" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="74">
+      <c r="B7" s="76">
         <v>45684</v>
       </c>
-      <c r="C7" s="73">
+      <c r="C7" s="75">
         <v>1.5</v>
       </c>
       <c r="D7" s="36" t="s">
@@ -3726,31 +3747,31 @@
       </c>
     </row>
     <row r="8" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="74"/>
-      <c r="C8" s="73"/>
+      <c r="B8" s="76"/>
+      <c r="C8" s="75"/>
       <c r="D8" s="37" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="9" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="74"/>
-      <c r="C9" s="73"/>
+      <c r="B9" s="76"/>
+      <c r="C9" s="75"/>
       <c r="D9" s="43" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="10" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="74"/>
-      <c r="C10" s="73"/>
+      <c r="B10" s="76"/>
+      <c r="C10" s="75"/>
       <c r="D10" s="44" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="74">
+      <c r="B11" s="76">
         <v>45686</v>
       </c>
-      <c r="C11" s="73">
+      <c r="C11" s="75">
         <v>3</v>
       </c>
       <c r="D11" s="35" t="s">
@@ -3758,38 +3779,38 @@
       </c>
     </row>
     <row r="12" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="74"/>
-      <c r="C12" s="73"/>
+      <c r="B12" s="76"/>
+      <c r="C12" s="75"/>
       <c r="D12" s="35" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="74"/>
-      <c r="C13" s="73"/>
+      <c r="B13" s="76"/>
+      <c r="C13" s="75"/>
       <c r="D13" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="74"/>
-      <c r="C14" s="73"/>
+      <c r="B14" s="76"/>
+      <c r="C14" s="75"/>
       <c r="D14" s="45" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="74"/>
-      <c r="C15" s="73"/>
+      <c r="B15" s="76"/>
+      <c r="C15" s="75"/>
       <c r="D15" s="42" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="74">
+      <c r="B16" s="76">
         <v>46053</v>
       </c>
-      <c r="C16" s="73">
+      <c r="C16" s="75">
         <v>4</v>
       </c>
       <c r="D16" s="38" t="s">
@@ -3797,80 +3818,80 @@
       </c>
     </row>
     <row r="17" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="74"/>
-      <c r="C17" s="73"/>
+      <c r="B17" s="76"/>
+      <c r="C17" s="75"/>
       <c r="D17" s="35" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="74"/>
-      <c r="C18" s="73"/>
+      <c r="B18" s="76"/>
+      <c r="C18" s="75"/>
       <c r="D18" s="35" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="19" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="74"/>
-      <c r="C19" s="73"/>
+      <c r="B19" s="76"/>
+      <c r="C19" s="75"/>
       <c r="D19" s="35" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="20" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="74"/>
-      <c r="C20" s="73"/>
+      <c r="B20" s="76"/>
+      <c r="C20" s="75"/>
       <c r="D20" s="35" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="21" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="74"/>
-      <c r="C21" s="73"/>
+      <c r="B21" s="76"/>
+      <c r="C21" s="75"/>
       <c r="D21" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="74"/>
-      <c r="C22" s="73"/>
+      <c r="B22" s="76"/>
+      <c r="C22" s="75"/>
       <c r="D22" s="45" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="23" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="74"/>
-      <c r="C23" s="73"/>
+      <c r="B23" s="76"/>
+      <c r="C23" s="75"/>
       <c r="D23" s="41" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="24" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="74"/>
-      <c r="C24" s="73"/>
+      <c r="B24" s="76"/>
+      <c r="C24" s="75"/>
       <c r="D24" s="41" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="25" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="74"/>
-      <c r="C25" s="73"/>
+      <c r="B25" s="76"/>
+      <c r="C25" s="75"/>
       <c r="D25" s="41" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="26" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="74"/>
-      <c r="C26" s="73"/>
+      <c r="B26" s="76"/>
+      <c r="C26" s="75"/>
       <c r="D26" s="46" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="27" spans="2:4" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="74">
+      <c r="B27" s="76">
         <v>46054</v>
       </c>
-      <c r="C27" s="73">
+      <c r="C27" s="75">
         <v>1</v>
       </c>
       <c r="D27" s="35" t="s">
@@ -3878,31 +3899,31 @@
       </c>
     </row>
     <row r="28" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="74"/>
-      <c r="C28" s="73"/>
+      <c r="B28" s="76"/>
+      <c r="C28" s="75"/>
       <c r="D28" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="29" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="74"/>
-      <c r="C29" s="73"/>
+      <c r="B29" s="76"/>
+      <c r="C29" s="75"/>
       <c r="D29" s="41" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="30" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="74"/>
-      <c r="C30" s="73"/>
+      <c r="B30" s="76"/>
+      <c r="C30" s="75"/>
       <c r="D30" s="42" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="31" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B31" s="74">
+      <c r="B31" s="76">
         <v>46055</v>
       </c>
-      <c r="C31" s="73">
+      <c r="C31" s="75">
         <v>4</v>
       </c>
       <c r="D31" s="39" t="s">
@@ -3910,45 +3931,45 @@
       </c>
     </row>
     <row r="32" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B32" s="74"/>
-      <c r="C32" s="73"/>
+      <c r="B32" s="76"/>
+      <c r="C32" s="75"/>
       <c r="D32" s="40" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="33" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="74"/>
-      <c r="C33" s="73"/>
+      <c r="B33" s="76"/>
+      <c r="C33" s="75"/>
       <c r="D33" s="40" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="34" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B34" s="74"/>
-      <c r="C34" s="73"/>
+      <c r="B34" s="76"/>
+      <c r="C34" s="75"/>
       <c r="D34" s="40" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="35" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B35" s="74"/>
-      <c r="C35" s="73"/>
+      <c r="B35" s="76"/>
+      <c r="C35" s="75"/>
       <c r="D35" s="47" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="36" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B36" s="74"/>
-      <c r="C36" s="73"/>
+      <c r="B36" s="76"/>
+      <c r="C36" s="75"/>
       <c r="D36" s="48" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="37" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="74">
+      <c r="B37" s="76">
         <v>46056</v>
       </c>
-      <c r="C37" s="73">
+      <c r="C37" s="75">
         <v>3</v>
       </c>
       <c r="D37" s="35" t="s">
@@ -3956,38 +3977,38 @@
       </c>
     </row>
     <row r="38" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B38" s="74"/>
-      <c r="C38" s="73"/>
+      <c r="B38" s="76"/>
+      <c r="C38" s="75"/>
       <c r="D38" s="35" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="39" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B39" s="74"/>
-      <c r="C39" s="73"/>
+      <c r="B39" s="76"/>
+      <c r="C39" s="75"/>
       <c r="D39" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="40" spans="2:4" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B40" s="74"/>
-      <c r="C40" s="73"/>
+      <c r="B40" s="76"/>
+      <c r="C40" s="75"/>
       <c r="D40" s="41" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="41" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B41" s="74"/>
-      <c r="C41" s="73"/>
+      <c r="B41" s="76"/>
+      <c r="C41" s="75"/>
       <c r="D41" s="42" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="42" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B42" s="74">
+      <c r="B42" s="76">
         <v>46057</v>
       </c>
-      <c r="C42" s="73">
+      <c r="C42" s="75">
         <v>4</v>
       </c>
       <c r="D42" s="38" t="s">
@@ -3995,24 +4016,24 @@
       </c>
     </row>
     <row r="43" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B43" s="74"/>
-      <c r="C43" s="73"/>
+      <c r="B43" s="76"/>
+      <c r="C43" s="75"/>
       <c r="D43" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="44" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B44" s="74"/>
-      <c r="C44" s="73"/>
+      <c r="B44" s="76"/>
+      <c r="C44" s="75"/>
       <c r="D44" s="42" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="45" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B45" s="75">
+      <c r="B45" s="77">
         <v>46059</v>
       </c>
-      <c r="C45" s="78">
+      <c r="C45" s="80">
         <v>2</v>
       </c>
       <c r="D45" s="50" t="s">
@@ -4020,38 +4041,38 @@
       </c>
     </row>
     <row r="46" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B46" s="76"/>
-      <c r="C46" s="79"/>
+      <c r="B46" s="78"/>
+      <c r="C46" s="81"/>
       <c r="D46" s="49" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="47" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B47" s="76"/>
-      <c r="C47" s="79"/>
+      <c r="B47" s="78"/>
+      <c r="C47" s="81"/>
       <c r="D47" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="48" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B48" s="76"/>
-      <c r="C48" s="79"/>
+      <c r="B48" s="78"/>
+      <c r="C48" s="81"/>
       <c r="D48" s="42" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="49" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B49" s="77"/>
-      <c r="C49" s="80"/>
+      <c r="B49" s="79"/>
+      <c r="C49" s="82"/>
       <c r="D49" s="46" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="50" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B50" s="75">
+      <c r="B50" s="77">
         <v>46061</v>
       </c>
-      <c r="C50" s="78">
+      <c r="C50" s="80">
         <v>1.5</v>
       </c>
       <c r="D50" s="50" t="s">
@@ -4059,38 +4080,38 @@
       </c>
     </row>
     <row r="51" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B51" s="76"/>
-      <c r="C51" s="79"/>
+      <c r="B51" s="78"/>
+      <c r="C51" s="81"/>
       <c r="D51" s="35" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="52" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B52" s="76"/>
-      <c r="C52" s="79"/>
+      <c r="B52" s="78"/>
+      <c r="C52" s="81"/>
       <c r="D52" s="42" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="53" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B53" s="76"/>
-      <c r="C53" s="79"/>
+      <c r="B53" s="78"/>
+      <c r="C53" s="81"/>
       <c r="D53" s="42" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="54" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B54" s="77"/>
-      <c r="C54" s="80"/>
+      <c r="B54" s="79"/>
+      <c r="C54" s="82"/>
       <c r="D54" s="46" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="55" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="75">
+      <c r="B55" s="77">
         <v>46062</v>
       </c>
-      <c r="C55" s="78">
+      <c r="C55" s="80">
         <v>2</v>
       </c>
       <c r="D55" s="54" t="s">
@@ -4098,31 +4119,31 @@
       </c>
     </row>
     <row r="56" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B56" s="76"/>
-      <c r="C56" s="79"/>
+      <c r="B56" s="78"/>
+      <c r="C56" s="81"/>
       <c r="D56" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="57" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B57" s="76"/>
-      <c r="C57" s="79"/>
+      <c r="B57" s="78"/>
+      <c r="C57" s="81"/>
       <c r="D57" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="58" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B58" s="77"/>
-      <c r="C58" s="80"/>
+      <c r="B58" s="79"/>
+      <c r="C58" s="82"/>
       <c r="D58" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="59" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="75">
+      <c r="B59" s="77">
         <v>46063</v>
       </c>
-      <c r="C59" s="78">
+      <c r="C59" s="80">
         <v>3</v>
       </c>
       <c r="D59" s="54" t="s">
@@ -4130,38 +4151,38 @@
       </c>
     </row>
     <row r="60" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B60" s="76"/>
-      <c r="C60" s="79"/>
+      <c r="B60" s="78"/>
+      <c r="C60" s="81"/>
       <c r="D60" s="55" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="61" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B61" s="76"/>
-      <c r="C61" s="79"/>
+      <c r="B61" s="78"/>
+      <c r="C61" s="81"/>
       <c r="D61" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="62" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B62" s="76"/>
-      <c r="C62" s="79"/>
+      <c r="B62" s="78"/>
+      <c r="C62" s="81"/>
       <c r="D62" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="63" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B63" s="77"/>
-      <c r="C63" s="80"/>
+      <c r="B63" s="79"/>
+      <c r="C63" s="82"/>
       <c r="D63" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="64" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B64" s="75">
+      <c r="B64" s="77">
         <v>46064</v>
       </c>
-      <c r="C64" s="78">
+      <c r="C64" s="80">
         <v>3</v>
       </c>
       <c r="D64" s="54" t="s">
@@ -4169,38 +4190,38 @@
       </c>
     </row>
     <row r="65" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B65" s="76"/>
-      <c r="C65" s="79"/>
+      <c r="B65" s="78"/>
+      <c r="C65" s="81"/>
       <c r="D65" s="55" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="66" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B66" s="76"/>
-      <c r="C66" s="79"/>
+      <c r="B66" s="78"/>
+      <c r="C66" s="81"/>
       <c r="D66" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="67" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B67" s="76"/>
-      <c r="C67" s="79"/>
+      <c r="B67" s="78"/>
+      <c r="C67" s="81"/>
       <c r="D67" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="68" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B68" s="77"/>
-      <c r="C68" s="80"/>
+      <c r="B68" s="79"/>
+      <c r="C68" s="82"/>
       <c r="D68" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="69" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B69" s="81">
+      <c r="B69" s="83">
         <v>46066</v>
       </c>
-      <c r="C69" s="78">
+      <c r="C69" s="80">
         <v>2</v>
       </c>
       <c r="D69" s="54" t="s">
@@ -4208,45 +4229,45 @@
       </c>
     </row>
     <row r="70" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B70" s="82"/>
-      <c r="C70" s="79"/>
+      <c r="B70" s="84"/>
+      <c r="C70" s="81"/>
       <c r="D70" s="55" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="71" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B71" s="82"/>
-      <c r="C71" s="79"/>
+      <c r="B71" s="84"/>
+      <c r="C71" s="81"/>
       <c r="D71" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="72" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B72" s="82"/>
-      <c r="C72" s="79"/>
+      <c r="B72" s="84"/>
+      <c r="C72" s="81"/>
       <c r="D72" s="42" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="73" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B73" s="82"/>
-      <c r="C73" s="79"/>
+      <c r="B73" s="84"/>
+      <c r="C73" s="81"/>
       <c r="D73" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="74" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B74" s="83"/>
-      <c r="C74" s="80"/>
+      <c r="B74" s="85"/>
+      <c r="C74" s="82"/>
       <c r="D74" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="75" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B75" s="67">
+      <c r="B75" s="69">
         <v>46068</v>
       </c>
-      <c r="C75" s="70">
+      <c r="C75" s="72">
         <v>2.5</v>
       </c>
       <c r="D75" s="54" t="s">
@@ -4254,52 +4275,52 @@
       </c>
     </row>
     <row r="76" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B76" s="68"/>
-      <c r="C76" s="71"/>
+      <c r="B76" s="70"/>
+      <c r="C76" s="73"/>
       <c r="D76" s="55" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="77" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B77" s="68"/>
-      <c r="C77" s="71"/>
+      <c r="B77" s="70"/>
+      <c r="C77" s="73"/>
       <c r="D77" s="55" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="78" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B78" s="68"/>
-      <c r="C78" s="71"/>
+      <c r="B78" s="70"/>
+      <c r="C78" s="73"/>
       <c r="D78" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="79" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B79" s="68"/>
-      <c r="C79" s="71"/>
+      <c r="B79" s="70"/>
+      <c r="C79" s="73"/>
       <c r="D79" s="42" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="80" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B80" s="68"/>
-      <c r="C80" s="71"/>
+      <c r="B80" s="70"/>
+      <c r="C80" s="73"/>
       <c r="D80" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="81" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B81" s="69"/>
-      <c r="C81" s="72"/>
+      <c r="B81" s="71"/>
+      <c r="C81" s="74"/>
       <c r="D81" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="82" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B82" s="67">
+      <c r="B82" s="69">
         <v>46070</v>
       </c>
-      <c r="C82" s="70">
+      <c r="C82" s="72">
         <v>3</v>
       </c>
       <c r="D82" s="54" t="s">
@@ -4307,52 +4328,52 @@
       </c>
     </row>
     <row r="83" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B83" s="68"/>
-      <c r="C83" s="71"/>
+      <c r="B83" s="70"/>
+      <c r="C83" s="73"/>
       <c r="D83" s="55" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="84" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B84" s="68"/>
-      <c r="C84" s="71"/>
+      <c r="B84" s="70"/>
+      <c r="C84" s="73"/>
       <c r="D84" s="55" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="85" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B85" s="68"/>
-      <c r="C85" s="71"/>
+      <c r="B85" s="70"/>
+      <c r="C85" s="73"/>
       <c r="D85" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="86" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B86" s="68"/>
-      <c r="C86" s="71"/>
+      <c r="B86" s="70"/>
+      <c r="C86" s="73"/>
       <c r="D86" s="42" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="87" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B87" s="68"/>
-      <c r="C87" s="71"/>
+      <c r="B87" s="70"/>
+      <c r="C87" s="73"/>
       <c r="D87" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="88" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B88" s="69"/>
-      <c r="C88" s="72"/>
+      <c r="B88" s="71"/>
+      <c r="C88" s="74"/>
       <c r="D88" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="89" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B89" s="67">
+      <c r="B89" s="69">
         <v>46071</v>
       </c>
-      <c r="C89" s="70">
+      <c r="C89" s="72">
         <v>2</v>
       </c>
       <c r="D89" s="54" t="s">
@@ -4360,38 +4381,38 @@
       </c>
     </row>
     <row r="90" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B90" s="68"/>
-      <c r="C90" s="71"/>
+      <c r="B90" s="70"/>
+      <c r="C90" s="73"/>
       <c r="D90" s="55" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="91" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B91" s="68"/>
-      <c r="C91" s="71"/>
+      <c r="B91" s="70"/>
+      <c r="C91" s="73"/>
       <c r="D91" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="92" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B92" s="68"/>
-      <c r="C92" s="71"/>
+      <c r="B92" s="70"/>
+      <c r="C92" s="73"/>
       <c r="D92" s="42" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="93" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B93" s="69"/>
-      <c r="C93" s="72"/>
+      <c r="B93" s="71"/>
+      <c r="C93" s="74"/>
       <c r="D93" s="46" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="94" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B94" s="67">
+      <c r="B94" s="69">
         <v>46074</v>
       </c>
-      <c r="C94" s="70">
+      <c r="C94" s="72">
         <v>3</v>
       </c>
       <c r="D94" s="57" t="s">
@@ -4399,24 +4420,24 @@
       </c>
     </row>
     <row r="95" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B95" s="68"/>
-      <c r="C95" s="71"/>
+      <c r="B95" s="70"/>
+      <c r="C95" s="73"/>
       <c r="D95" s="58" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="96" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B96" s="69"/>
-      <c r="C96" s="72"/>
+      <c r="B96" s="71"/>
+      <c r="C96" s="74"/>
       <c r="D96" s="46" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="97" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B97" s="67">
+      <c r="B97" s="69">
         <v>46075</v>
       </c>
-      <c r="C97" s="70">
+      <c r="C97" s="72">
         <v>3</v>
       </c>
       <c r="D97" s="54" t="s">
@@ -4424,22 +4445,22 @@
       </c>
     </row>
     <row r="98" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B98" s="68"/>
-      <c r="C98" s="71"/>
+      <c r="B98" s="70"/>
+      <c r="C98" s="73"/>
       <c r="D98" s="55" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="99" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B99" s="68"/>
-      <c r="C99" s="71"/>
+      <c r="B99" s="70"/>
+      <c r="C99" s="73"/>
       <c r="D99" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="100" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B100" s="69"/>
-      <c r="C100" s="72"/>
+      <c r="B100" s="71"/>
+      <c r="C100" s="74"/>
       <c r="D100" s="46" t="s">
         <v>23</v>
       </c>
@@ -4456,10 +4477,10 @@
       </c>
     </row>
     <row r="102" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B102" s="67">
+      <c r="B102" s="69">
         <v>46077</v>
       </c>
-      <c r="C102" s="70">
+      <c r="C102" s="72">
         <v>2</v>
       </c>
       <c r="D102" s="54" t="s">
@@ -4467,38 +4488,38 @@
       </c>
     </row>
     <row r="103" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B103" s="68"/>
-      <c r="C103" s="71"/>
+      <c r="B103" s="70"/>
+      <c r="C103" s="73"/>
       <c r="D103" s="55" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="104" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B104" s="68"/>
-      <c r="C104" s="71"/>
+      <c r="B104" s="70"/>
+      <c r="C104" s="73"/>
       <c r="D104" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="105" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B105" s="68"/>
-      <c r="C105" s="71"/>
+      <c r="B105" s="70"/>
+      <c r="C105" s="73"/>
       <c r="D105" s="42" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="106" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B106" s="69"/>
-      <c r="C106" s="72"/>
+      <c r="B106" s="71"/>
+      <c r="C106" s="74"/>
       <c r="D106" s="46" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="107" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B107" s="67">
+      <c r="B107" s="69">
         <v>46078</v>
       </c>
-      <c r="C107" s="70">
+      <c r="C107" s="72">
         <v>1</v>
       </c>
       <c r="D107" s="65" t="s">
@@ -4506,38 +4527,38 @@
       </c>
     </row>
     <row r="108" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B108" s="68"/>
-      <c r="C108" s="71"/>
+      <c r="B108" s="70"/>
+      <c r="C108" s="73"/>
       <c r="D108" s="55" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="109" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B109" s="68"/>
-      <c r="C109" s="71"/>
+      <c r="B109" s="70"/>
+      <c r="C109" s="73"/>
       <c r="D109" s="42" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="110" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B110" s="68"/>
-      <c r="C110" s="71"/>
+      <c r="B110" s="70"/>
+      <c r="C110" s="73"/>
       <c r="D110" s="42" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="111" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B111" s="69"/>
-      <c r="C111" s="72"/>
+      <c r="B111" s="71"/>
+      <c r="C111" s="74"/>
       <c r="D111" s="66" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="112" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B112" s="67">
+      <c r="B112" s="69">
         <v>46079</v>
       </c>
-      <c r="C112" s="70">
+      <c r="C112" s="72">
         <v>2</v>
       </c>
       <c r="D112" s="65" t="s">
@@ -4545,31 +4566,31 @@
       </c>
     </row>
     <row r="113" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B113" s="68"/>
-      <c r="C113" s="71"/>
+      <c r="B113" s="70"/>
+      <c r="C113" s="73"/>
       <c r="D113" s="55" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="114" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B114" s="68"/>
-      <c r="C114" s="71"/>
+      <c r="B114" s="70"/>
+      <c r="C114" s="73"/>
       <c r="D114" s="42" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="115" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B115" s="69"/>
-      <c r="C115" s="72"/>
+      <c r="B115" s="71"/>
+      <c r="C115" s="74"/>
       <c r="D115" s="46" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="116" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B116" s="67">
+      <c r="B116" s="69">
         <v>46083</v>
       </c>
-      <c r="C116" s="70">
+      <c r="C116" s="72">
         <v>3</v>
       </c>
       <c r="D116" s="65" t="s">
@@ -4577,31 +4598,31 @@
       </c>
     </row>
     <row r="117" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B117" s="68"/>
-      <c r="C117" s="71"/>
+      <c r="B117" s="70"/>
+      <c r="C117" s="73"/>
       <c r="D117" s="55" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="118" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B118" s="68"/>
-      <c r="C118" s="71"/>
+      <c r="B118" s="70"/>
+      <c r="C118" s="73"/>
       <c r="D118" s="55" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="119" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B119" s="69"/>
-      <c r="C119" s="72"/>
+      <c r="B119" s="71"/>
+      <c r="C119" s="74"/>
       <c r="D119" s="46" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="120" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B120" s="67">
+      <c r="B120" s="69">
         <v>411326</v>
       </c>
-      <c r="C120" s="70">
+      <c r="C120" s="72">
         <v>5</v>
       </c>
       <c r="D120" s="65" t="s">
@@ -4609,43 +4630,57 @@
       </c>
     </row>
     <row r="121" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B121" s="68"/>
-      <c r="C121" s="71"/>
+      <c r="B121" s="70"/>
+      <c r="C121" s="73"/>
       <c r="D121" s="55" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="122" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B122" s="69"/>
-      <c r="C122" s="72"/>
-      <c r="D122" s="89" t="s">
+      <c r="B122" s="71"/>
+      <c r="C122" s="74"/>
+      <c r="D122" s="67" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="123" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B123" s="56"/>
-      <c r="C123" s="56"/>
-      <c r="D123" s="51"/>
+      <c r="B123" s="68">
+        <v>46085</v>
+      </c>
+      <c r="C123" s="56">
+        <v>4</v>
+      </c>
+      <c r="D123" s="65" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="124" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B124" s="56"/>
       <c r="C124" s="56"/>
-      <c r="D124" s="51"/>
+      <c r="D124" s="55" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="125" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B125" s="32"/>
       <c r="C125" s="32"/>
-      <c r="D125" s="33"/>
-    </row>
-    <row r="126" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B126" s="32"/>
-      <c r="C126" s="32"/>
-      <c r="D126" s="33"/>
-    </row>
-    <row r="127" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B127" s="56"/>
-      <c r="C127" s="56"/>
-      <c r="D127" s="51"/>
+      <c r="D125" s="55" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="126" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B126" s="56"/>
+      <c r="C126" s="56"/>
+      <c r="D126" s="42" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="127" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B127" s="32"/>
+      <c r="C127" s="32"/>
+      <c r="D127" s="42" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="128" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B128" s="32"/>
@@ -4653,14 +4688,14 @@
       <c r="D128" s="33"/>
     </row>
     <row r="129" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B129" s="32"/>
-      <c r="C129" s="32"/>
-      <c r="D129" s="33"/>
+      <c r="B129" s="56"/>
+      <c r="C129" s="56"/>
+      <c r="D129" s="51"/>
     </row>
     <row r="130" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B130" s="56"/>
-      <c r="C130" s="56"/>
-      <c r="D130" s="51"/>
+      <c r="B130" s="32"/>
+      <c r="C130" s="32"/>
+      <c r="D130" s="33"/>
     </row>
     <row r="131" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B131" s="32"/>
@@ -4668,14 +4703,14 @@
       <c r="D131" s="33"/>
     </row>
     <row r="132" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B132" s="32"/>
-      <c r="C132" s="32"/>
-      <c r="D132" s="33"/>
+      <c r="B132" s="56"/>
+      <c r="C132" s="56"/>
+      <c r="D132" s="51"/>
     </row>
     <row r="133" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B133" s="56"/>
-      <c r="C133" s="56"/>
-      <c r="D133" s="51"/>
+      <c r="B133" s="32"/>
+      <c r="C133" s="32"/>
+      <c r="D133" s="33"/>
     </row>
     <row r="134" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B134" s="32"/>
@@ -4683,14 +4718,14 @@
       <c r="D134" s="33"/>
     </row>
     <row r="135" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B135" s="32"/>
-      <c r="C135" s="32"/>
-      <c r="D135" s="33"/>
+      <c r="B135" s="56"/>
+      <c r="C135" s="56"/>
+      <c r="D135" s="51"/>
     </row>
     <row r="136" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B136" s="56"/>
-      <c r="C136" s="56"/>
-      <c r="D136" s="51"/>
+      <c r="B136" s="32"/>
+      <c r="C136" s="32"/>
+      <c r="D136" s="33"/>
     </row>
     <row r="137" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B137" s="32"/>
@@ -4698,24 +4733,19 @@
       <c r="D137" s="33"/>
     </row>
     <row r="138" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B138" s="32"/>
-      <c r="C138" s="32"/>
-      <c r="D138" s="33"/>
+      <c r="B138" s="56"/>
+      <c r="C138" s="56"/>
+      <c r="D138" s="51"/>
     </row>
     <row r="139" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B139" s="56"/>
-      <c r="C139" s="56"/>
-      <c r="D139" s="51"/>
+      <c r="B139" s="32"/>
+      <c r="C139" s="32"/>
+      <c r="D139" s="33"/>
     </row>
     <row r="140" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B140" s="32"/>
       <c r="C140" s="32"/>
       <c r="D140" s="33"/>
-    </row>
-    <row r="141" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B141" s="32"/>
-      <c r="C141" s="32"/>
-      <c r="D141" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="48">
@@ -4795,36 +4825,36 @@
       </c>
     </row>
     <row r="3" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D3" s="84" t="s">
+      <c r="D3" s="86" t="s">
         <v>8</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F3" s="86" t="s">
+      <c r="F3" s="88" t="s">
         <v>1</v>
       </c>
-      <c r="G3" s="87"/>
-      <c r="H3" s="87"/>
-      <c r="I3" s="88"/>
-      <c r="J3" s="86" t="s">
+      <c r="G3" s="89"/>
+      <c r="H3" s="89"/>
+      <c r="I3" s="90"/>
+      <c r="J3" s="88" t="s">
         <v>2</v>
       </c>
-      <c r="K3" s="87"/>
-      <c r="L3" s="87"/>
-      <c r="M3" s="88"/>
-      <c r="N3" s="86" t="s">
+      <c r="K3" s="89"/>
+      <c r="L3" s="89"/>
+      <c r="M3" s="90"/>
+      <c r="N3" s="88" t="s">
         <v>3</v>
       </c>
-      <c r="O3" s="87"/>
-      <c r="P3" s="87"/>
-      <c r="Q3" s="88"/>
+      <c r="O3" s="89"/>
+      <c r="P3" s="89"/>
+      <c r="Q3" s="90"/>
       <c r="R3" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="4:18" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D4" s="85"/>
+      <c r="D4" s="87"/>
       <c r="E4" s="4" t="s">
         <v>4</v>
       </c>
@@ -4995,36 +5025,36 @@
       </c>
     </row>
     <row r="15" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D15" s="84" t="s">
+      <c r="D15" s="86" t="s">
         <v>8</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F15" s="86" t="s">
+      <c r="F15" s="88" t="s">
         <v>1</v>
       </c>
-      <c r="G15" s="87"/>
-      <c r="H15" s="87"/>
-      <c r="I15" s="88"/>
-      <c r="J15" s="86" t="s">
+      <c r="G15" s="89"/>
+      <c r="H15" s="89"/>
+      <c r="I15" s="90"/>
+      <c r="J15" s="88" t="s">
         <v>2</v>
       </c>
-      <c r="K15" s="87"/>
-      <c r="L15" s="87"/>
-      <c r="M15" s="88"/>
-      <c r="N15" s="86" t="s">
+      <c r="K15" s="89"/>
+      <c r="L15" s="89"/>
+      <c r="M15" s="90"/>
+      <c r="N15" s="88" t="s">
         <v>3</v>
       </c>
-      <c r="O15" s="87"/>
-      <c r="P15" s="87"/>
-      <c r="Q15" s="88"/>
+      <c r="O15" s="89"/>
+      <c r="P15" s="89"/>
+      <c r="Q15" s="90"/>
       <c r="R15" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="16" spans="4:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D16" s="85"/>
+      <c r="D16" s="87"/>
       <c r="E16" s="4" t="s">
         <v>4</v>
       </c>
@@ -5209,36 +5239,36 @@
       <c r="R26" s="53"/>
     </row>
     <row r="27" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D27" s="84" t="s">
+      <c r="D27" s="86" t="s">
         <v>8</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F27" s="86" t="s">
+      <c r="F27" s="88" t="s">
         <v>1</v>
       </c>
-      <c r="G27" s="87"/>
-      <c r="H27" s="87"/>
-      <c r="I27" s="88"/>
-      <c r="J27" s="86" t="s">
+      <c r="G27" s="89"/>
+      <c r="H27" s="89"/>
+      <c r="I27" s="90"/>
+      <c r="J27" s="88" t="s">
         <v>2</v>
       </c>
-      <c r="K27" s="87"/>
-      <c r="L27" s="87"/>
-      <c r="M27" s="88"/>
-      <c r="N27" s="86" t="s">
+      <c r="K27" s="89"/>
+      <c r="L27" s="89"/>
+      <c r="M27" s="90"/>
+      <c r="N27" s="88" t="s">
         <v>3</v>
       </c>
-      <c r="O27" s="87"/>
-      <c r="P27" s="87"/>
-      <c r="Q27" s="88"/>
+      <c r="O27" s="89"/>
+      <c r="P27" s="89"/>
+      <c r="Q27" s="90"/>
       <c r="R27" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="28" spans="4:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D28" s="85"/>
+      <c r="D28" s="87"/>
       <c r="E28" s="4" t="s">
         <v>4</v>
       </c>
@@ -5430,7 +5460,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="B2:B51"/>
+  <dimension ref="B2:B53"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="245.33203125" customWidth="1"/>
@@ -5684,6 +5714,16 @@
     <row r="51" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B51" s="64" t="s">
         <v>153</v>
+      </c>
+    </row>
+    <row r="52" spans="2:2" ht="15" x14ac:dyDescent="0.3">
+      <c r="B52" s="62" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="53" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B53" s="64" t="s">
+        <v>156</v>
       </c>
     </row>
   </sheetData>
@@ -5698,6 +5738,8 @@
     <hyperlink ref="B47" r:id="rId8" xr:uid="{BFE14320-69A1-490D-AB67-F9FA78E446C6}"/>
     <hyperlink ref="B49" r:id="rId9" xr:uid="{7818186A-BA4A-4BB4-91D9-A4C948B644CE}"/>
     <hyperlink ref="B51" r:id="rId10" xr:uid="{DCC352E9-F585-47DE-BCF7-0C1F3F51E01B}"/>
+    <hyperlink ref="B45" r:id="rId11" xr:uid="{500C1AC5-73B0-417C-9903-2460A3E5FD4B}"/>
+    <hyperlink ref="B53" r:id="rId12" location="h-what-is-monthly-recurring-revenue-mrr" xr:uid="{756E4B61-8845-414D-9B64-D39C0AD55437}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
debugged data loading code, and SQL queries
</commit_message>
<xml_diff>
--- a/DocumentsAndReports/0. WorkLog_Charts.xlsx
+++ b/DocumentsAndReports/0. WorkLog_Charts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qhung\Videos\CSIS4495 - Applied Research  Project\W26_4495_S2_HughT\DocumentsAndReports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{993C92A9-B969-4B34-9BFF-CBE6F2F8407F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E3B3EEF-7650-4D38-8461-8FBEFDFAB5D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="720" windowWidth="21600" windowHeight="11232" xr2:uid="{E067A1E6-0DC4-42DD-AAF8-D95EFF7A112F}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="175">
   <si>
     <t>January</t>
   </si>
@@ -949,6 +949,48 @@
   </si>
   <si>
     <t>- Created SQL queries for the KPI metrics</t>
+  </si>
+  <si>
+    <t>- Debugged data loading code</t>
+  </si>
+  <si>
+    <t>"what is this error "pyodbc.ProgrammingError: ('42000', '[42000] [Microsoft][ODBC Driver 17 for SQL Server][SQL Server]The incoming tabular data stream (TDS) remote procedure call (RPC) protocol stream is incorrect. Parameter 5 (""): The supplied value is not a valid instance of data type float. Check the source data for invalid values. An example of an invalid value is data of numeric type with scale greater than precision. (8023) (SQLExecDirectW)')"</t>
+  </si>
+  <si>
+    <t>"explain set() and raise in python"</t>
+  </si>
+  <si>
+    <t>"explain this error: pyodbc.ProgrammingError: ('42000', "[42000] [Microsoft][ODBC Driver 17 for SQL Server][SQL Server]String or binary data would be truncated in table 'IBP.rawT.customer_review', column 'ProductName'. Truncated value: 'Passion Rx enhances libido, erections, and orgasms/climaxes in men and women. Formulated by Ray Sahe'. (2628) (SQLExecDirectW); [42000] [Microsoft][ODBC Driver 17 for SQL Server][SQL Server]The statement has been terminated. (3621)")"</t>
+  </si>
+  <si>
+    <t>"i want to debug by insert row by row until it fails, write this function"</t>
+  </si>
+  <si>
+    <t>"i removed a number of columns in rawT.customer_review and it remains only 4 columns, but the error of parameter 5 keep displaying, could it be a connecting mechanism between odbc and sql?, I meant not by datatype?"</t>
+  </si>
+  <si>
+    <t>"KeyError: "['CustomerID', 'Country'] not in index" =&gt; i check on any issue when inserting the purchase file, and it showed KeyError(f"{not_found} not in index", however .csv and db dont have these columns, i dont know why these columns appearred here. Of note, althought these warning, but the data successfully inserted into the database =&gt; could it be any issue of temporary memory of local machine regarding other projects?"</t>
+  </si>
+  <si>
+    <t>"their is another column in .csv, which has datatype in both date and integer, when i checked its datatype in pandas then result is str. Of note, i did not load this column into database. So, might the problem come from this column?"</t>
+  </si>
+  <si>
+    <t>"860630400 is a value of date column in .csv, can it be converted to datetype? how?"</t>
+  </si>
+  <si>
+    <t>"is the inserted value too long? "pyodbc.ProgrammingError: ('42000', "[42000] [Microsoft][ODBC Driver 17 for SQL Server][SQL Server]String or binary data would be truncated in table 'IBP.rawT.customer_review', column 'ProductName'. Truncated value: 'Lord of the Rings - Deluxe Gift Pack - With 9 Figures and One Ring to Rule Them All (Includes Frodo,'. (2628) (SQLExecDirectW); [42000] [Microsoft][ODBC Driver 17 for SQL Server][SQL Server]The statement has been terminated. (3621)")"</t>
+  </si>
+  <si>
+    <t>"need to remove primary key, right? : pyodbc.IntegrityError: ('23000', "[23000] [Microsoft][ODBC Driver 17 for SQL Server][SQL Server]Violation of PRIMARY KEY constraint 'PK__customer__1788CCAC055B0016'. Cannot insert duplicate key in object 'rawT.customer_review'. The duplicate key value is (unknown). (2627) (SQLExecDirectW); [23000] [Microsoft][ODBC Driver 17 for SQL Server][SQL Server]The statement has been terminated. (3621)")"</t>
+  </si>
+  <si>
+    <t>"(batch_id,) is a tuple =&gt; why have to use the tuple here"</t>
+  </si>
+  <si>
+    <t>"review the whole code"</t>
+  </si>
+  <si>
+    <t>- Modified SQL queries in database</t>
   </si>
 </sst>
 </file>
@@ -1561,7 +1603,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1617,7 +1659,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1665,7 +1706,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="31" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="25" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -1733,39 +1773,39 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="15" fontId="7" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="15" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="15" fontId="7" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="15" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1780,6 +1820,27 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3681,7 +3742,7 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="B1:D140"/>
+  <dimension ref="B1:D174"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="2"/>
@@ -3693,1094 +3754,1266 @@
   <sheetData>
     <row r="1" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:4" s="31" customFormat="1" ht="22.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="34" t="s">
+      <c r="B2" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="34" t="s">
+      <c r="C2" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="34" t="s">
+      <c r="D2" s="33" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="3" spans="2:4" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="76">
+      <c r="B3" s="82">
         <v>45683</v>
       </c>
-      <c r="C3" s="75">
+      <c r="C3" s="83">
         <v>2</v>
       </c>
-      <c r="D3" s="35" t="s">
+      <c r="D3" s="34" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="4" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="76"/>
-      <c r="C4" s="75"/>
-      <c r="D4" s="35" t="s">
+      <c r="B4" s="82"/>
+      <c r="C4" s="83"/>
+      <c r="D4" s="34" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="76"/>
-      <c r="C5" s="75"/>
-      <c r="D5" s="41" t="s">
+      <c r="B5" s="82"/>
+      <c r="C5" s="83"/>
+      <c r="D5" s="40" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="76"/>
-      <c r="C6" s="75"/>
-      <c r="D6" s="42" t="s">
+      <c r="B6" s="82"/>
+      <c r="C6" s="83"/>
+      <c r="D6" s="41" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="7" spans="2:4" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="76">
+      <c r="B7" s="82">
         <v>45684</v>
       </c>
-      <c r="C7" s="75">
+      <c r="C7" s="83">
         <v>1.5</v>
       </c>
-      <c r="D7" s="36" t="s">
+      <c r="D7" s="35" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="8" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="76"/>
-      <c r="C8" s="75"/>
-      <c r="D8" s="37" t="s">
+      <c r="B8" s="82"/>
+      <c r="C8" s="83"/>
+      <c r="D8" s="36" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="9" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="76"/>
-      <c r="C9" s="75"/>
-      <c r="D9" s="43" t="s">
+      <c r="B9" s="82"/>
+      <c r="C9" s="83"/>
+      <c r="D9" s="42" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="10" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="76"/>
-      <c r="C10" s="75"/>
-      <c r="D10" s="44" t="s">
+      <c r="B10" s="82"/>
+      <c r="C10" s="83"/>
+      <c r="D10" s="43" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="76">
+      <c r="B11" s="82">
         <v>45686</v>
       </c>
-      <c r="C11" s="75">
+      <c r="C11" s="83">
         <v>3</v>
       </c>
-      <c r="D11" s="35" t="s">
+      <c r="D11" s="34" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="12" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="76"/>
-      <c r="C12" s="75"/>
-      <c r="D12" s="35" t="s">
+      <c r="B12" s="82"/>
+      <c r="C12" s="83"/>
+      <c r="D12" s="34" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="76"/>
-      <c r="C13" s="75"/>
-      <c r="D13" s="35" t="s">
+      <c r="B13" s="82"/>
+      <c r="C13" s="83"/>
+      <c r="D13" s="34" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="76"/>
-      <c r="C14" s="75"/>
-      <c r="D14" s="45" t="s">
+      <c r="B14" s="82"/>
+      <c r="C14" s="83"/>
+      <c r="D14" s="44" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="76"/>
-      <c r="C15" s="75"/>
-      <c r="D15" s="42" t="s">
+      <c r="B15" s="82"/>
+      <c r="C15" s="83"/>
+      <c r="D15" s="41" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="76">
+      <c r="B16" s="82">
         <v>46053</v>
       </c>
-      <c r="C16" s="75">
+      <c r="C16" s="83">
         <v>4</v>
       </c>
-      <c r="D16" s="38" t="s">
+      <c r="D16" s="37" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="76"/>
-      <c r="C17" s="75"/>
-      <c r="D17" s="35" t="s">
+      <c r="B17" s="82"/>
+      <c r="C17" s="83"/>
+      <c r="D17" s="34" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="76"/>
-      <c r="C18" s="75"/>
-      <c r="D18" s="35" t="s">
+      <c r="B18" s="82"/>
+      <c r="C18" s="83"/>
+      <c r="D18" s="34" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="19" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="76"/>
-      <c r="C19" s="75"/>
-      <c r="D19" s="35" t="s">
+      <c r="B19" s="82"/>
+      <c r="C19" s="83"/>
+      <c r="D19" s="34" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="20" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="76"/>
-      <c r="C20" s="75"/>
-      <c r="D20" s="35" t="s">
+      <c r="B20" s="82"/>
+      <c r="C20" s="83"/>
+      <c r="D20" s="34" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="21" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="76"/>
-      <c r="C21" s="75"/>
-      <c r="D21" s="35" t="s">
+      <c r="B21" s="82"/>
+      <c r="C21" s="83"/>
+      <c r="D21" s="34" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="76"/>
-      <c r="C22" s="75"/>
-      <c r="D22" s="45" t="s">
+      <c r="B22" s="82"/>
+      <c r="C22" s="83"/>
+      <c r="D22" s="44" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="23" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="76"/>
-      <c r="C23" s="75"/>
-      <c r="D23" s="41" t="s">
+      <c r="B23" s="82"/>
+      <c r="C23" s="83"/>
+      <c r="D23" s="40" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="24" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="76"/>
-      <c r="C24" s="75"/>
-      <c r="D24" s="41" t="s">
+      <c r="B24" s="82"/>
+      <c r="C24" s="83"/>
+      <c r="D24" s="40" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="25" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="76"/>
-      <c r="C25" s="75"/>
-      <c r="D25" s="41" t="s">
+      <c r="B25" s="82"/>
+      <c r="C25" s="83"/>
+      <c r="D25" s="40" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="26" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="76"/>
-      <c r="C26" s="75"/>
-      <c r="D26" s="46" t="s">
+      <c r="B26" s="82"/>
+      <c r="C26" s="83"/>
+      <c r="D26" s="45" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="27" spans="2:4" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="76">
+      <c r="B27" s="82">
         <v>46054</v>
       </c>
-      <c r="C27" s="75">
+      <c r="C27" s="83">
         <v>1</v>
       </c>
-      <c r="D27" s="35" t="s">
+      <c r="D27" s="34" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="28" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="76"/>
-      <c r="C28" s="75"/>
-      <c r="D28" s="35" t="s">
+      <c r="B28" s="82"/>
+      <c r="C28" s="83"/>
+      <c r="D28" s="34" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="29" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="76"/>
-      <c r="C29" s="75"/>
-      <c r="D29" s="41" t="s">
+      <c r="B29" s="82"/>
+      <c r="C29" s="83"/>
+      <c r="D29" s="40" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="30" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="76"/>
-      <c r="C30" s="75"/>
-      <c r="D30" s="42" t="s">
+      <c r="B30" s="82"/>
+      <c r="C30" s="83"/>
+      <c r="D30" s="41" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="31" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B31" s="76">
+      <c r="B31" s="82">
         <v>46055</v>
       </c>
-      <c r="C31" s="75">
+      <c r="C31" s="83">
         <v>4</v>
       </c>
-      <c r="D31" s="39" t="s">
+      <c r="D31" s="38" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="32" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B32" s="76"/>
-      <c r="C32" s="75"/>
-      <c r="D32" s="40" t="s">
+      <c r="B32" s="82"/>
+      <c r="C32" s="83"/>
+      <c r="D32" s="39" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="33" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="76"/>
-      <c r="C33" s="75"/>
-      <c r="D33" s="40" t="s">
+      <c r="B33" s="82"/>
+      <c r="C33" s="83"/>
+      <c r="D33" s="39" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="34" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B34" s="76"/>
-      <c r="C34" s="75"/>
-      <c r="D34" s="40" t="s">
+      <c r="B34" s="82"/>
+      <c r="C34" s="83"/>
+      <c r="D34" s="39" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="35" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B35" s="76"/>
-      <c r="C35" s="75"/>
-      <c r="D35" s="47" t="s">
+      <c r="B35" s="82"/>
+      <c r="C35" s="83"/>
+      <c r="D35" s="46" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="36" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B36" s="76"/>
-      <c r="C36" s="75"/>
-      <c r="D36" s="48" t="s">
+      <c r="B36" s="82"/>
+      <c r="C36" s="83"/>
+      <c r="D36" s="47" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="37" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="76">
+      <c r="B37" s="82">
         <v>46056</v>
       </c>
-      <c r="C37" s="75">
+      <c r="C37" s="83">
         <v>3</v>
       </c>
-      <c r="D37" s="35" t="s">
+      <c r="D37" s="34" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="38" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B38" s="76"/>
-      <c r="C38" s="75"/>
-      <c r="D38" s="35" t="s">
+      <c r="B38" s="82"/>
+      <c r="C38" s="83"/>
+      <c r="D38" s="34" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="39" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B39" s="76"/>
-      <c r="C39" s="75"/>
-      <c r="D39" s="35" t="s">
+      <c r="B39" s="82"/>
+      <c r="C39" s="83"/>
+      <c r="D39" s="34" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="40" spans="2:4" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B40" s="76"/>
-      <c r="C40" s="75"/>
-      <c r="D40" s="41" t="s">
+      <c r="B40" s="82"/>
+      <c r="C40" s="83"/>
+      <c r="D40" s="40" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="41" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B41" s="76"/>
-      <c r="C41" s="75"/>
-      <c r="D41" s="42" t="s">
+      <c r="B41" s="82"/>
+      <c r="C41" s="83"/>
+      <c r="D41" s="41" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="42" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B42" s="76">
+      <c r="B42" s="82">
         <v>46057</v>
       </c>
-      <c r="C42" s="75">
+      <c r="C42" s="83">
         <v>4</v>
       </c>
-      <c r="D42" s="38" t="s">
+      <c r="D42" s="37" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="43" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B43" s="76"/>
-      <c r="C43" s="75"/>
-      <c r="D43" s="35" t="s">
+      <c r="B43" s="82"/>
+      <c r="C43" s="83"/>
+      <c r="D43" s="34" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="44" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B44" s="76"/>
-      <c r="C44" s="75"/>
-      <c r="D44" s="42" t="s">
+      <c r="B44" s="82"/>
+      <c r="C44" s="83"/>
+      <c r="D44" s="41" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="45" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B45" s="77">
+      <c r="B45" s="79">
         <v>46059</v>
       </c>
-      <c r="C45" s="80">
+      <c r="C45" s="76">
         <v>2</v>
       </c>
-      <c r="D45" s="50" t="s">
+      <c r="D45" s="49" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="46" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B46" s="78"/>
-      <c r="C46" s="81"/>
-      <c r="D46" s="49" t="s">
+      <c r="B46" s="80"/>
+      <c r="C46" s="77"/>
+      <c r="D46" s="48" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="47" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B47" s="78"/>
-      <c r="C47" s="81"/>
-      <c r="D47" s="35" t="s">
+      <c r="B47" s="80"/>
+      <c r="C47" s="77"/>
+      <c r="D47" s="34" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="48" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B48" s="78"/>
-      <c r="C48" s="81"/>
-      <c r="D48" s="42" t="s">
+      <c r="B48" s="80"/>
+      <c r="C48" s="77"/>
+      <c r="D48" s="41" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="49" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B49" s="79"/>
-      <c r="C49" s="82"/>
-      <c r="D49" s="46" t="s">
+      <c r="B49" s="81"/>
+      <c r="C49" s="78"/>
+      <c r="D49" s="45" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="50" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B50" s="77">
+      <c r="B50" s="79">
         <v>46061</v>
       </c>
-      <c r="C50" s="80">
+      <c r="C50" s="76">
         <v>1.5</v>
       </c>
-      <c r="D50" s="50" t="s">
+      <c r="D50" s="49" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="51" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B51" s="78"/>
-      <c r="C51" s="81"/>
-      <c r="D51" s="35" t="s">
+      <c r="B51" s="80"/>
+      <c r="C51" s="77"/>
+      <c r="D51" s="34" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="52" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B52" s="78"/>
-      <c r="C52" s="81"/>
-      <c r="D52" s="42" t="s">
+      <c r="B52" s="80"/>
+      <c r="C52" s="77"/>
+      <c r="D52" s="41" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="53" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B53" s="78"/>
-      <c r="C53" s="81"/>
-      <c r="D53" s="42" t="s">
+      <c r="B53" s="80"/>
+      <c r="C53" s="77"/>
+      <c r="D53" s="41" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="54" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B54" s="79"/>
-      <c r="C54" s="82"/>
-      <c r="D54" s="46" t="s">
+      <c r="B54" s="81"/>
+      <c r="C54" s="78"/>
+      <c r="D54" s="45" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="55" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="77">
+      <c r="B55" s="79">
         <v>46062</v>
       </c>
-      <c r="C55" s="80">
+      <c r="C55" s="76">
         <v>2</v>
       </c>
-      <c r="D55" s="54" t="s">
+      <c r="D55" s="52" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="56" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B56" s="78"/>
-      <c r="C56" s="81"/>
-      <c r="D56" s="55" t="s">
+      <c r="B56" s="80"/>
+      <c r="C56" s="77"/>
+      <c r="D56" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="57" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B57" s="78"/>
-      <c r="C57" s="81"/>
-      <c r="D57" s="42" t="s">
+      <c r="B57" s="80"/>
+      <c r="C57" s="77"/>
+      <c r="D57" s="41" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="58" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B58" s="79"/>
-      <c r="C58" s="82"/>
-      <c r="D58" s="46" t="s">
+      <c r="B58" s="81"/>
+      <c r="C58" s="78"/>
+      <c r="D58" s="45" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="59" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="77">
+      <c r="B59" s="79">
         <v>46063</v>
       </c>
-      <c r="C59" s="80">
+      <c r="C59" s="76">
         <v>3</v>
       </c>
-      <c r="D59" s="54" t="s">
+      <c r="D59" s="52" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="60" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B60" s="78"/>
-      <c r="C60" s="81"/>
-      <c r="D60" s="55" t="s">
+      <c r="B60" s="80"/>
+      <c r="C60" s="77"/>
+      <c r="D60" s="53" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="61" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B61" s="78"/>
-      <c r="C61" s="81"/>
-      <c r="D61" s="55" t="s">
+      <c r="B61" s="80"/>
+      <c r="C61" s="77"/>
+      <c r="D61" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="62" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B62" s="78"/>
-      <c r="C62" s="81"/>
-      <c r="D62" s="42" t="s">
+      <c r="B62" s="80"/>
+      <c r="C62" s="77"/>
+      <c r="D62" s="41" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="63" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B63" s="79"/>
-      <c r="C63" s="82"/>
-      <c r="D63" s="46" t="s">
+      <c r="B63" s="81"/>
+      <c r="C63" s="78"/>
+      <c r="D63" s="45" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="64" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B64" s="77">
+      <c r="B64" s="79">
         <v>46064</v>
       </c>
-      <c r="C64" s="80">
+      <c r="C64" s="76">
         <v>3</v>
       </c>
-      <c r="D64" s="54" t="s">
+      <c r="D64" s="52" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="65" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B65" s="78"/>
-      <c r="C65" s="81"/>
-      <c r="D65" s="55" t="s">
+      <c r="B65" s="80"/>
+      <c r="C65" s="77"/>
+      <c r="D65" s="53" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="66" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B66" s="78"/>
-      <c r="C66" s="81"/>
-      <c r="D66" s="55" t="s">
+      <c r="B66" s="80"/>
+      <c r="C66" s="77"/>
+      <c r="D66" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="67" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B67" s="78"/>
-      <c r="C67" s="81"/>
-      <c r="D67" s="42" t="s">
+      <c r="B67" s="80"/>
+      <c r="C67" s="77"/>
+      <c r="D67" s="41" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="68" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B68" s="79"/>
-      <c r="C68" s="82"/>
-      <c r="D68" s="46" t="s">
+      <c r="B68" s="81"/>
+      <c r="C68" s="78"/>
+      <c r="D68" s="45" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="69" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B69" s="83">
+      <c r="B69" s="73">
         <v>46066</v>
       </c>
-      <c r="C69" s="80">
+      <c r="C69" s="76">
         <v>2</v>
       </c>
-      <c r="D69" s="54" t="s">
+      <c r="D69" s="52" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="70" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B70" s="84"/>
-      <c r="C70" s="81"/>
-      <c r="D70" s="55" t="s">
+      <c r="B70" s="74"/>
+      <c r="C70" s="77"/>
+      <c r="D70" s="53" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="71" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B71" s="84"/>
-      <c r="C71" s="81"/>
-      <c r="D71" s="55" t="s">
+      <c r="B71" s="74"/>
+      <c r="C71" s="77"/>
+      <c r="D71" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="72" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B72" s="84"/>
-      <c r="C72" s="81"/>
-      <c r="D72" s="42" t="s">
+      <c r="B72" s="74"/>
+      <c r="C72" s="77"/>
+      <c r="D72" s="41" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="73" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B73" s="84"/>
-      <c r="C73" s="81"/>
-      <c r="D73" s="42" t="s">
+      <c r="B73" s="74"/>
+      <c r="C73" s="77"/>
+      <c r="D73" s="41" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="74" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B74" s="85"/>
-      <c r="C74" s="82"/>
-      <c r="D74" s="46" t="s">
+      <c r="B74" s="75"/>
+      <c r="C74" s="78"/>
+      <c r="D74" s="45" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="75" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B75" s="69">
+      <c r="B75" s="67">
         <v>46068</v>
       </c>
-      <c r="C75" s="72">
+      <c r="C75" s="70">
         <v>2.5</v>
       </c>
-      <c r="D75" s="54" t="s">
+      <c r="D75" s="52" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="76" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B76" s="70"/>
-      <c r="C76" s="73"/>
-      <c r="D76" s="55" t="s">
+      <c r="B76" s="68"/>
+      <c r="C76" s="71"/>
+      <c r="D76" s="53" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="77" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B77" s="70"/>
-      <c r="C77" s="73"/>
-      <c r="D77" s="55" t="s">
+      <c r="B77" s="68"/>
+      <c r="C77" s="71"/>
+      <c r="D77" s="53" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="78" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B78" s="70"/>
-      <c r="C78" s="73"/>
-      <c r="D78" s="55" t="s">
+      <c r="B78" s="68"/>
+      <c r="C78" s="71"/>
+      <c r="D78" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="79" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B79" s="70"/>
-      <c r="C79" s="73"/>
-      <c r="D79" s="42" t="s">
+      <c r="B79" s="68"/>
+      <c r="C79" s="71"/>
+      <c r="D79" s="41" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="80" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B80" s="70"/>
-      <c r="C80" s="73"/>
-      <c r="D80" s="42" t="s">
+      <c r="B80" s="68"/>
+      <c r="C80" s="71"/>
+      <c r="D80" s="41" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="81" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B81" s="71"/>
-      <c r="C81" s="74"/>
-      <c r="D81" s="46" t="s">
+      <c r="B81" s="69"/>
+      <c r="C81" s="72"/>
+      <c r="D81" s="45" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="82" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B82" s="69">
+      <c r="B82" s="67">
         <v>46070</v>
       </c>
-      <c r="C82" s="72">
+      <c r="C82" s="70">
         <v>3</v>
       </c>
-      <c r="D82" s="54" t="s">
+      <c r="D82" s="52" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="83" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B83" s="70"/>
-      <c r="C83" s="73"/>
-      <c r="D83" s="55" t="s">
+      <c r="B83" s="68"/>
+      <c r="C83" s="71"/>
+      <c r="D83" s="53" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="84" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B84" s="70"/>
-      <c r="C84" s="73"/>
-      <c r="D84" s="55" t="s">
+      <c r="B84" s="68"/>
+      <c r="C84" s="71"/>
+      <c r="D84" s="53" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="85" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B85" s="70"/>
-      <c r="C85" s="73"/>
-      <c r="D85" s="55" t="s">
+      <c r="B85" s="68"/>
+      <c r="C85" s="71"/>
+      <c r="D85" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="86" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B86" s="70"/>
-      <c r="C86" s="73"/>
-      <c r="D86" s="42" t="s">
+      <c r="B86" s="68"/>
+      <c r="C86" s="71"/>
+      <c r="D86" s="41" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="87" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B87" s="70"/>
-      <c r="C87" s="73"/>
-      <c r="D87" s="42" t="s">
+      <c r="B87" s="68"/>
+      <c r="C87" s="71"/>
+      <c r="D87" s="41" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="88" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B88" s="71"/>
-      <c r="C88" s="74"/>
-      <c r="D88" s="46" t="s">
+      <c r="B88" s="69"/>
+      <c r="C88" s="72"/>
+      <c r="D88" s="45" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="89" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B89" s="69">
+      <c r="B89" s="67">
         <v>46071</v>
       </c>
-      <c r="C89" s="72">
+      <c r="C89" s="70">
         <v>2</v>
       </c>
-      <c r="D89" s="54" t="s">
+      <c r="D89" s="52" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="90" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B90" s="70"/>
-      <c r="C90" s="73"/>
-      <c r="D90" s="55" t="s">
+      <c r="B90" s="68"/>
+      <c r="C90" s="71"/>
+      <c r="D90" s="53" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="91" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B91" s="70"/>
-      <c r="C91" s="73"/>
-      <c r="D91" s="55" t="s">
+      <c r="B91" s="68"/>
+      <c r="C91" s="71"/>
+      <c r="D91" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="92" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B92" s="70"/>
-      <c r="C92" s="73"/>
-      <c r="D92" s="42" t="s">
+      <c r="B92" s="68"/>
+      <c r="C92" s="71"/>
+      <c r="D92" s="41" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="93" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B93" s="71"/>
-      <c r="C93" s="74"/>
-      <c r="D93" s="46" t="s">
+      <c r="B93" s="69"/>
+      <c r="C93" s="72"/>
+      <c r="D93" s="45" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="94" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B94" s="69">
+      <c r="B94" s="67">
         <v>46074</v>
       </c>
-      <c r="C94" s="72">
+      <c r="C94" s="70">
         <v>3</v>
       </c>
-      <c r="D94" s="57" t="s">
+      <c r="D94" s="55" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="95" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B95" s="70"/>
-      <c r="C95" s="73"/>
-      <c r="D95" s="58" t="s">
+      <c r="B95" s="68"/>
+      <c r="C95" s="71"/>
+      <c r="D95" s="56" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="96" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B96" s="71"/>
-      <c r="C96" s="74"/>
-      <c r="D96" s="46" t="s">
+      <c r="B96" s="69"/>
+      <c r="C96" s="72"/>
+      <c r="D96" s="45" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="97" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B97" s="69">
+      <c r="B97" s="67">
         <v>46075</v>
       </c>
-      <c r="C97" s="72">
+      <c r="C97" s="70">
         <v>3</v>
       </c>
-      <c r="D97" s="54" t="s">
+      <c r="D97" s="52" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="98" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B98" s="70"/>
-      <c r="C98" s="73"/>
-      <c r="D98" s="55" t="s">
+      <c r="B98" s="68"/>
+      <c r="C98" s="71"/>
+      <c r="D98" s="53" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="99" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B99" s="70"/>
-      <c r="C99" s="73"/>
-      <c r="D99" s="55" t="s">
+      <c r="B99" s="68"/>
+      <c r="C99" s="71"/>
+      <c r="D99" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="100" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B100" s="71"/>
-      <c r="C100" s="74"/>
-      <c r="D100" s="46" t="s">
+      <c r="B100" s="69"/>
+      <c r="C100" s="72"/>
+      <c r="D100" s="45" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="101" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B101" s="59">
+      <c r="B101" s="57">
         <v>46076</v>
       </c>
-      <c r="C101" s="60">
+      <c r="C101" s="58">
         <v>4</v>
       </c>
-      <c r="D101" s="61" t="s">
+      <c r="D101" s="59" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="102" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B102" s="69">
+      <c r="B102" s="67">
         <v>46077</v>
       </c>
-      <c r="C102" s="72">
+      <c r="C102" s="70">
         <v>2</v>
       </c>
-      <c r="D102" s="54" t="s">
+      <c r="D102" s="52" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="103" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B103" s="70"/>
-      <c r="C103" s="73"/>
-      <c r="D103" s="55" t="s">
+      <c r="B103" s="68"/>
+      <c r="C103" s="71"/>
+      <c r="D103" s="53" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="104" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B104" s="70"/>
-      <c r="C104" s="73"/>
-      <c r="D104" s="55" t="s">
+      <c r="B104" s="68"/>
+      <c r="C104" s="71"/>
+      <c r="D104" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="105" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B105" s="70"/>
-      <c r="C105" s="73"/>
-      <c r="D105" s="42" t="s">
+      <c r="B105" s="68"/>
+      <c r="C105" s="71"/>
+      <c r="D105" s="41" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="106" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B106" s="71"/>
-      <c r="C106" s="74"/>
-      <c r="D106" s="46" t="s">
+      <c r="B106" s="69"/>
+      <c r="C106" s="72"/>
+      <c r="D106" s="45" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="107" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B107" s="69">
+      <c r="B107" s="67">
         <v>46078</v>
       </c>
-      <c r="C107" s="72">
+      <c r="C107" s="70">
         <v>1</v>
       </c>
-      <c r="D107" s="65" t="s">
+      <c r="D107" s="63" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="108" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B108" s="70"/>
-      <c r="C108" s="73"/>
-      <c r="D108" s="55" t="s">
+      <c r="B108" s="68"/>
+      <c r="C108" s="71"/>
+      <c r="D108" s="53" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="109" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B109" s="70"/>
-      <c r="C109" s="73"/>
-      <c r="D109" s="42" t="s">
+      <c r="B109" s="68"/>
+      <c r="C109" s="71"/>
+      <c r="D109" s="41" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="110" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B110" s="70"/>
-      <c r="C110" s="73"/>
-      <c r="D110" s="42" t="s">
+      <c r="B110" s="68"/>
+      <c r="C110" s="71"/>
+      <c r="D110" s="41" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="111" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B111" s="71"/>
-      <c r="C111" s="74"/>
-      <c r="D111" s="66" t="s">
+      <c r="B111" s="69"/>
+      <c r="C111" s="72"/>
+      <c r="D111" s="64" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="112" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B112" s="69">
+      <c r="B112" s="67">
         <v>46079</v>
       </c>
-      <c r="C112" s="72">
+      <c r="C112" s="70">
         <v>2</v>
       </c>
-      <c r="D112" s="65" t="s">
+      <c r="D112" s="63" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="113" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B113" s="70"/>
-      <c r="C113" s="73"/>
-      <c r="D113" s="55" t="s">
+      <c r="B113" s="68"/>
+      <c r="C113" s="71"/>
+      <c r="D113" s="53" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="114" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B114" s="70"/>
-      <c r="C114" s="73"/>
-      <c r="D114" s="42" t="s">
+      <c r="B114" s="68"/>
+      <c r="C114" s="71"/>
+      <c r="D114" s="41" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="115" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B115" s="71"/>
-      <c r="C115" s="74"/>
-      <c r="D115" s="46" t="s">
+      <c r="B115" s="69"/>
+      <c r="C115" s="72"/>
+      <c r="D115" s="45" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="116" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B116" s="69">
+      <c r="B116" s="67">
         <v>46083</v>
       </c>
-      <c r="C116" s="72">
+      <c r="C116" s="70">
         <v>3</v>
       </c>
-      <c r="D116" s="65" t="s">
+      <c r="D116" s="63" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="117" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B117" s="70"/>
-      <c r="C117" s="73"/>
-      <c r="D117" s="55" t="s">
+      <c r="B117" s="68"/>
+      <c r="C117" s="71"/>
+      <c r="D117" s="53" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="118" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B118" s="70"/>
-      <c r="C118" s="73"/>
-      <c r="D118" s="55" t="s">
+      <c r="B118" s="68"/>
+      <c r="C118" s="71"/>
+      <c r="D118" s="53" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="119" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B119" s="71"/>
-      <c r="C119" s="74"/>
-      <c r="D119" s="46" t="s">
+      <c r="B119" s="69"/>
+      <c r="C119" s="72"/>
+      <c r="D119" s="45" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="120" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B120" s="69">
+      <c r="B120" s="67">
         <v>411326</v>
       </c>
-      <c r="C120" s="72">
+      <c r="C120" s="70">
         <v>5</v>
       </c>
-      <c r="D120" s="65" t="s">
+      <c r="D120" s="63" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="121" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B121" s="70"/>
-      <c r="C121" s="73"/>
-      <c r="D121" s="55" t="s">
+      <c r="B121" s="68"/>
+      <c r="C121" s="71"/>
+      <c r="D121" s="53" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="122" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B122" s="71"/>
-      <c r="C122" s="74"/>
-      <c r="D122" s="67" t="s">
+      <c r="B122" s="69"/>
+      <c r="C122" s="72"/>
+      <c r="D122" s="65" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="123" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B123" s="68">
+      <c r="B123" s="89">
         <v>46085</v>
       </c>
-      <c r="C123" s="56">
+      <c r="C123" s="90">
         <v>4</v>
       </c>
-      <c r="D123" s="65" t="s">
+      <c r="D123" s="63" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="124" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B124" s="56"/>
-      <c r="C124" s="56"/>
-      <c r="D124" s="55" t="s">
+      <c r="B124" s="91"/>
+      <c r="C124" s="92"/>
+      <c r="D124" s="53" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="125" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B125" s="32"/>
-      <c r="C125" s="32"/>
-      <c r="D125" s="55" t="s">
+      <c r="B125" s="91"/>
+      <c r="C125" s="92"/>
+      <c r="D125" s="53" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="126" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B126" s="56"/>
-      <c r="C126" s="56"/>
-      <c r="D126" s="42" t="s">
+      <c r="B126" s="91"/>
+      <c r="C126" s="92"/>
+      <c r="D126" s="41" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="127" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B127" s="32"/>
-      <c r="C127" s="32"/>
-      <c r="D127" s="42" t="s">
+    <row r="127" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B127" s="93"/>
+      <c r="C127" s="94"/>
+      <c r="D127" s="45" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="128" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B128" s="32"/>
-      <c r="C128" s="32"/>
-      <c r="D128" s="33"/>
+      <c r="B128" s="66">
+        <v>46086</v>
+      </c>
+      <c r="C128" s="54">
+        <v>6</v>
+      </c>
+      <c r="D128" s="63" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="129" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B129" s="56"/>
-      <c r="C129" s="56"/>
-      <c r="D129" s="51"/>
+      <c r="B129" s="66"/>
+      <c r="C129" s="54"/>
+      <c r="D129" s="53" t="s">
+        <v>174</v>
+      </c>
     </row>
     <row r="130" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B130" s="32"/>
-      <c r="C130" s="32"/>
-      <c r="D130" s="33"/>
-    </row>
-    <row r="131" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B131" s="32"/>
-      <c r="C131" s="32"/>
-      <c r="D131" s="33"/>
-    </row>
-    <row r="132" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B132" s="56"/>
-      <c r="C132" s="56"/>
-      <c r="D132" s="51"/>
-    </row>
-    <row r="133" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B130" s="54"/>
+      <c r="C130" s="54"/>
+      <c r="D130" s="53" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="131" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B131" s="54"/>
+      <c r="C131" s="54"/>
+      <c r="D131" s="95" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="132" spans="2:4" ht="78" x14ac:dyDescent="0.3">
+      <c r="B132" s="32"/>
+      <c r="C132" s="32"/>
+      <c r="D132" s="95" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="133" spans="2:4" ht="78" x14ac:dyDescent="0.3">
       <c r="B133" s="32"/>
       <c r="C133" s="32"/>
-      <c r="D133" s="33"/>
-    </row>
-    <row r="134" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B134" s="32"/>
-      <c r="C134" s="32"/>
-      <c r="D134" s="33"/>
-    </row>
-    <row r="135" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B135" s="56"/>
-      <c r="C135" s="56"/>
-      <c r="D135" s="51"/>
-    </row>
-    <row r="136" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="D133" s="95" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="134" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B134" s="54"/>
+      <c r="C134" s="54"/>
+      <c r="D134" s="95" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="135" spans="2:4" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="B135" s="32"/>
+      <c r="C135" s="32"/>
+      <c r="D135" s="95" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="136" spans="2:4" ht="62.4" x14ac:dyDescent="0.3">
       <c r="B136" s="32"/>
       <c r="C136" s="32"/>
-      <c r="D136" s="33"/>
-    </row>
-    <row r="137" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B137" s="32"/>
-      <c r="C137" s="32"/>
-      <c r="D137" s="33"/>
-    </row>
-    <row r="138" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B138" s="56"/>
-      <c r="C138" s="56"/>
-      <c r="D138" s="51"/>
-    </row>
-    <row r="139" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="D136" s="95" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="137" spans="2:4" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="B137" s="54"/>
+      <c r="C137"/>
+      <c r="D137" s="95" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="138" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B138" s="32"/>
+      <c r="C138"/>
+      <c r="D138" s="95" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="139" spans="2:4" ht="78" x14ac:dyDescent="0.3">
       <c r="B139" s="32"/>
       <c r="C139" s="32"/>
-      <c r="D139" s="33"/>
-    </row>
-    <row r="140" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B140" s="32"/>
-      <c r="C140" s="32"/>
-      <c r="D140" s="33"/>
+      <c r="D139" s="95" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="140" spans="2:4" ht="78" x14ac:dyDescent="0.3">
+      <c r="B140" s="54"/>
+      <c r="C140" s="54"/>
+      <c r="D140" s="95" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="141" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B141" s="32"/>
+      <c r="C141" s="32"/>
+      <c r="D141" s="95" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="142" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B142" s="32"/>
+      <c r="C142" s="32"/>
+      <c r="D142" s="95" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="143" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B143" s="32"/>
+      <c r="C143" s="32"/>
+      <c r="D143" s="95"/>
+    </row>
+    <row r="144" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B144" s="32"/>
+      <c r="C144" s="32"/>
+      <c r="D144" s="95"/>
+    </row>
+    <row r="145" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B145" s="32"/>
+      <c r="C145" s="32"/>
+      <c r="D145" s="95"/>
+    </row>
+    <row r="146" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B146" s="32"/>
+      <c r="C146" s="32"/>
+      <c r="D146" s="95"/>
+    </row>
+    <row r="147" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B147" s="32"/>
+      <c r="C147" s="32"/>
+      <c r="D147" s="95"/>
+    </row>
+    <row r="148" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B148" s="32"/>
+      <c r="C148" s="32"/>
+      <c r="D148" s="95"/>
+    </row>
+    <row r="149" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B149" s="32"/>
+      <c r="C149" s="32"/>
+      <c r="D149" s="95"/>
+    </row>
+    <row r="150" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B150" s="32"/>
+      <c r="C150" s="32"/>
+      <c r="D150" s="95"/>
+    </row>
+    <row r="151" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B151" s="32"/>
+      <c r="C151" s="32"/>
+      <c r="D151" s="95"/>
+    </row>
+    <row r="152" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B152" s="32"/>
+      <c r="C152" s="32"/>
+      <c r="D152" s="95"/>
+    </row>
+    <row r="153" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B153" s="32"/>
+      <c r="C153" s="32"/>
+      <c r="D153" s="95"/>
+    </row>
+    <row r="154" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B154" s="32"/>
+      <c r="C154" s="32"/>
+      <c r="D154" s="95"/>
+    </row>
+    <row r="155" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B155" s="32"/>
+      <c r="C155" s="32"/>
+      <c r="D155" s="95"/>
+    </row>
+    <row r="156" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B156" s="32"/>
+      <c r="C156" s="32"/>
+      <c r="D156" s="95"/>
+    </row>
+    <row r="157" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B157" s="32"/>
+      <c r="C157" s="32"/>
+      <c r="D157" s="95"/>
+    </row>
+    <row r="158" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B158" s="32"/>
+      <c r="C158" s="32"/>
+      <c r="D158" s="95"/>
+    </row>
+    <row r="159" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B159" s="32"/>
+      <c r="C159" s="32"/>
+      <c r="D159" s="95"/>
+    </row>
+    <row r="160" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B160" s="32"/>
+      <c r="C160" s="32"/>
+      <c r="D160" s="95"/>
+    </row>
+    <row r="161" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B161" s="32"/>
+      <c r="C161" s="32"/>
+      <c r="D161" s="95"/>
+    </row>
+    <row r="162" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B162" s="32"/>
+      <c r="C162" s="32"/>
+      <c r="D162" s="95"/>
+    </row>
+    <row r="163" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B163" s="32"/>
+      <c r="C163" s="32"/>
+      <c r="D163" s="95"/>
+    </row>
+    <row r="164" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B164" s="32"/>
+      <c r="C164" s="32"/>
+      <c r="D164" s="95"/>
+    </row>
+    <row r="165" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B165" s="32"/>
+      <c r="C165" s="32"/>
+      <c r="D165" s="95"/>
+    </row>
+    <row r="166" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B166" s="32"/>
+      <c r="C166" s="32"/>
+      <c r="D166" s="95"/>
+    </row>
+    <row r="167" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B167" s="32"/>
+      <c r="C167" s="32"/>
+      <c r="D167" s="95"/>
+    </row>
+    <row r="168" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B168" s="32"/>
+      <c r="C168" s="32"/>
+      <c r="D168" s="95"/>
+    </row>
+    <row r="169" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B169" s="32"/>
+      <c r="C169" s="32"/>
+      <c r="D169" s="95"/>
+    </row>
+    <row r="170" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B170" s="32"/>
+      <c r="C170" s="32"/>
+      <c r="D170" s="95"/>
+    </row>
+    <row r="171" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B171" s="32"/>
+      <c r="C171" s="32"/>
+      <c r="D171" s="95"/>
+    </row>
+    <row r="172" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B172" s="32"/>
+      <c r="C172" s="32"/>
+      <c r="D172" s="95"/>
+    </row>
+    <row r="173" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B173" s="32"/>
+      <c r="C173" s="32"/>
+      <c r="D173" s="95"/>
+    </row>
+    <row r="174" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D174" s="95"/>
     </row>
   </sheetData>
-  <mergeCells count="48">
-    <mergeCell ref="B120:B122"/>
-    <mergeCell ref="C120:C122"/>
-    <mergeCell ref="B112:B115"/>
-    <mergeCell ref="C112:C115"/>
-    <mergeCell ref="B116:B119"/>
-    <mergeCell ref="C116:C119"/>
-    <mergeCell ref="B69:B74"/>
-    <mergeCell ref="C69:C74"/>
-    <mergeCell ref="B75:B81"/>
-    <mergeCell ref="C75:C81"/>
-    <mergeCell ref="B102:B106"/>
-    <mergeCell ref="C102:C106"/>
-    <mergeCell ref="B97:B100"/>
-    <mergeCell ref="C97:C100"/>
-    <mergeCell ref="B82:B88"/>
-    <mergeCell ref="C82:C88"/>
-    <mergeCell ref="B89:B93"/>
-    <mergeCell ref="C89:C93"/>
-    <mergeCell ref="B94:B96"/>
-    <mergeCell ref="C94:C96"/>
-    <mergeCell ref="B45:B49"/>
-    <mergeCell ref="C45:C49"/>
-    <mergeCell ref="B50:B54"/>
-    <mergeCell ref="C50:C54"/>
-    <mergeCell ref="B64:B68"/>
-    <mergeCell ref="C64:C68"/>
-    <mergeCell ref="B3:B6"/>
-    <mergeCell ref="C3:C6"/>
-    <mergeCell ref="B7:B10"/>
-    <mergeCell ref="C7:C10"/>
-    <mergeCell ref="B11:B15"/>
-    <mergeCell ref="C11:C15"/>
+  <mergeCells count="50">
+    <mergeCell ref="B123:B127"/>
+    <mergeCell ref="C123:C127"/>
     <mergeCell ref="B107:B111"/>
     <mergeCell ref="C107:C111"/>
     <mergeCell ref="C16:C26"/>
@@ -4797,6 +5030,38 @@
     <mergeCell ref="C55:C58"/>
     <mergeCell ref="B59:B63"/>
     <mergeCell ref="C59:C63"/>
+    <mergeCell ref="B3:B6"/>
+    <mergeCell ref="C3:C6"/>
+    <mergeCell ref="B7:B10"/>
+    <mergeCell ref="C7:C10"/>
+    <mergeCell ref="B11:B15"/>
+    <mergeCell ref="C11:C15"/>
+    <mergeCell ref="B45:B49"/>
+    <mergeCell ref="C45:C49"/>
+    <mergeCell ref="B50:B54"/>
+    <mergeCell ref="C50:C54"/>
+    <mergeCell ref="B64:B68"/>
+    <mergeCell ref="C64:C68"/>
+    <mergeCell ref="B69:B74"/>
+    <mergeCell ref="C69:C74"/>
+    <mergeCell ref="B75:B81"/>
+    <mergeCell ref="C75:C81"/>
+    <mergeCell ref="B102:B106"/>
+    <mergeCell ref="C102:C106"/>
+    <mergeCell ref="B97:B100"/>
+    <mergeCell ref="C97:C100"/>
+    <mergeCell ref="B82:B88"/>
+    <mergeCell ref="C82:C88"/>
+    <mergeCell ref="B89:B93"/>
+    <mergeCell ref="C89:C93"/>
+    <mergeCell ref="B94:B96"/>
+    <mergeCell ref="C94:C96"/>
+    <mergeCell ref="B120:B122"/>
+    <mergeCell ref="C120:C122"/>
+    <mergeCell ref="B112:B115"/>
+    <mergeCell ref="C112:C115"/>
+    <mergeCell ref="B116:B119"/>
+    <mergeCell ref="C116:C119"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4820,41 +5085,41 @@
   </cols>
   <sheetData>
     <row r="2" spans="4:18" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D2" s="52" t="s">
+      <c r="D2" s="50" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="3" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D3" s="86" t="s">
+      <c r="D3" s="84" t="s">
         <v>8</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F3" s="88" t="s">
+      <c r="F3" s="86" t="s">
         <v>1</v>
       </c>
-      <c r="G3" s="89"/>
-      <c r="H3" s="89"/>
-      <c r="I3" s="90"/>
-      <c r="J3" s="88" t="s">
+      <c r="G3" s="87"/>
+      <c r="H3" s="87"/>
+      <c r="I3" s="88"/>
+      <c r="J3" s="86" t="s">
         <v>2</v>
       </c>
-      <c r="K3" s="89"/>
-      <c r="L3" s="89"/>
-      <c r="M3" s="90"/>
-      <c r="N3" s="88" t="s">
+      <c r="K3" s="87"/>
+      <c r="L3" s="87"/>
+      <c r="M3" s="88"/>
+      <c r="N3" s="86" t="s">
         <v>3</v>
       </c>
-      <c r="O3" s="89"/>
-      <c r="P3" s="89"/>
-      <c r="Q3" s="90"/>
+      <c r="O3" s="87"/>
+      <c r="P3" s="87"/>
+      <c r="Q3" s="88"/>
       <c r="R3" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="4:18" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D4" s="87"/>
+      <c r="D4" s="85"/>
       <c r="E4" s="4" t="s">
         <v>4</v>
       </c>
@@ -5019,42 +5284,42 @@
       <c r="Q11" s="14"/>
       <c r="R11" s="11"/>
     </row>
-    <row r="14" spans="4:18" s="53" customFormat="1" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D14" s="52" t="s">
+    <row r="14" spans="4:18" s="51" customFormat="1" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D14" s="50" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="15" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D15" s="86" t="s">
+      <c r="D15" s="84" t="s">
         <v>8</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F15" s="88" t="s">
+      <c r="F15" s="86" t="s">
         <v>1</v>
       </c>
-      <c r="G15" s="89"/>
-      <c r="H15" s="89"/>
-      <c r="I15" s="90"/>
-      <c r="J15" s="88" t="s">
+      <c r="G15" s="87"/>
+      <c r="H15" s="87"/>
+      <c r="I15" s="88"/>
+      <c r="J15" s="86" t="s">
         <v>2</v>
       </c>
-      <c r="K15" s="89"/>
-      <c r="L15" s="89"/>
-      <c r="M15" s="90"/>
-      <c r="N15" s="88" t="s">
+      <c r="K15" s="87"/>
+      <c r="L15" s="87"/>
+      <c r="M15" s="88"/>
+      <c r="N15" s="86" t="s">
         <v>3</v>
       </c>
-      <c r="O15" s="89"/>
-      <c r="P15" s="89"/>
-      <c r="Q15" s="90"/>
+      <c r="O15" s="87"/>
+      <c r="P15" s="87"/>
+      <c r="Q15" s="88"/>
       <c r="R15" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="16" spans="4:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D16" s="87"/>
+      <c r="D16" s="85"/>
       <c r="E16" s="4" t="s">
         <v>4</v>
       </c>
@@ -5220,55 +5485,55 @@
       <c r="R23" s="11"/>
     </row>
     <row r="26" spans="4:18" ht="33.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D26" s="52" t="s">
+      <c r="D26" s="50" t="s">
         <v>150</v>
       </c>
-      <c r="E26" s="53"/>
-      <c r="F26" s="53"/>
-      <c r="G26" s="53"/>
-      <c r="H26" s="53"/>
-      <c r="I26" s="53"/>
-      <c r="J26" s="53"/>
-      <c r="K26" s="53"/>
-      <c r="L26" s="53"/>
-      <c r="M26" s="53"/>
-      <c r="N26" s="53"/>
-      <c r="O26" s="53"/>
-      <c r="P26" s="53"/>
-      <c r="Q26" s="53"/>
-      <c r="R26" s="53"/>
+      <c r="E26" s="51"/>
+      <c r="F26" s="51"/>
+      <c r="G26" s="51"/>
+      <c r="H26" s="51"/>
+      <c r="I26" s="51"/>
+      <c r="J26" s="51"/>
+      <c r="K26" s="51"/>
+      <c r="L26" s="51"/>
+      <c r="M26" s="51"/>
+      <c r="N26" s="51"/>
+      <c r="O26" s="51"/>
+      <c r="P26" s="51"/>
+      <c r="Q26" s="51"/>
+      <c r="R26" s="51"/>
     </row>
     <row r="27" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D27" s="86" t="s">
+      <c r="D27" s="84" t="s">
         <v>8</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F27" s="88" t="s">
+      <c r="F27" s="86" t="s">
         <v>1</v>
       </c>
-      <c r="G27" s="89"/>
-      <c r="H27" s="89"/>
-      <c r="I27" s="90"/>
-      <c r="J27" s="88" t="s">
+      <c r="G27" s="87"/>
+      <c r="H27" s="87"/>
+      <c r="I27" s="88"/>
+      <c r="J27" s="86" t="s">
         <v>2</v>
       </c>
-      <c r="K27" s="89"/>
-      <c r="L27" s="89"/>
-      <c r="M27" s="90"/>
-      <c r="N27" s="88" t="s">
+      <c r="K27" s="87"/>
+      <c r="L27" s="87"/>
+      <c r="M27" s="88"/>
+      <c r="N27" s="86" t="s">
         <v>3</v>
       </c>
-      <c r="O27" s="89"/>
-      <c r="P27" s="89"/>
-      <c r="Q27" s="90"/>
+      <c r="O27" s="87"/>
+      <c r="P27" s="87"/>
+      <c r="Q27" s="88"/>
       <c r="R27" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="28" spans="4:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D28" s="87"/>
+      <c r="D28" s="85"/>
       <c r="E28" s="4" t="s">
         <v>4</v>
       </c>
@@ -5467,262 +5732,262 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="62" t="s">
+      <c r="B2" s="60" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="3" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="63" t="s">
+      <c r="B3" s="61" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="4" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="62" t="s">
+      <c r="B4" s="60" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="5" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="64" t="s">
+      <c r="B5" s="62" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="6" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="62" t="s">
+      <c r="B6" s="60" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="7" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="64" t="s">
+      <c r="B7" s="62" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="8" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="62" t="s">
+      <c r="B8" s="60" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="9" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="64" t="s">
+      <c r="B9" s="62" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="10" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="62" t="s">
+      <c r="B10" s="60" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="11" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="64" t="s">
+      <c r="B11" s="62" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="12" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="62" t="s">
+      <c r="B12" s="60" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="13" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="64" t="s">
+      <c r="B13" s="62" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="14" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="62" t="s">
+      <c r="B14" s="60" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="15" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="64" t="s">
+      <c r="B15" s="62" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="16" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="62" t="s">
+      <c r="B16" s="60" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="17" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="64" t="s">
+      <c r="B17" s="62" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="18" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="62" t="s">
+      <c r="B18" s="60" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="19" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="63" t="s">
+      <c r="B19" s="61" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="20" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="62" t="s">
+      <c r="B20" s="60" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="21" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="64" t="s">
+      <c r="B21" s="62" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="22" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="62" t="s">
+      <c r="B22" s="60" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="23" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="64" t="s">
+      <c r="B23" s="62" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="24" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="62" t="s">
+      <c r="B24" s="60" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="25" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="63" t="s">
+      <c r="B25" s="61" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="26" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="62" t="s">
+      <c r="B26" s="60" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="27" spans="2:2" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="B27" s="64" t="s">
+      <c r="B27" s="62" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="28" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="62" t="s">
+      <c r="B28" s="60" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="29" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="64" t="s">
+      <c r="B29" s="62" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="30" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="62" t="s">
+      <c r="B30" s="60" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="31" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="64" t="s">
+      <c r="B31" s="62" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="32" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="62" t="s">
+      <c r="B32" s="60" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="33" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="64" t="s">
+      <c r="B33" s="62" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="34" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="62" t="s">
+      <c r="B34" s="60" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="35" spans="2:2" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="64" t="s">
+      <c r="B35" s="62" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="36" spans="2:2" ht="15" x14ac:dyDescent="0.3">
-      <c r="B36" s="62" t="s">
+      <c r="B36" s="60" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="37" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B37" s="64" t="s">
+      <c r="B37" s="62" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="38" spans="2:2" ht="15" x14ac:dyDescent="0.3">
-      <c r="B38" s="62" t="s">
+      <c r="B38" s="60" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="39" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B39" s="64" t="s">
+      <c r="B39" s="62" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="40" spans="2:2" ht="15" x14ac:dyDescent="0.3">
-      <c r="B40" s="62" t="s">
+      <c r="B40" s="60" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="41" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B41" s="64" t="s">
+      <c r="B41" s="62" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="42" spans="2:2" ht="15" x14ac:dyDescent="0.3">
-      <c r="B42" s="62" t="s">
+      <c r="B42" s="60" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="43" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B43" s="64" t="s">
+      <c r="B43" s="62" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="44" spans="2:2" ht="15" x14ac:dyDescent="0.3">
-      <c r="B44" s="62" t="s">
+      <c r="B44" s="60" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="45" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B45" s="64" t="s">
+      <c r="B45" s="62" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="46" spans="2:2" ht="15" x14ac:dyDescent="0.3">
-      <c r="B46" s="62" t="s">
+      <c r="B46" s="60" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="47" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B47" s="64" t="s">
+      <c r="B47" s="62" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="48" spans="2:2" ht="15" x14ac:dyDescent="0.3">
-      <c r="B48" s="62" t="s">
+      <c r="B48" s="60" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="49" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B49" s="64" t="s">
+      <c r="B49" s="62" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="50" spans="2:2" ht="15" x14ac:dyDescent="0.3">
-      <c r="B50" s="62" t="s">
+      <c r="B50" s="60" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="51" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B51" s="64" t="s">
+      <c r="B51" s="62" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="52" spans="2:2" ht="15" x14ac:dyDescent="0.3">
-      <c r="B52" s="62" t="s">
+      <c r="B52" s="60" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="53" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B53" s="64" t="s">
+      <c r="B53" s="62" t="s">
         <v>156</v>
       </c>
     </row>

</xml_diff>

<commit_message>
debugged generation of dim-fact tables, created dashboard in PowerBI
</commit_message>
<xml_diff>
--- a/DocumentsAndReports/0. WorkLog_Charts.xlsx
+++ b/DocumentsAndReports/0. WorkLog_Charts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qhung\Videos\CSIS4495 - Applied Research  Project\W26_4495_S2_HughT\DocumentsAndReports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E3B3EEF-7650-4D38-8461-8FBEFDFAB5D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBA05676-7437-428C-BA2C-C8DB64E88782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="720" windowWidth="21600" windowHeight="11232" xr2:uid="{E067A1E6-0DC4-42DD-AAF8-D95EFF7A112F}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="184">
   <si>
     <t>January</t>
   </si>
@@ -991,6 +991,33 @@
   </si>
   <si>
     <t>- Modified SQL queries in database</t>
+  </si>
+  <si>
+    <t>- Debugged the generation of dim-fact tables</t>
+  </si>
+  <si>
+    <t>-  Created dashboard in PowerBI</t>
+  </si>
+  <si>
+    <t>"cur.executemany( """ INSERT INTO cleaned.dim_customer (CustomerID, CustomerName, City) SELECT ?, ?, ? WHERE NOT EXISTS (SELECT 1 FROM clean.dim_customer WHERE CustomerID = ?); """, [(r.CustomerID, r.CustomerName, r.City) for r in dim_customer.itertuples(index=False)] ) =&gt; explain in details"</t>
+  </si>
+  <si>
+    <t>"do this project really need 3 layers (raw-cleaned-analytics)? i think the analytics can be performed directly from the cleaned layer in powerBI with its measure feature"</t>
+  </si>
+  <si>
+    <t>"what is regular expression?"</t>
+  </si>
+  <si>
+    <t>".replace(r"\s+", "", regex=True)=&gt; explain in detail, why  not regex=False?"</t>
+  </si>
+  <si>
+    <t>"# 2) Delete only this batch from facts, then insert batch facts cur.execute("DELETE FROM clean.fact_sales WHERE batch_id = ?;", (batch_id,)) =&gt; question is: everytime run ETL it create a unique batch. If so, is this delete really needed? I think it will only need when peforming CRUD"</t>
+  </si>
+  <si>
+    <t>27. Klipfolio, Average Profit Margin Metric</t>
+  </si>
+  <si>
+    <t>https://www.klipfolio.com/resources/kpi-examples/sales/average-profit-margin</t>
   </si>
 </sst>
 </file>
@@ -1603,7 +1630,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1755,6 +1782,27 @@
     <xf numFmtId="14" fontId="0" fillId="2" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -1773,6 +1821,30 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="14" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -1782,30 +1854,6 @@
     <xf numFmtId="14" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="15" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="15" fontId="7" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="15" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="15" fontId="7" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1821,25 +1869,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3765,10 +3795,10 @@
       </c>
     </row>
     <row r="3" spans="2:4" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="82">
+      <c r="B3" s="81">
         <v>45683</v>
       </c>
-      <c r="C3" s="83">
+      <c r="C3" s="80">
         <v>2</v>
       </c>
       <c r="D3" s="34" t="s">
@@ -3776,31 +3806,31 @@
       </c>
     </row>
     <row r="4" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="82"/>
-      <c r="C4" s="83"/>
+      <c r="B4" s="81"/>
+      <c r="C4" s="80"/>
       <c r="D4" s="34" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="82"/>
-      <c r="C5" s="83"/>
+      <c r="B5" s="81"/>
+      <c r="C5" s="80"/>
       <c r="D5" s="40" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="82"/>
-      <c r="C6" s="83"/>
+      <c r="B6" s="81"/>
+      <c r="C6" s="80"/>
       <c r="D6" s="41" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="7" spans="2:4" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="82">
+      <c r="B7" s="81">
         <v>45684</v>
       </c>
-      <c r="C7" s="83">
+      <c r="C7" s="80">
         <v>1.5</v>
       </c>
       <c r="D7" s="35" t="s">
@@ -3808,31 +3838,31 @@
       </c>
     </row>
     <row r="8" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="82"/>
-      <c r="C8" s="83"/>
+      <c r="B8" s="81"/>
+      <c r="C8" s="80"/>
       <c r="D8" s="36" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="9" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="82"/>
-      <c r="C9" s="83"/>
+      <c r="B9" s="81"/>
+      <c r="C9" s="80"/>
       <c r="D9" s="42" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="10" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="82"/>
-      <c r="C10" s="83"/>
+      <c r="B10" s="81"/>
+      <c r="C10" s="80"/>
       <c r="D10" s="43" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="82">
+      <c r="B11" s="81">
         <v>45686</v>
       </c>
-      <c r="C11" s="83">
+      <c r="C11" s="80">
         <v>3</v>
       </c>
       <c r="D11" s="34" t="s">
@@ -3840,38 +3870,38 @@
       </c>
     </row>
     <row r="12" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="82"/>
-      <c r="C12" s="83"/>
+      <c r="B12" s="81"/>
+      <c r="C12" s="80"/>
       <c r="D12" s="34" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="82"/>
-      <c r="C13" s="83"/>
+      <c r="B13" s="81"/>
+      <c r="C13" s="80"/>
       <c r="D13" s="34" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="82"/>
-      <c r="C14" s="83"/>
+      <c r="B14" s="81"/>
+      <c r="C14" s="80"/>
       <c r="D14" s="44" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="82"/>
-      <c r="C15" s="83"/>
+      <c r="B15" s="81"/>
+      <c r="C15" s="80"/>
       <c r="D15" s="41" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="82">
+      <c r="B16" s="81">
         <v>46053</v>
       </c>
-      <c r="C16" s="83">
+      <c r="C16" s="80">
         <v>4</v>
       </c>
       <c r="D16" s="37" t="s">
@@ -3879,80 +3909,80 @@
       </c>
     </row>
     <row r="17" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="82"/>
-      <c r="C17" s="83"/>
+      <c r="B17" s="81"/>
+      <c r="C17" s="80"/>
       <c r="D17" s="34" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="82"/>
-      <c r="C18" s="83"/>
+      <c r="B18" s="81"/>
+      <c r="C18" s="80"/>
       <c r="D18" s="34" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="19" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="82"/>
-      <c r="C19" s="83"/>
+      <c r="B19" s="81"/>
+      <c r="C19" s="80"/>
       <c r="D19" s="34" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="20" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="82"/>
-      <c r="C20" s="83"/>
+      <c r="B20" s="81"/>
+      <c r="C20" s="80"/>
       <c r="D20" s="34" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="21" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="82"/>
-      <c r="C21" s="83"/>
+      <c r="B21" s="81"/>
+      <c r="C21" s="80"/>
       <c r="D21" s="34" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="82"/>
-      <c r="C22" s="83"/>
+      <c r="B22" s="81"/>
+      <c r="C22" s="80"/>
       <c r="D22" s="44" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="23" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="82"/>
-      <c r="C23" s="83"/>
+      <c r="B23" s="81"/>
+      <c r="C23" s="80"/>
       <c r="D23" s="40" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="24" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="82"/>
-      <c r="C24" s="83"/>
+      <c r="B24" s="81"/>
+      <c r="C24" s="80"/>
       <c r="D24" s="40" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="25" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="82"/>
-      <c r="C25" s="83"/>
+      <c r="B25" s="81"/>
+      <c r="C25" s="80"/>
       <c r="D25" s="40" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="26" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="82"/>
-      <c r="C26" s="83"/>
+      <c r="B26" s="81"/>
+      <c r="C26" s="80"/>
       <c r="D26" s="45" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="27" spans="2:4" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="82">
+      <c r="B27" s="81">
         <v>46054</v>
       </c>
-      <c r="C27" s="83">
+      <c r="C27" s="80">
         <v>1</v>
       </c>
       <c r="D27" s="34" t="s">
@@ -3960,31 +3990,31 @@
       </c>
     </row>
     <row r="28" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="82"/>
-      <c r="C28" s="83"/>
+      <c r="B28" s="81"/>
+      <c r="C28" s="80"/>
       <c r="D28" s="34" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="29" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="82"/>
-      <c r="C29" s="83"/>
+      <c r="B29" s="81"/>
+      <c r="C29" s="80"/>
       <c r="D29" s="40" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="30" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="82"/>
-      <c r="C30" s="83"/>
+      <c r="B30" s="81"/>
+      <c r="C30" s="80"/>
       <c r="D30" s="41" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="31" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B31" s="82">
+      <c r="B31" s="81">
         <v>46055</v>
       </c>
-      <c r="C31" s="83">
+      <c r="C31" s="80">
         <v>4</v>
       </c>
       <c r="D31" s="38" t="s">
@@ -3992,45 +4022,45 @@
       </c>
     </row>
     <row r="32" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B32" s="82"/>
-      <c r="C32" s="83"/>
+      <c r="B32" s="81"/>
+      <c r="C32" s="80"/>
       <c r="D32" s="39" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="33" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="82"/>
-      <c r="C33" s="83"/>
+      <c r="B33" s="81"/>
+      <c r="C33" s="80"/>
       <c r="D33" s="39" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="34" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B34" s="82"/>
-      <c r="C34" s="83"/>
+      <c r="B34" s="81"/>
+      <c r="C34" s="80"/>
       <c r="D34" s="39" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="35" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B35" s="82"/>
-      <c r="C35" s="83"/>
+      <c r="B35" s="81"/>
+      <c r="C35" s="80"/>
       <c r="D35" s="46" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="36" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B36" s="82"/>
-      <c r="C36" s="83"/>
+      <c r="B36" s="81"/>
+      <c r="C36" s="80"/>
       <c r="D36" s="47" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="37" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="82">
+      <c r="B37" s="81">
         <v>46056</v>
       </c>
-      <c r="C37" s="83">
+      <c r="C37" s="80">
         <v>3</v>
       </c>
       <c r="D37" s="34" t="s">
@@ -4038,38 +4068,38 @@
       </c>
     </row>
     <row r="38" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B38" s="82"/>
-      <c r="C38" s="83"/>
+      <c r="B38" s="81"/>
+      <c r="C38" s="80"/>
       <c r="D38" s="34" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="39" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B39" s="82"/>
-      <c r="C39" s="83"/>
+      <c r="B39" s="81"/>
+      <c r="C39" s="80"/>
       <c r="D39" s="34" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="40" spans="2:4" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B40" s="82"/>
-      <c r="C40" s="83"/>
+      <c r="B40" s="81"/>
+      <c r="C40" s="80"/>
       <c r="D40" s="40" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="41" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B41" s="82"/>
-      <c r="C41" s="83"/>
+      <c r="B41" s="81"/>
+      <c r="C41" s="80"/>
       <c r="D41" s="41" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="42" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B42" s="82">
+      <c r="B42" s="81">
         <v>46057</v>
       </c>
-      <c r="C42" s="83">
+      <c r="C42" s="80">
         <v>4</v>
       </c>
       <c r="D42" s="37" t="s">
@@ -4077,24 +4107,24 @@
       </c>
     </row>
     <row r="43" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B43" s="82"/>
-      <c r="C43" s="83"/>
+      <c r="B43" s="81"/>
+      <c r="C43" s="80"/>
       <c r="D43" s="34" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="44" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B44" s="82"/>
-      <c r="C44" s="83"/>
+      <c r="B44" s="81"/>
+      <c r="C44" s="80"/>
       <c r="D44" s="41" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="45" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B45" s="79">
+      <c r="B45" s="82">
         <v>46059</v>
       </c>
-      <c r="C45" s="76">
+      <c r="C45" s="85">
         <v>2</v>
       </c>
       <c r="D45" s="49" t="s">
@@ -4102,38 +4132,38 @@
       </c>
     </row>
     <row r="46" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B46" s="80"/>
-      <c r="C46" s="77"/>
+      <c r="B46" s="83"/>
+      <c r="C46" s="86"/>
       <c r="D46" s="48" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="47" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B47" s="80"/>
-      <c r="C47" s="77"/>
+      <c r="B47" s="83"/>
+      <c r="C47" s="86"/>
       <c r="D47" s="34" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="48" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B48" s="80"/>
-      <c r="C48" s="77"/>
+      <c r="B48" s="83"/>
+      <c r="C48" s="86"/>
       <c r="D48" s="41" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="49" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B49" s="81"/>
-      <c r="C49" s="78"/>
+      <c r="B49" s="84"/>
+      <c r="C49" s="87"/>
       <c r="D49" s="45" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="50" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B50" s="79">
+      <c r="B50" s="82">
         <v>46061</v>
       </c>
-      <c r="C50" s="76">
+      <c r="C50" s="85">
         <v>1.5</v>
       </c>
       <c r="D50" s="49" t="s">
@@ -4141,38 +4171,38 @@
       </c>
     </row>
     <row r="51" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B51" s="80"/>
-      <c r="C51" s="77"/>
+      <c r="B51" s="83"/>
+      <c r="C51" s="86"/>
       <c r="D51" s="34" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="52" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B52" s="80"/>
-      <c r="C52" s="77"/>
+      <c r="B52" s="83"/>
+      <c r="C52" s="86"/>
       <c r="D52" s="41" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="53" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B53" s="80"/>
-      <c r="C53" s="77"/>
+      <c r="B53" s="83"/>
+      <c r="C53" s="86"/>
       <c r="D53" s="41" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="54" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B54" s="81"/>
-      <c r="C54" s="78"/>
+      <c r="B54" s="84"/>
+      <c r="C54" s="87"/>
       <c r="D54" s="45" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="55" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="79">
+      <c r="B55" s="82">
         <v>46062</v>
       </c>
-      <c r="C55" s="76">
+      <c r="C55" s="85">
         <v>2</v>
       </c>
       <c r="D55" s="52" t="s">
@@ -4180,31 +4210,31 @@
       </c>
     </row>
     <row r="56" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B56" s="80"/>
-      <c r="C56" s="77"/>
+      <c r="B56" s="83"/>
+      <c r="C56" s="86"/>
       <c r="D56" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="57" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B57" s="80"/>
-      <c r="C57" s="77"/>
+      <c r="B57" s="83"/>
+      <c r="C57" s="86"/>
       <c r="D57" s="41" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="58" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B58" s="81"/>
-      <c r="C58" s="78"/>
+      <c r="B58" s="84"/>
+      <c r="C58" s="87"/>
       <c r="D58" s="45" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="59" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="79">
+      <c r="B59" s="82">
         <v>46063</v>
       </c>
-      <c r="C59" s="76">
+      <c r="C59" s="85">
         <v>3</v>
       </c>
       <c r="D59" s="52" t="s">
@@ -4212,38 +4242,38 @@
       </c>
     </row>
     <row r="60" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B60" s="80"/>
-      <c r="C60" s="77"/>
+      <c r="B60" s="83"/>
+      <c r="C60" s="86"/>
       <c r="D60" s="53" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="61" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B61" s="80"/>
-      <c r="C61" s="77"/>
+      <c r="B61" s="83"/>
+      <c r="C61" s="86"/>
       <c r="D61" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="62" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B62" s="80"/>
-      <c r="C62" s="77"/>
+      <c r="B62" s="83"/>
+      <c r="C62" s="86"/>
       <c r="D62" s="41" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="63" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B63" s="81"/>
-      <c r="C63" s="78"/>
+      <c r="B63" s="84"/>
+      <c r="C63" s="87"/>
       <c r="D63" s="45" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="64" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B64" s="79">
+      <c r="B64" s="82">
         <v>46064</v>
       </c>
-      <c r="C64" s="76">
+      <c r="C64" s="85">
         <v>3</v>
       </c>
       <c r="D64" s="52" t="s">
@@ -4251,38 +4281,38 @@
       </c>
     </row>
     <row r="65" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B65" s="80"/>
-      <c r="C65" s="77"/>
+      <c r="B65" s="83"/>
+      <c r="C65" s="86"/>
       <c r="D65" s="53" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="66" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B66" s="80"/>
-      <c r="C66" s="77"/>
+      <c r="B66" s="83"/>
+      <c r="C66" s="86"/>
       <c r="D66" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="67" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B67" s="80"/>
-      <c r="C67" s="77"/>
+      <c r="B67" s="83"/>
+      <c r="C67" s="86"/>
       <c r="D67" s="41" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="68" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B68" s="81"/>
-      <c r="C68" s="78"/>
+      <c r="B68" s="84"/>
+      <c r="C68" s="87"/>
       <c r="D68" s="45" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="69" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B69" s="73">
+      <c r="B69" s="88">
         <v>46066</v>
       </c>
-      <c r="C69" s="76">
+      <c r="C69" s="85">
         <v>2</v>
       </c>
       <c r="D69" s="52" t="s">
@@ -4290,45 +4320,45 @@
       </c>
     </row>
     <row r="70" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B70" s="74"/>
-      <c r="C70" s="77"/>
+      <c r="B70" s="89"/>
+      <c r="C70" s="86"/>
       <c r="D70" s="53" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="71" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B71" s="74"/>
-      <c r="C71" s="77"/>
+      <c r="B71" s="89"/>
+      <c r="C71" s="86"/>
       <c r="D71" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="72" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B72" s="74"/>
-      <c r="C72" s="77"/>
+      <c r="B72" s="89"/>
+      <c r="C72" s="86"/>
       <c r="D72" s="41" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="73" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B73" s="74"/>
-      <c r="C73" s="77"/>
+      <c r="B73" s="89"/>
+      <c r="C73" s="86"/>
       <c r="D73" s="41" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="74" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B74" s="75"/>
-      <c r="C74" s="78"/>
+      <c r="B74" s="90"/>
+      <c r="C74" s="87"/>
       <c r="D74" s="45" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="75" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B75" s="67">
+      <c r="B75" s="74">
         <v>46068</v>
       </c>
-      <c r="C75" s="70">
+      <c r="C75" s="77">
         <v>2.5</v>
       </c>
       <c r="D75" s="52" t="s">
@@ -4336,52 +4366,52 @@
       </c>
     </row>
     <row r="76" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B76" s="68"/>
-      <c r="C76" s="71"/>
+      <c r="B76" s="75"/>
+      <c r="C76" s="78"/>
       <c r="D76" s="53" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="77" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B77" s="68"/>
-      <c r="C77" s="71"/>
+      <c r="B77" s="75"/>
+      <c r="C77" s="78"/>
       <c r="D77" s="53" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="78" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B78" s="68"/>
-      <c r="C78" s="71"/>
+      <c r="B78" s="75"/>
+      <c r="C78" s="78"/>
       <c r="D78" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="79" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B79" s="68"/>
-      <c r="C79" s="71"/>
+      <c r="B79" s="75"/>
+      <c r="C79" s="78"/>
       <c r="D79" s="41" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="80" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B80" s="68"/>
-      <c r="C80" s="71"/>
+      <c r="B80" s="75"/>
+      <c r="C80" s="78"/>
       <c r="D80" s="41" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="81" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B81" s="69"/>
-      <c r="C81" s="72"/>
+      <c r="B81" s="76"/>
+      <c r="C81" s="79"/>
       <c r="D81" s="45" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="82" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B82" s="67">
+      <c r="B82" s="74">
         <v>46070</v>
       </c>
-      <c r="C82" s="70">
+      <c r="C82" s="77">
         <v>3</v>
       </c>
       <c r="D82" s="52" t="s">
@@ -4389,52 +4419,52 @@
       </c>
     </row>
     <row r="83" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B83" s="68"/>
-      <c r="C83" s="71"/>
+      <c r="B83" s="75"/>
+      <c r="C83" s="78"/>
       <c r="D83" s="53" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="84" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B84" s="68"/>
-      <c r="C84" s="71"/>
+      <c r="B84" s="75"/>
+      <c r="C84" s="78"/>
       <c r="D84" s="53" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="85" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B85" s="68"/>
-      <c r="C85" s="71"/>
+      <c r="B85" s="75"/>
+      <c r="C85" s="78"/>
       <c r="D85" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="86" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B86" s="68"/>
-      <c r="C86" s="71"/>
+      <c r="B86" s="75"/>
+      <c r="C86" s="78"/>
       <c r="D86" s="41" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="87" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B87" s="68"/>
-      <c r="C87" s="71"/>
+      <c r="B87" s="75"/>
+      <c r="C87" s="78"/>
       <c r="D87" s="41" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="88" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B88" s="69"/>
-      <c r="C88" s="72"/>
+      <c r="B88" s="76"/>
+      <c r="C88" s="79"/>
       <c r="D88" s="45" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="89" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B89" s="67">
+      <c r="B89" s="74">
         <v>46071</v>
       </c>
-      <c r="C89" s="70">
+      <c r="C89" s="77">
         <v>2</v>
       </c>
       <c r="D89" s="52" t="s">
@@ -4442,38 +4472,38 @@
       </c>
     </row>
     <row r="90" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B90" s="68"/>
-      <c r="C90" s="71"/>
+      <c r="B90" s="75"/>
+      <c r="C90" s="78"/>
       <c r="D90" s="53" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="91" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B91" s="68"/>
-      <c r="C91" s="71"/>
+      <c r="B91" s="75"/>
+      <c r="C91" s="78"/>
       <c r="D91" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="92" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B92" s="68"/>
-      <c r="C92" s="71"/>
+      <c r="B92" s="75"/>
+      <c r="C92" s="78"/>
       <c r="D92" s="41" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="93" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B93" s="69"/>
-      <c r="C93" s="72"/>
+      <c r="B93" s="76"/>
+      <c r="C93" s="79"/>
       <c r="D93" s="45" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="94" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B94" s="67">
+      <c r="B94" s="74">
         <v>46074</v>
       </c>
-      <c r="C94" s="70">
+      <c r="C94" s="77">
         <v>3</v>
       </c>
       <c r="D94" s="55" t="s">
@@ -4481,24 +4511,24 @@
       </c>
     </row>
     <row r="95" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B95" s="68"/>
-      <c r="C95" s="71"/>
+      <c r="B95" s="75"/>
+      <c r="C95" s="78"/>
       <c r="D95" s="56" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="96" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B96" s="69"/>
-      <c r="C96" s="72"/>
+      <c r="B96" s="76"/>
+      <c r="C96" s="79"/>
       <c r="D96" s="45" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="97" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B97" s="67">
+      <c r="B97" s="74">
         <v>46075</v>
       </c>
-      <c r="C97" s="70">
+      <c r="C97" s="77">
         <v>3</v>
       </c>
       <c r="D97" s="52" t="s">
@@ -4506,22 +4536,22 @@
       </c>
     </row>
     <row r="98" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B98" s="68"/>
-      <c r="C98" s="71"/>
+      <c r="B98" s="75"/>
+      <c r="C98" s="78"/>
       <c r="D98" s="53" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="99" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B99" s="68"/>
-      <c r="C99" s="71"/>
+      <c r="B99" s="75"/>
+      <c r="C99" s="78"/>
       <c r="D99" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="100" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B100" s="69"/>
-      <c r="C100" s="72"/>
+      <c r="B100" s="76"/>
+      <c r="C100" s="79"/>
       <c r="D100" s="45" t="s">
         <v>23</v>
       </c>
@@ -4538,10 +4568,10 @@
       </c>
     </row>
     <row r="102" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B102" s="67">
+      <c r="B102" s="74">
         <v>46077</v>
       </c>
-      <c r="C102" s="70">
+      <c r="C102" s="77">
         <v>2</v>
       </c>
       <c r="D102" s="52" t="s">
@@ -4549,38 +4579,38 @@
       </c>
     </row>
     <row r="103" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B103" s="68"/>
-      <c r="C103" s="71"/>
+      <c r="B103" s="75"/>
+      <c r="C103" s="78"/>
       <c r="D103" s="53" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="104" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B104" s="68"/>
-      <c r="C104" s="71"/>
+      <c r="B104" s="75"/>
+      <c r="C104" s="78"/>
       <c r="D104" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="105" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B105" s="68"/>
-      <c r="C105" s="71"/>
+      <c r="B105" s="75"/>
+      <c r="C105" s="78"/>
       <c r="D105" s="41" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="106" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B106" s="69"/>
-      <c r="C106" s="72"/>
+      <c r="B106" s="76"/>
+      <c r="C106" s="79"/>
       <c r="D106" s="45" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="107" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B107" s="67">
+      <c r="B107" s="74">
         <v>46078</v>
       </c>
-      <c r="C107" s="70">
+      <c r="C107" s="77">
         <v>1</v>
       </c>
       <c r="D107" s="63" t="s">
@@ -4588,38 +4618,38 @@
       </c>
     </row>
     <row r="108" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B108" s="68"/>
-      <c r="C108" s="71"/>
+      <c r="B108" s="75"/>
+      <c r="C108" s="78"/>
       <c r="D108" s="53" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="109" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B109" s="68"/>
-      <c r="C109" s="71"/>
+      <c r="B109" s="75"/>
+      <c r="C109" s="78"/>
       <c r="D109" s="41" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="110" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B110" s="68"/>
-      <c r="C110" s="71"/>
+      <c r="B110" s="75"/>
+      <c r="C110" s="78"/>
       <c r="D110" s="41" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="111" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B111" s="69"/>
-      <c r="C111" s="72"/>
+      <c r="B111" s="76"/>
+      <c r="C111" s="79"/>
       <c r="D111" s="64" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="112" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B112" s="67">
+      <c r="B112" s="74">
         <v>46079</v>
       </c>
-      <c r="C112" s="70">
+      <c r="C112" s="77">
         <v>2</v>
       </c>
       <c r="D112" s="63" t="s">
@@ -4627,31 +4657,31 @@
       </c>
     </row>
     <row r="113" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B113" s="68"/>
-      <c r="C113" s="71"/>
+      <c r="B113" s="75"/>
+      <c r="C113" s="78"/>
       <c r="D113" s="53" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="114" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B114" s="68"/>
-      <c r="C114" s="71"/>
+      <c r="B114" s="75"/>
+      <c r="C114" s="78"/>
       <c r="D114" s="41" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="115" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B115" s="69"/>
-      <c r="C115" s="72"/>
+      <c r="B115" s="76"/>
+      <c r="C115" s="79"/>
       <c r="D115" s="45" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="116" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B116" s="67">
+      <c r="B116" s="74">
         <v>46083</v>
       </c>
-      <c r="C116" s="70">
+      <c r="C116" s="77">
         <v>3</v>
       </c>
       <c r="D116" s="63" t="s">
@@ -4659,31 +4689,31 @@
       </c>
     </row>
     <row r="117" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B117" s="68"/>
-      <c r="C117" s="71"/>
+      <c r="B117" s="75"/>
+      <c r="C117" s="78"/>
       <c r="D117" s="53" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="118" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B118" s="68"/>
-      <c r="C118" s="71"/>
+      <c r="B118" s="75"/>
+      <c r="C118" s="78"/>
       <c r="D118" s="53" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="119" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B119" s="69"/>
-      <c r="C119" s="72"/>
+      <c r="B119" s="76"/>
+      <c r="C119" s="79"/>
       <c r="D119" s="45" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="120" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B120" s="67">
+      <c r="B120" s="74">
         <v>411326</v>
       </c>
-      <c r="C120" s="70">
+      <c r="C120" s="77">
         <v>5</v>
       </c>
       <c r="D120" s="63" t="s">
@@ -4691,24 +4721,24 @@
       </c>
     </row>
     <row r="121" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B121" s="68"/>
-      <c r="C121" s="71"/>
+      <c r="B121" s="75"/>
+      <c r="C121" s="78"/>
       <c r="D121" s="53" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="122" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B122" s="69"/>
-      <c r="C122" s="72"/>
+      <c r="B122" s="76"/>
+      <c r="C122" s="79"/>
       <c r="D122" s="65" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="123" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B123" s="89">
+      <c r="B123" s="68">
         <v>46085</v>
       </c>
-      <c r="C123" s="90">
+      <c r="C123" s="71">
         <v>4</v>
       </c>
       <c r="D123" s="63" t="s">
@@ -4716,38 +4746,38 @@
       </c>
     </row>
     <row r="124" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B124" s="91"/>
-      <c r="C124" s="92"/>
+      <c r="B124" s="69"/>
+      <c r="C124" s="72"/>
       <c r="D124" s="53" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="125" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B125" s="91"/>
-      <c r="C125" s="92"/>
+      <c r="B125" s="69"/>
+      <c r="C125" s="72"/>
       <c r="D125" s="53" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="126" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B126" s="91"/>
-      <c r="C126" s="92"/>
+      <c r="B126" s="69"/>
+      <c r="C126" s="72"/>
       <c r="D126" s="41" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="127" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B127" s="93"/>
-      <c r="C127" s="94"/>
+      <c r="B127" s="70"/>
+      <c r="C127" s="73"/>
       <c r="D127" s="45" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="128" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B128" s="66">
+      <c r="B128" s="74">
         <v>46086</v>
       </c>
-      <c r="C128" s="54">
+      <c r="C128" s="77">
         <v>6</v>
       </c>
       <c r="D128" s="63" t="s">
@@ -4755,263 +4785,321 @@
       </c>
     </row>
     <row r="129" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B129" s="66"/>
-      <c r="C129" s="54"/>
+      <c r="B129" s="75"/>
+      <c r="C129" s="78"/>
       <c r="D129" s="53" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="130" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B130" s="54"/>
-      <c r="C130" s="54"/>
+      <c r="B130" s="75"/>
+      <c r="C130" s="78"/>
       <c r="D130" s="53" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="131" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B131" s="54"/>
-      <c r="C131" s="54"/>
-      <c r="D131" s="95" t="s">
+      <c r="B131" s="75"/>
+      <c r="C131" s="78"/>
+      <c r="D131" s="67" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="132" spans="2:4" ht="78" x14ac:dyDescent="0.3">
-      <c r="B132" s="32"/>
-      <c r="C132" s="32"/>
-      <c r="D132" s="95" t="s">
+      <c r="B132" s="75"/>
+      <c r="C132" s="78"/>
+      <c r="D132" s="67" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="133" spans="2:4" ht="78" x14ac:dyDescent="0.3">
-      <c r="B133" s="32"/>
-      <c r="C133" s="32"/>
-      <c r="D133" s="95" t="s">
+      <c r="B133" s="75"/>
+      <c r="C133" s="78"/>
+      <c r="D133" s="67" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="134" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B134" s="54"/>
-      <c r="C134" s="54"/>
-      <c r="D134" s="95" t="s">
+      <c r="B134" s="75"/>
+      <c r="C134" s="78"/>
+      <c r="D134" s="67" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="135" spans="2:4" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B135" s="32"/>
-      <c r="C135" s="32"/>
-      <c r="D135" s="95" t="s">
+      <c r="B135" s="75"/>
+      <c r="C135" s="78"/>
+      <c r="D135" s="67" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="136" spans="2:4" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="B136" s="32"/>
-      <c r="C136" s="32"/>
-      <c r="D136" s="95" t="s">
+      <c r="B136" s="75"/>
+      <c r="C136" s="78"/>
+      <c r="D136" s="67" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="137" spans="2:4" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B137" s="54"/>
-      <c r="C137"/>
-      <c r="D137" s="95" t="s">
+      <c r="B137" s="75"/>
+      <c r="C137" s="78"/>
+      <c r="D137" s="67" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="138" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B138" s="32"/>
-      <c r="C138"/>
-      <c r="D138" s="95" t="s">
+      <c r="B138" s="75"/>
+      <c r="C138" s="78"/>
+      <c r="D138" s="67" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="139" spans="2:4" ht="78" x14ac:dyDescent="0.3">
-      <c r="B139" s="32"/>
-      <c r="C139" s="32"/>
-      <c r="D139" s="95" t="s">
+      <c r="B139" s="75"/>
+      <c r="C139" s="78"/>
+      <c r="D139" s="67" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="140" spans="2:4" ht="78" x14ac:dyDescent="0.3">
-      <c r="B140" s="54"/>
-      <c r="C140" s="54"/>
-      <c r="D140" s="95" t="s">
+      <c r="B140" s="75"/>
+      <c r="C140" s="78"/>
+      <c r="D140" s="67" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="141" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B141" s="32"/>
-      <c r="C141" s="32"/>
-      <c r="D141" s="95" t="s">
+      <c r="B141" s="75"/>
+      <c r="C141" s="78"/>
+      <c r="D141" s="67" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="142" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B142" s="32"/>
-      <c r="C142" s="32"/>
-      <c r="D142" s="95" t="s">
+    <row r="142" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B142" s="76"/>
+      <c r="C142" s="79"/>
+      <c r="D142" s="96" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="143" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B143" s="32"/>
-      <c r="C143" s="32"/>
-      <c r="D143" s="95"/>
-    </row>
-    <row r="144" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="143" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B143" s="66">
+        <v>46087</v>
+      </c>
+      <c r="C143" s="54">
+        <v>4</v>
+      </c>
+      <c r="D143" s="63" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="144" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B144" s="32"/>
       <c r="C144" s="32"/>
-      <c r="D144" s="95"/>
-    </row>
-    <row r="145" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D144" s="53" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="145" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B145" s="32"/>
       <c r="C145" s="32"/>
-      <c r="D145" s="95"/>
-    </row>
-    <row r="146" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D145" s="53" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="146" spans="2:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="B146" s="32"/>
       <c r="C146" s="32"/>
-      <c r="D146" s="95"/>
-    </row>
-    <row r="147" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D146" s="67" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="147" spans="2:4" ht="46.8" x14ac:dyDescent="0.3">
       <c r="B147" s="32"/>
       <c r="C147" s="32"/>
-      <c r="D147" s="95"/>
+      <c r="D147" s="67" t="s">
+        <v>181</v>
+      </c>
     </row>
     <row r="148" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B148" s="32"/>
       <c r="C148" s="32"/>
-      <c r="D148" s="95"/>
+      <c r="D148" s="67" t="s">
+        <v>180</v>
+      </c>
     </row>
     <row r="149" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B149" s="32"/>
       <c r="C149" s="32"/>
-      <c r="D149" s="95"/>
+      <c r="D149" s="67" t="s">
+        <v>179</v>
+      </c>
     </row>
     <row r="150" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B150" s="32"/>
       <c r="C150" s="32"/>
-      <c r="D150" s="95"/>
-    </row>
-    <row r="151" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D150" s="67" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="151" spans="2:4" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B151" s="32"/>
       <c r="C151" s="32"/>
-      <c r="D151" s="95"/>
+      <c r="D151" s="67" t="s">
+        <v>178</v>
+      </c>
     </row>
     <row r="152" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B152" s="32"/>
       <c r="C152" s="32"/>
-      <c r="D152" s="95"/>
+      <c r="D152" s="67"/>
     </row>
     <row r="153" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B153" s="32"/>
       <c r="C153" s="32"/>
-      <c r="D153" s="95"/>
+      <c r="D153" s="67"/>
     </row>
     <row r="154" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B154" s="32"/>
       <c r="C154" s="32"/>
-      <c r="D154" s="95"/>
+      <c r="D154" s="67"/>
     </row>
     <row r="155" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B155" s="32"/>
       <c r="C155" s="32"/>
-      <c r="D155" s="95"/>
+      <c r="D155" s="67"/>
     </row>
     <row r="156" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B156" s="32"/>
       <c r="C156" s="32"/>
-      <c r="D156" s="95"/>
+      <c r="D156" s="67"/>
     </row>
     <row r="157" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B157" s="32"/>
       <c r="C157" s="32"/>
-      <c r="D157" s="95"/>
+      <c r="D157" s="67"/>
     </row>
     <row r="158" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B158" s="32"/>
       <c r="C158" s="32"/>
-      <c r="D158" s="95"/>
+      <c r="D158" s="67"/>
     </row>
     <row r="159" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B159" s="32"/>
       <c r="C159" s="32"/>
-      <c r="D159" s="95"/>
+      <c r="D159" s="67"/>
     </row>
     <row r="160" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B160" s="32"/>
       <c r="C160" s="32"/>
-      <c r="D160" s="95"/>
+      <c r="D160" s="67"/>
     </row>
     <row r="161" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B161" s="32"/>
       <c r="C161" s="32"/>
-      <c r="D161" s="95"/>
+      <c r="D161" s="67"/>
     </row>
     <row r="162" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B162" s="32"/>
       <c r="C162" s="32"/>
-      <c r="D162" s="95"/>
+      <c r="D162" s="67"/>
     </row>
     <row r="163" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B163" s="32"/>
       <c r="C163" s="32"/>
-      <c r="D163" s="95"/>
+      <c r="D163" s="67"/>
     </row>
     <row r="164" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B164" s="32"/>
       <c r="C164" s="32"/>
-      <c r="D164" s="95"/>
+      <c r="D164" s="67"/>
     </row>
     <row r="165" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B165" s="32"/>
       <c r="C165" s="32"/>
-      <c r="D165" s="95"/>
+      <c r="D165" s="67"/>
     </row>
     <row r="166" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B166" s="32"/>
       <c r="C166" s="32"/>
-      <c r="D166" s="95"/>
+      <c r="D166" s="67"/>
     </row>
     <row r="167" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B167" s="32"/>
       <c r="C167" s="32"/>
-      <c r="D167" s="95"/>
+      <c r="D167" s="67"/>
     </row>
     <row r="168" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B168" s="32"/>
       <c r="C168" s="32"/>
-      <c r="D168" s="95"/>
+      <c r="D168" s="67"/>
     </row>
     <row r="169" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B169" s="32"/>
       <c r="C169" s="32"/>
-      <c r="D169" s="95"/>
+      <c r="D169" s="67"/>
     </row>
     <row r="170" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B170" s="32"/>
       <c r="C170" s="32"/>
-      <c r="D170" s="95"/>
+      <c r="D170" s="67"/>
     </row>
     <row r="171" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B171" s="32"/>
       <c r="C171" s="32"/>
-      <c r="D171" s="95"/>
+      <c r="D171" s="67"/>
     </row>
     <row r="172" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B172" s="32"/>
       <c r="C172" s="32"/>
-      <c r="D172" s="95"/>
+      <c r="D172" s="67"/>
     </row>
     <row r="173" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B173" s="32"/>
       <c r="C173" s="32"/>
-      <c r="D173" s="95"/>
+      <c r="D173" s="67"/>
     </row>
     <row r="174" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="D174" s="95"/>
+      <c r="D174" s="67"/>
     </row>
   </sheetData>
-  <mergeCells count="50">
+  <mergeCells count="52">
+    <mergeCell ref="B128:B142"/>
+    <mergeCell ref="C128:C142"/>
+    <mergeCell ref="B120:B122"/>
+    <mergeCell ref="C120:C122"/>
+    <mergeCell ref="B112:B115"/>
+    <mergeCell ref="C112:C115"/>
+    <mergeCell ref="B116:B119"/>
+    <mergeCell ref="C116:C119"/>
+    <mergeCell ref="B102:B106"/>
+    <mergeCell ref="C102:C106"/>
+    <mergeCell ref="B97:B100"/>
+    <mergeCell ref="C97:C100"/>
+    <mergeCell ref="B82:B88"/>
+    <mergeCell ref="C82:C88"/>
+    <mergeCell ref="B89:B93"/>
+    <mergeCell ref="C89:C93"/>
+    <mergeCell ref="B94:B96"/>
+    <mergeCell ref="C94:C96"/>
+    <mergeCell ref="B64:B68"/>
+    <mergeCell ref="C64:C68"/>
+    <mergeCell ref="B69:B74"/>
+    <mergeCell ref="C69:C74"/>
+    <mergeCell ref="B75:B81"/>
+    <mergeCell ref="C75:C81"/>
+    <mergeCell ref="B59:B63"/>
+    <mergeCell ref="C59:C63"/>
+    <mergeCell ref="B3:B6"/>
+    <mergeCell ref="C3:C6"/>
+    <mergeCell ref="B7:B10"/>
+    <mergeCell ref="C7:C10"/>
+    <mergeCell ref="B11:B15"/>
+    <mergeCell ref="C11:C15"/>
+    <mergeCell ref="B45:B49"/>
+    <mergeCell ref="C45:C49"/>
+    <mergeCell ref="B50:B54"/>
+    <mergeCell ref="C50:C54"/>
     <mergeCell ref="B123:B127"/>
     <mergeCell ref="C123:C127"/>
     <mergeCell ref="B107:B111"/>
@@ -5028,40 +5116,6 @@
     <mergeCell ref="C42:C44"/>
     <mergeCell ref="B55:B58"/>
     <mergeCell ref="C55:C58"/>
-    <mergeCell ref="B59:B63"/>
-    <mergeCell ref="C59:C63"/>
-    <mergeCell ref="B3:B6"/>
-    <mergeCell ref="C3:C6"/>
-    <mergeCell ref="B7:B10"/>
-    <mergeCell ref="C7:C10"/>
-    <mergeCell ref="B11:B15"/>
-    <mergeCell ref="C11:C15"/>
-    <mergeCell ref="B45:B49"/>
-    <mergeCell ref="C45:C49"/>
-    <mergeCell ref="B50:B54"/>
-    <mergeCell ref="C50:C54"/>
-    <mergeCell ref="B64:B68"/>
-    <mergeCell ref="C64:C68"/>
-    <mergeCell ref="B69:B74"/>
-    <mergeCell ref="C69:C74"/>
-    <mergeCell ref="B75:B81"/>
-    <mergeCell ref="C75:C81"/>
-    <mergeCell ref="B102:B106"/>
-    <mergeCell ref="C102:C106"/>
-    <mergeCell ref="B97:B100"/>
-    <mergeCell ref="C97:C100"/>
-    <mergeCell ref="B82:B88"/>
-    <mergeCell ref="C82:C88"/>
-    <mergeCell ref="B89:B93"/>
-    <mergeCell ref="C89:C93"/>
-    <mergeCell ref="B94:B96"/>
-    <mergeCell ref="C94:C96"/>
-    <mergeCell ref="B120:B122"/>
-    <mergeCell ref="C120:C122"/>
-    <mergeCell ref="B112:B115"/>
-    <mergeCell ref="C112:C115"/>
-    <mergeCell ref="B116:B119"/>
-    <mergeCell ref="C116:C119"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5090,36 +5144,36 @@
       </c>
     </row>
     <row r="3" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D3" s="84" t="s">
+      <c r="D3" s="91" t="s">
         <v>8</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F3" s="86" t="s">
+      <c r="F3" s="93" t="s">
         <v>1</v>
       </c>
-      <c r="G3" s="87"/>
-      <c r="H3" s="87"/>
-      <c r="I3" s="88"/>
-      <c r="J3" s="86" t="s">
+      <c r="G3" s="94"/>
+      <c r="H3" s="94"/>
+      <c r="I3" s="95"/>
+      <c r="J3" s="93" t="s">
         <v>2</v>
       </c>
-      <c r="K3" s="87"/>
-      <c r="L3" s="87"/>
-      <c r="M3" s="88"/>
-      <c r="N3" s="86" t="s">
+      <c r="K3" s="94"/>
+      <c r="L3" s="94"/>
+      <c r="M3" s="95"/>
+      <c r="N3" s="93" t="s">
         <v>3</v>
       </c>
-      <c r="O3" s="87"/>
-      <c r="P3" s="87"/>
-      <c r="Q3" s="88"/>
+      <c r="O3" s="94"/>
+      <c r="P3" s="94"/>
+      <c r="Q3" s="95"/>
       <c r="R3" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="4:18" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D4" s="85"/>
+      <c r="D4" s="92"/>
       <c r="E4" s="4" t="s">
         <v>4</v>
       </c>
@@ -5290,36 +5344,36 @@
       </c>
     </row>
     <row r="15" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D15" s="84" t="s">
+      <c r="D15" s="91" t="s">
         <v>8</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F15" s="86" t="s">
+      <c r="F15" s="93" t="s">
         <v>1</v>
       </c>
-      <c r="G15" s="87"/>
-      <c r="H15" s="87"/>
-      <c r="I15" s="88"/>
-      <c r="J15" s="86" t="s">
+      <c r="G15" s="94"/>
+      <c r="H15" s="94"/>
+      <c r="I15" s="95"/>
+      <c r="J15" s="93" t="s">
         <v>2</v>
       </c>
-      <c r="K15" s="87"/>
-      <c r="L15" s="87"/>
-      <c r="M15" s="88"/>
-      <c r="N15" s="86" t="s">
+      <c r="K15" s="94"/>
+      <c r="L15" s="94"/>
+      <c r="M15" s="95"/>
+      <c r="N15" s="93" t="s">
         <v>3</v>
       </c>
-      <c r="O15" s="87"/>
-      <c r="P15" s="87"/>
-      <c r="Q15" s="88"/>
+      <c r="O15" s="94"/>
+      <c r="P15" s="94"/>
+      <c r="Q15" s="95"/>
       <c r="R15" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="16" spans="4:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D16" s="85"/>
+      <c r="D16" s="92"/>
       <c r="E16" s="4" t="s">
         <v>4</v>
       </c>
@@ -5504,36 +5558,36 @@
       <c r="R26" s="51"/>
     </row>
     <row r="27" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D27" s="84" t="s">
+      <c r="D27" s="91" t="s">
         <v>8</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F27" s="86" t="s">
+      <c r="F27" s="93" t="s">
         <v>1</v>
       </c>
-      <c r="G27" s="87"/>
-      <c r="H27" s="87"/>
-      <c r="I27" s="88"/>
-      <c r="J27" s="86" t="s">
+      <c r="G27" s="94"/>
+      <c r="H27" s="94"/>
+      <c r="I27" s="95"/>
+      <c r="J27" s="93" t="s">
         <v>2</v>
       </c>
-      <c r="K27" s="87"/>
-      <c r="L27" s="87"/>
-      <c r="M27" s="88"/>
-      <c r="N27" s="86" t="s">
+      <c r="K27" s="94"/>
+      <c r="L27" s="94"/>
+      <c r="M27" s="95"/>
+      <c r="N27" s="93" t="s">
         <v>3</v>
       </c>
-      <c r="O27" s="87"/>
-      <c r="P27" s="87"/>
-      <c r="Q27" s="88"/>
+      <c r="O27" s="94"/>
+      <c r="P27" s="94"/>
+      <c r="Q27" s="95"/>
       <c r="R27" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="28" spans="4:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D28" s="85"/>
+      <c r="D28" s="92"/>
       <c r="E28" s="4" t="s">
         <v>4</v>
       </c>
@@ -5725,7 +5779,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="B2:B53"/>
+  <dimension ref="B2:B55"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="245.33203125" customWidth="1"/>
@@ -5989,6 +6043,16 @@
     <row r="53" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B53" s="62" t="s">
         <v>156</v>
+      </c>
+    </row>
+    <row r="54" spans="2:2" ht="15" x14ac:dyDescent="0.3">
+      <c r="B54" s="60" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="55" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B55" s="62" t="s">
+        <v>183</v>
       </c>
     </row>
   </sheetData>
@@ -6005,6 +6069,7 @@
     <hyperlink ref="B51" r:id="rId10" xr:uid="{DCC352E9-F585-47DE-BCF7-0C1F3F51E01B}"/>
     <hyperlink ref="B45" r:id="rId11" xr:uid="{500C1AC5-73B0-417C-9903-2460A3E5FD4B}"/>
     <hyperlink ref="B53" r:id="rId12" location="h-what-is-monthly-recurring-revenue-mrr" xr:uid="{756E4B61-8845-414D-9B64-D39C0AD55437}"/>
+    <hyperlink ref="B55" r:id="rId13" xr:uid="{401991D6-68FF-44A7-9CB9-41CC84F63BFB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
built KPIs dashboard in PowerBI
</commit_message>
<xml_diff>
--- a/DocumentsAndReports/0. WorkLog_Charts.xlsx
+++ b/DocumentsAndReports/0. WorkLog_Charts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qhung\Videos\CSIS4495 - Applied Research  Project\W26_4495_S2_HughT\DocumentsAndReports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBA05676-7437-428C-BA2C-C8DB64E88782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00A0FF61-82BC-46A5-B63E-C51EAC3770BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="720" windowWidth="21600" windowHeight="11232" xr2:uid="{E067A1E6-0DC4-42DD-AAF8-D95EFF7A112F}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="185">
   <si>
     <t>January</t>
   </si>
@@ -1018,6 +1018,9 @@
   </si>
   <si>
     <t>https://www.klipfolio.com/resources/kpi-examples/sales/average-profit-margin</t>
+  </si>
+  <si>
+    <t>- Built KPIs dashboard in PowerBI</t>
   </si>
 </sst>
 </file>
@@ -1785,6 +1788,60 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1803,57 +1860,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="15" fontId="7" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="15" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="15" fontId="7" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="15" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1868,9 +1874,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3795,10 +3798,10 @@
       </c>
     </row>
     <row r="3" spans="2:4" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="81">
+      <c r="B3" s="84">
         <v>45683</v>
       </c>
-      <c r="C3" s="80">
+      <c r="C3" s="85">
         <v>2</v>
       </c>
       <c r="D3" s="34" t="s">
@@ -3806,31 +3809,31 @@
       </c>
     </row>
     <row r="4" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="81"/>
-      <c r="C4" s="80"/>
+      <c r="B4" s="84"/>
+      <c r="C4" s="85"/>
       <c r="D4" s="34" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="81"/>
-      <c r="C5" s="80"/>
+      <c r="B5" s="84"/>
+      <c r="C5" s="85"/>
       <c r="D5" s="40" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="81"/>
-      <c r="C6" s="80"/>
+      <c r="B6" s="84"/>
+      <c r="C6" s="85"/>
       <c r="D6" s="41" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="7" spans="2:4" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="81">
+      <c r="B7" s="84">
         <v>45684</v>
       </c>
-      <c r="C7" s="80">
+      <c r="C7" s="85">
         <v>1.5</v>
       </c>
       <c r="D7" s="35" t="s">
@@ -3838,31 +3841,31 @@
       </c>
     </row>
     <row r="8" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="81"/>
-      <c r="C8" s="80"/>
+      <c r="B8" s="84"/>
+      <c r="C8" s="85"/>
       <c r="D8" s="36" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="9" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="81"/>
-      <c r="C9" s="80"/>
+      <c r="B9" s="84"/>
+      <c r="C9" s="85"/>
       <c r="D9" s="42" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="10" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="81"/>
-      <c r="C10" s="80"/>
+      <c r="B10" s="84"/>
+      <c r="C10" s="85"/>
       <c r="D10" s="43" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="81">
+      <c r="B11" s="84">
         <v>45686</v>
       </c>
-      <c r="C11" s="80">
+      <c r="C11" s="85">
         <v>3</v>
       </c>
       <c r="D11" s="34" t="s">
@@ -3870,38 +3873,38 @@
       </c>
     </row>
     <row r="12" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="81"/>
-      <c r="C12" s="80"/>
+      <c r="B12" s="84"/>
+      <c r="C12" s="85"/>
       <c r="D12" s="34" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="81"/>
-      <c r="C13" s="80"/>
+      <c r="B13" s="84"/>
+      <c r="C13" s="85"/>
       <c r="D13" s="34" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="81"/>
-      <c r="C14" s="80"/>
+      <c r="B14" s="84"/>
+      <c r="C14" s="85"/>
       <c r="D14" s="44" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="81"/>
-      <c r="C15" s="80"/>
+      <c r="B15" s="84"/>
+      <c r="C15" s="85"/>
       <c r="D15" s="41" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="81">
+      <c r="B16" s="84">
         <v>46053</v>
       </c>
-      <c r="C16" s="80">
+      <c r="C16" s="85">
         <v>4</v>
       </c>
       <c r="D16" s="37" t="s">
@@ -3909,80 +3912,80 @@
       </c>
     </row>
     <row r="17" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="81"/>
-      <c r="C17" s="80"/>
+      <c r="B17" s="84"/>
+      <c r="C17" s="85"/>
       <c r="D17" s="34" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="81"/>
-      <c r="C18" s="80"/>
+      <c r="B18" s="84"/>
+      <c r="C18" s="85"/>
       <c r="D18" s="34" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="19" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="81"/>
-      <c r="C19" s="80"/>
+      <c r="B19" s="84"/>
+      <c r="C19" s="85"/>
       <c r="D19" s="34" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="20" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="81"/>
-      <c r="C20" s="80"/>
+      <c r="B20" s="84"/>
+      <c r="C20" s="85"/>
       <c r="D20" s="34" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="21" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="81"/>
-      <c r="C21" s="80"/>
+      <c r="B21" s="84"/>
+      <c r="C21" s="85"/>
       <c r="D21" s="34" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="81"/>
-      <c r="C22" s="80"/>
+      <c r="B22" s="84"/>
+      <c r="C22" s="85"/>
       <c r="D22" s="44" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="23" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="81"/>
-      <c r="C23" s="80"/>
+      <c r="B23" s="84"/>
+      <c r="C23" s="85"/>
       <c r="D23" s="40" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="24" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="81"/>
-      <c r="C24" s="80"/>
+      <c r="B24" s="84"/>
+      <c r="C24" s="85"/>
       <c r="D24" s="40" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="25" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="81"/>
-      <c r="C25" s="80"/>
+      <c r="B25" s="84"/>
+      <c r="C25" s="85"/>
       <c r="D25" s="40" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="26" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="81"/>
-      <c r="C26" s="80"/>
+      <c r="B26" s="84"/>
+      <c r="C26" s="85"/>
       <c r="D26" s="45" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="27" spans="2:4" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="81">
+      <c r="B27" s="84">
         <v>46054</v>
       </c>
-      <c r="C27" s="80">
+      <c r="C27" s="85">
         <v>1</v>
       </c>
       <c r="D27" s="34" t="s">
@@ -3990,31 +3993,31 @@
       </c>
     </row>
     <row r="28" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="81"/>
-      <c r="C28" s="80"/>
+      <c r="B28" s="84"/>
+      <c r="C28" s="85"/>
       <c r="D28" s="34" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="29" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="81"/>
-      <c r="C29" s="80"/>
+      <c r="B29" s="84"/>
+      <c r="C29" s="85"/>
       <c r="D29" s="40" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="30" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="81"/>
-      <c r="C30" s="80"/>
+      <c r="B30" s="84"/>
+      <c r="C30" s="85"/>
       <c r="D30" s="41" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="31" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B31" s="81">
+      <c r="B31" s="84">
         <v>46055</v>
       </c>
-      <c r="C31" s="80">
+      <c r="C31" s="85">
         <v>4</v>
       </c>
       <c r="D31" s="38" t="s">
@@ -4022,45 +4025,45 @@
       </c>
     </row>
     <row r="32" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B32" s="81"/>
-      <c r="C32" s="80"/>
+      <c r="B32" s="84"/>
+      <c r="C32" s="85"/>
       <c r="D32" s="39" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="33" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="81"/>
-      <c r="C33" s="80"/>
+      <c r="B33" s="84"/>
+      <c r="C33" s="85"/>
       <c r="D33" s="39" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="34" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B34" s="81"/>
-      <c r="C34" s="80"/>
+      <c r="B34" s="84"/>
+      <c r="C34" s="85"/>
       <c r="D34" s="39" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="35" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B35" s="81"/>
-      <c r="C35" s="80"/>
+      <c r="B35" s="84"/>
+      <c r="C35" s="85"/>
       <c r="D35" s="46" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="36" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B36" s="81"/>
-      <c r="C36" s="80"/>
+      <c r="B36" s="84"/>
+      <c r="C36" s="85"/>
       <c r="D36" s="47" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="37" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="81">
+      <c r="B37" s="84">
         <v>46056</v>
       </c>
-      <c r="C37" s="80">
+      <c r="C37" s="85">
         <v>3</v>
       </c>
       <c r="D37" s="34" t="s">
@@ -4068,38 +4071,38 @@
       </c>
     </row>
     <row r="38" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B38" s="81"/>
-      <c r="C38" s="80"/>
+      <c r="B38" s="84"/>
+      <c r="C38" s="85"/>
       <c r="D38" s="34" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="39" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B39" s="81"/>
-      <c r="C39" s="80"/>
+      <c r="B39" s="84"/>
+      <c r="C39" s="85"/>
       <c r="D39" s="34" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="40" spans="2:4" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B40" s="81"/>
-      <c r="C40" s="80"/>
+      <c r="B40" s="84"/>
+      <c r="C40" s="85"/>
       <c r="D40" s="40" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="41" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B41" s="81"/>
-      <c r="C41" s="80"/>
+      <c r="B41" s="84"/>
+      <c r="C41" s="85"/>
       <c r="D41" s="41" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="42" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B42" s="81">
+      <c r="B42" s="84">
         <v>46057</v>
       </c>
-      <c r="C42" s="80">
+      <c r="C42" s="85">
         <v>4</v>
       </c>
       <c r="D42" s="37" t="s">
@@ -4107,24 +4110,24 @@
       </c>
     </row>
     <row r="43" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B43" s="81"/>
-      <c r="C43" s="80"/>
+      <c r="B43" s="84"/>
+      <c r="C43" s="85"/>
       <c r="D43" s="34" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="44" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B44" s="81"/>
-      <c r="C44" s="80"/>
+      <c r="B44" s="84"/>
+      <c r="C44" s="85"/>
       <c r="D44" s="41" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="45" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B45" s="82">
+      <c r="B45" s="75">
         <v>46059</v>
       </c>
-      <c r="C45" s="85">
+      <c r="C45" s="78">
         <v>2</v>
       </c>
       <c r="D45" s="49" t="s">
@@ -4132,38 +4135,38 @@
       </c>
     </row>
     <row r="46" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B46" s="83"/>
-      <c r="C46" s="86"/>
+      <c r="B46" s="76"/>
+      <c r="C46" s="79"/>
       <c r="D46" s="48" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="47" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B47" s="83"/>
-      <c r="C47" s="86"/>
+      <c r="B47" s="76"/>
+      <c r="C47" s="79"/>
       <c r="D47" s="34" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="48" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B48" s="83"/>
-      <c r="C48" s="86"/>
+      <c r="B48" s="76"/>
+      <c r="C48" s="79"/>
       <c r="D48" s="41" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="49" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B49" s="84"/>
-      <c r="C49" s="87"/>
+      <c r="B49" s="77"/>
+      <c r="C49" s="80"/>
       <c r="D49" s="45" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="50" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B50" s="82">
+      <c r="B50" s="75">
         <v>46061</v>
       </c>
-      <c r="C50" s="85">
+      <c r="C50" s="78">
         <v>1.5</v>
       </c>
       <c r="D50" s="49" t="s">
@@ -4171,38 +4174,38 @@
       </c>
     </row>
     <row r="51" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B51" s="83"/>
-      <c r="C51" s="86"/>
+      <c r="B51" s="76"/>
+      <c r="C51" s="79"/>
       <c r="D51" s="34" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="52" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B52" s="83"/>
-      <c r="C52" s="86"/>
+      <c r="B52" s="76"/>
+      <c r="C52" s="79"/>
       <c r="D52" s="41" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="53" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B53" s="83"/>
-      <c r="C53" s="86"/>
+      <c r="B53" s="76"/>
+      <c r="C53" s="79"/>
       <c r="D53" s="41" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="54" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B54" s="84"/>
-      <c r="C54" s="87"/>
+      <c r="B54" s="77"/>
+      <c r="C54" s="80"/>
       <c r="D54" s="45" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="55" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="82">
+      <c r="B55" s="75">
         <v>46062</v>
       </c>
-      <c r="C55" s="85">
+      <c r="C55" s="78">
         <v>2</v>
       </c>
       <c r="D55" s="52" t="s">
@@ -4210,31 +4213,31 @@
       </c>
     </row>
     <row r="56" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B56" s="83"/>
-      <c r="C56" s="86"/>
+      <c r="B56" s="76"/>
+      <c r="C56" s="79"/>
       <c r="D56" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="57" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B57" s="83"/>
-      <c r="C57" s="86"/>
+      <c r="B57" s="76"/>
+      <c r="C57" s="79"/>
       <c r="D57" s="41" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="58" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B58" s="84"/>
-      <c r="C58" s="87"/>
+      <c r="B58" s="77"/>
+      <c r="C58" s="80"/>
       <c r="D58" s="45" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="59" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="82">
+      <c r="B59" s="75">
         <v>46063</v>
       </c>
-      <c r="C59" s="85">
+      <c r="C59" s="78">
         <v>3</v>
       </c>
       <c r="D59" s="52" t="s">
@@ -4242,38 +4245,38 @@
       </c>
     </row>
     <row r="60" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B60" s="83"/>
-      <c r="C60" s="86"/>
+      <c r="B60" s="76"/>
+      <c r="C60" s="79"/>
       <c r="D60" s="53" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="61" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B61" s="83"/>
-      <c r="C61" s="86"/>
+      <c r="B61" s="76"/>
+      <c r="C61" s="79"/>
       <c r="D61" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="62" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B62" s="83"/>
-      <c r="C62" s="86"/>
+      <c r="B62" s="76"/>
+      <c r="C62" s="79"/>
       <c r="D62" s="41" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="63" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B63" s="84"/>
-      <c r="C63" s="87"/>
+      <c r="B63" s="77"/>
+      <c r="C63" s="80"/>
       <c r="D63" s="45" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="64" spans="2:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B64" s="82">
+      <c r="B64" s="75">
         <v>46064</v>
       </c>
-      <c r="C64" s="85">
+      <c r="C64" s="78">
         <v>3</v>
       </c>
       <c r="D64" s="52" t="s">
@@ -4281,38 +4284,38 @@
       </c>
     </row>
     <row r="65" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B65" s="83"/>
-      <c r="C65" s="86"/>
+      <c r="B65" s="76"/>
+      <c r="C65" s="79"/>
       <c r="D65" s="53" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="66" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B66" s="83"/>
-      <c r="C66" s="86"/>
+      <c r="B66" s="76"/>
+      <c r="C66" s="79"/>
       <c r="D66" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="67" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B67" s="83"/>
-      <c r="C67" s="86"/>
+      <c r="B67" s="76"/>
+      <c r="C67" s="79"/>
       <c r="D67" s="41" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="68" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B68" s="84"/>
-      <c r="C68" s="87"/>
+      <c r="B68" s="77"/>
+      <c r="C68" s="80"/>
       <c r="D68" s="45" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="69" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B69" s="88">
+      <c r="B69" s="81">
         <v>46066</v>
       </c>
-      <c r="C69" s="85">
+      <c r="C69" s="78">
         <v>2</v>
       </c>
       <c r="D69" s="52" t="s">
@@ -4320,45 +4323,45 @@
       </c>
     </row>
     <row r="70" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B70" s="89"/>
-      <c r="C70" s="86"/>
+      <c r="B70" s="82"/>
+      <c r="C70" s="79"/>
       <c r="D70" s="53" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="71" spans="2:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B71" s="89"/>
-      <c r="C71" s="86"/>
+      <c r="B71" s="82"/>
+      <c r="C71" s="79"/>
       <c r="D71" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="72" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B72" s="89"/>
-      <c r="C72" s="86"/>
+      <c r="B72" s="82"/>
+      <c r="C72" s="79"/>
       <c r="D72" s="41" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="73" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B73" s="89"/>
-      <c r="C73" s="86"/>
+      <c r="B73" s="82"/>
+      <c r="C73" s="79"/>
       <c r="D73" s="41" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="74" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B74" s="90"/>
-      <c r="C74" s="87"/>
+      <c r="B74" s="83"/>
+      <c r="C74" s="80"/>
       <c r="D74" s="45" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="75" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B75" s="74">
+      <c r="B75" s="69">
         <v>46068</v>
       </c>
-      <c r="C75" s="77">
+      <c r="C75" s="72">
         <v>2.5</v>
       </c>
       <c r="D75" s="52" t="s">
@@ -4366,52 +4369,52 @@
       </c>
     </row>
     <row r="76" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B76" s="75"/>
-      <c r="C76" s="78"/>
+      <c r="B76" s="70"/>
+      <c r="C76" s="73"/>
       <c r="D76" s="53" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="77" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B77" s="75"/>
-      <c r="C77" s="78"/>
+      <c r="B77" s="70"/>
+      <c r="C77" s="73"/>
       <c r="D77" s="53" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="78" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B78" s="75"/>
-      <c r="C78" s="78"/>
+      <c r="B78" s="70"/>
+      <c r="C78" s="73"/>
       <c r="D78" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="79" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B79" s="75"/>
-      <c r="C79" s="78"/>
+      <c r="B79" s="70"/>
+      <c r="C79" s="73"/>
       <c r="D79" s="41" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="80" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B80" s="75"/>
-      <c r="C80" s="78"/>
+      <c r="B80" s="70"/>
+      <c r="C80" s="73"/>
       <c r="D80" s="41" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="81" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B81" s="76"/>
-      <c r="C81" s="79"/>
+      <c r="B81" s="71"/>
+      <c r="C81" s="74"/>
       <c r="D81" s="45" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="82" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B82" s="74">
+      <c r="B82" s="69">
         <v>46070</v>
       </c>
-      <c r="C82" s="77">
+      <c r="C82" s="72">
         <v>3</v>
       </c>
       <c r="D82" s="52" t="s">
@@ -4419,52 +4422,52 @@
       </c>
     </row>
     <row r="83" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B83" s="75"/>
-      <c r="C83" s="78"/>
+      <c r="B83" s="70"/>
+      <c r="C83" s="73"/>
       <c r="D83" s="53" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="84" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B84" s="75"/>
-      <c r="C84" s="78"/>
+      <c r="B84" s="70"/>
+      <c r="C84" s="73"/>
       <c r="D84" s="53" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="85" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B85" s="75"/>
-      <c r="C85" s="78"/>
+      <c r="B85" s="70"/>
+      <c r="C85" s="73"/>
       <c r="D85" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="86" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B86" s="75"/>
-      <c r="C86" s="78"/>
+      <c r="B86" s="70"/>
+      <c r="C86" s="73"/>
       <c r="D86" s="41" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="87" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B87" s="75"/>
-      <c r="C87" s="78"/>
+      <c r="B87" s="70"/>
+      <c r="C87" s="73"/>
       <c r="D87" s="41" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="88" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B88" s="76"/>
-      <c r="C88" s="79"/>
+      <c r="B88" s="71"/>
+      <c r="C88" s="74"/>
       <c r="D88" s="45" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="89" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B89" s="74">
+      <c r="B89" s="69">
         <v>46071</v>
       </c>
-      <c r="C89" s="77">
+      <c r="C89" s="72">
         <v>2</v>
       </c>
       <c r="D89" s="52" t="s">
@@ -4472,38 +4475,38 @@
       </c>
     </row>
     <row r="90" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B90" s="75"/>
-      <c r="C90" s="78"/>
+      <c r="B90" s="70"/>
+      <c r="C90" s="73"/>
       <c r="D90" s="53" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="91" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B91" s="75"/>
-      <c r="C91" s="78"/>
+      <c r="B91" s="70"/>
+      <c r="C91" s="73"/>
       <c r="D91" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="92" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B92" s="75"/>
-      <c r="C92" s="78"/>
+      <c r="B92" s="70"/>
+      <c r="C92" s="73"/>
       <c r="D92" s="41" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="93" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B93" s="76"/>
-      <c r="C93" s="79"/>
+      <c r="B93" s="71"/>
+      <c r="C93" s="74"/>
       <c r="D93" s="45" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="94" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B94" s="74">
+      <c r="B94" s="69">
         <v>46074</v>
       </c>
-      <c r="C94" s="77">
+      <c r="C94" s="72">
         <v>3</v>
       </c>
       <c r="D94" s="55" t="s">
@@ -4511,24 +4514,24 @@
       </c>
     </row>
     <row r="95" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B95" s="75"/>
-      <c r="C95" s="78"/>
+      <c r="B95" s="70"/>
+      <c r="C95" s="73"/>
       <c r="D95" s="56" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="96" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B96" s="76"/>
-      <c r="C96" s="79"/>
+      <c r="B96" s="71"/>
+      <c r="C96" s="74"/>
       <c r="D96" s="45" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="97" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B97" s="74">
+      <c r="B97" s="69">
         <v>46075</v>
       </c>
-      <c r="C97" s="77">
+      <c r="C97" s="72">
         <v>3</v>
       </c>
       <c r="D97" s="52" t="s">
@@ -4536,22 +4539,22 @@
       </c>
     </row>
     <row r="98" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B98" s="75"/>
-      <c r="C98" s="78"/>
+      <c r="B98" s="70"/>
+      <c r="C98" s="73"/>
       <c r="D98" s="53" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="99" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B99" s="75"/>
-      <c r="C99" s="78"/>
+      <c r="B99" s="70"/>
+      <c r="C99" s="73"/>
       <c r="D99" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="100" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B100" s="76"/>
-      <c r="C100" s="79"/>
+      <c r="B100" s="71"/>
+      <c r="C100" s="74"/>
       <c r="D100" s="45" t="s">
         <v>23</v>
       </c>
@@ -4568,10 +4571,10 @@
       </c>
     </row>
     <row r="102" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B102" s="74">
+      <c r="B102" s="69">
         <v>46077</v>
       </c>
-      <c r="C102" s="77">
+      <c r="C102" s="72">
         <v>2</v>
       </c>
       <c r="D102" s="52" t="s">
@@ -4579,38 +4582,38 @@
       </c>
     </row>
     <row r="103" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B103" s="75"/>
-      <c r="C103" s="78"/>
+      <c r="B103" s="70"/>
+      <c r="C103" s="73"/>
       <c r="D103" s="53" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="104" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B104" s="75"/>
-      <c r="C104" s="78"/>
+      <c r="B104" s="70"/>
+      <c r="C104" s="73"/>
       <c r="D104" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="105" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B105" s="75"/>
-      <c r="C105" s="78"/>
+      <c r="B105" s="70"/>
+      <c r="C105" s="73"/>
       <c r="D105" s="41" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="106" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B106" s="76"/>
-      <c r="C106" s="79"/>
+      <c r="B106" s="71"/>
+      <c r="C106" s="74"/>
       <c r="D106" s="45" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="107" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B107" s="74">
+      <c r="B107" s="69">
         <v>46078</v>
       </c>
-      <c r="C107" s="77">
+      <c r="C107" s="72">
         <v>1</v>
       </c>
       <c r="D107" s="63" t="s">
@@ -4618,38 +4621,38 @@
       </c>
     </row>
     <row r="108" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B108" s="75"/>
-      <c r="C108" s="78"/>
+      <c r="B108" s="70"/>
+      <c r="C108" s="73"/>
       <c r="D108" s="53" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="109" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B109" s="75"/>
-      <c r="C109" s="78"/>
+      <c r="B109" s="70"/>
+      <c r="C109" s="73"/>
       <c r="D109" s="41" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="110" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B110" s="75"/>
-      <c r="C110" s="78"/>
+      <c r="B110" s="70"/>
+      <c r="C110" s="73"/>
       <c r="D110" s="41" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="111" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B111" s="76"/>
-      <c r="C111" s="79"/>
+      <c r="B111" s="71"/>
+      <c r="C111" s="74"/>
       <c r="D111" s="64" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="112" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B112" s="74">
+      <c r="B112" s="69">
         <v>46079</v>
       </c>
-      <c r="C112" s="77">
+      <c r="C112" s="72">
         <v>2</v>
       </c>
       <c r="D112" s="63" t="s">
@@ -4657,31 +4660,31 @@
       </c>
     </row>
     <row r="113" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B113" s="75"/>
-      <c r="C113" s="78"/>
+      <c r="B113" s="70"/>
+      <c r="C113" s="73"/>
       <c r="D113" s="53" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="114" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B114" s="75"/>
-      <c r="C114" s="78"/>
+      <c r="B114" s="70"/>
+      <c r="C114" s="73"/>
       <c r="D114" s="41" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="115" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B115" s="76"/>
-      <c r="C115" s="79"/>
+      <c r="B115" s="71"/>
+      <c r="C115" s="74"/>
       <c r="D115" s="45" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="116" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B116" s="74">
+      <c r="B116" s="69">
         <v>46083</v>
       </c>
-      <c r="C116" s="77">
+      <c r="C116" s="72">
         <v>3</v>
       </c>
       <c r="D116" s="63" t="s">
@@ -4689,31 +4692,31 @@
       </c>
     </row>
     <row r="117" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B117" s="75"/>
-      <c r="C117" s="78"/>
+      <c r="B117" s="70"/>
+      <c r="C117" s="73"/>
       <c r="D117" s="53" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="118" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B118" s="75"/>
-      <c r="C118" s="78"/>
+      <c r="B118" s="70"/>
+      <c r="C118" s="73"/>
       <c r="D118" s="53" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="119" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B119" s="76"/>
-      <c r="C119" s="79"/>
+      <c r="B119" s="71"/>
+      <c r="C119" s="74"/>
       <c r="D119" s="45" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="120" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B120" s="74">
+      <c r="B120" s="69">
         <v>411326</v>
       </c>
-      <c r="C120" s="77">
+      <c r="C120" s="72">
         <v>5</v>
       </c>
       <c r="D120" s="63" t="s">
@@ -4721,24 +4724,24 @@
       </c>
     </row>
     <row r="121" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B121" s="75"/>
-      <c r="C121" s="78"/>
+      <c r="B121" s="70"/>
+      <c r="C121" s="73"/>
       <c r="D121" s="53" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="122" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B122" s="76"/>
-      <c r="C122" s="79"/>
+      <c r="B122" s="71"/>
+      <c r="C122" s="74"/>
       <c r="D122" s="65" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="123" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B123" s="68">
+      <c r="B123" s="86">
         <v>46085</v>
       </c>
-      <c r="C123" s="71">
+      <c r="C123" s="89">
         <v>4</v>
       </c>
       <c r="D123" s="63" t="s">
@@ -4746,38 +4749,38 @@
       </c>
     </row>
     <row r="124" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B124" s="69"/>
-      <c r="C124" s="72"/>
+      <c r="B124" s="87"/>
+      <c r="C124" s="90"/>
       <c r="D124" s="53" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="125" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B125" s="69"/>
-      <c r="C125" s="72"/>
+      <c r="B125" s="87"/>
+      <c r="C125" s="90"/>
       <c r="D125" s="53" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="126" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B126" s="69"/>
-      <c r="C126" s="72"/>
+      <c r="B126" s="87"/>
+      <c r="C126" s="90"/>
       <c r="D126" s="41" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="127" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B127" s="70"/>
-      <c r="C127" s="73"/>
+      <c r="B127" s="88"/>
+      <c r="C127" s="91"/>
       <c r="D127" s="45" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="128" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B128" s="74">
+      <c r="B128" s="69">
         <v>46086</v>
       </c>
-      <c r="C128" s="77">
+      <c r="C128" s="72">
         <v>6</v>
       </c>
       <c r="D128" s="63" t="s">
@@ -4785,108 +4788,108 @@
       </c>
     </row>
     <row r="129" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B129" s="75"/>
-      <c r="C129" s="78"/>
+      <c r="B129" s="70"/>
+      <c r="C129" s="73"/>
       <c r="D129" s="53" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="130" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B130" s="75"/>
-      <c r="C130" s="78"/>
+      <c r="B130" s="70"/>
+      <c r="C130" s="73"/>
       <c r="D130" s="53" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="131" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B131" s="75"/>
-      <c r="C131" s="78"/>
+      <c r="B131" s="70"/>
+      <c r="C131" s="73"/>
       <c r="D131" s="67" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="132" spans="2:4" ht="78" x14ac:dyDescent="0.3">
-      <c r="B132" s="75"/>
-      <c r="C132" s="78"/>
+      <c r="B132" s="70"/>
+      <c r="C132" s="73"/>
       <c r="D132" s="67" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="133" spans="2:4" ht="78" x14ac:dyDescent="0.3">
-      <c r="B133" s="75"/>
-      <c r="C133" s="78"/>
+      <c r="B133" s="70"/>
+      <c r="C133" s="73"/>
       <c r="D133" s="67" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="134" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B134" s="75"/>
-      <c r="C134" s="78"/>
+      <c r="B134" s="70"/>
+      <c r="C134" s="73"/>
       <c r="D134" s="67" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="135" spans="2:4" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B135" s="75"/>
-      <c r="C135" s="78"/>
+      <c r="B135" s="70"/>
+      <c r="C135" s="73"/>
       <c r="D135" s="67" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="136" spans="2:4" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="B136" s="75"/>
-      <c r="C136" s="78"/>
+      <c r="B136" s="70"/>
+      <c r="C136" s="73"/>
       <c r="D136" s="67" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="137" spans="2:4" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B137" s="75"/>
-      <c r="C137" s="78"/>
+      <c r="B137" s="70"/>
+      <c r="C137" s="73"/>
       <c r="D137" s="67" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="138" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B138" s="75"/>
-      <c r="C138" s="78"/>
+      <c r="B138" s="70"/>
+      <c r="C138" s="73"/>
       <c r="D138" s="67" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="139" spans="2:4" ht="78" x14ac:dyDescent="0.3">
-      <c r="B139" s="75"/>
-      <c r="C139" s="78"/>
+      <c r="B139" s="70"/>
+      <c r="C139" s="73"/>
       <c r="D139" s="67" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="140" spans="2:4" ht="78" x14ac:dyDescent="0.3">
-      <c r="B140" s="75"/>
-      <c r="C140" s="78"/>
+      <c r="B140" s="70"/>
+      <c r="C140" s="73"/>
       <c r="D140" s="67" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="141" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B141" s="75"/>
-      <c r="C141" s="78"/>
+      <c r="B141" s="70"/>
+      <c r="C141" s="73"/>
       <c r="D141" s="67" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="142" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B142" s="76"/>
-      <c r="C142" s="79"/>
-      <c r="D142" s="96" t="s">
+      <c r="B142" s="71"/>
+      <c r="C142" s="74"/>
+      <c r="D142" s="68" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="143" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B143" s="66">
+      <c r="B143" s="69">
         <v>46087</v>
       </c>
-      <c r="C143" s="54">
+      <c r="C143" s="72">
         <v>4</v>
       </c>
       <c r="D143" s="63" t="s">
@@ -4894,65 +4897,71 @@
       </c>
     </row>
     <row r="144" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B144" s="32"/>
-      <c r="C144" s="32"/>
+      <c r="B144" s="70"/>
+      <c r="C144" s="73"/>
       <c r="D144" s="53" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="145" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B145" s="32"/>
-      <c r="C145" s="32"/>
+      <c r="B145" s="70"/>
+      <c r="C145" s="73"/>
       <c r="D145" s="53" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="146" spans="2:4" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B146" s="32"/>
-      <c r="C146" s="32"/>
+      <c r="B146" s="70"/>
+      <c r="C146" s="73"/>
       <c r="D146" s="67" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="147" spans="2:4" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B147" s="32"/>
-      <c r="C147" s="32"/>
+      <c r="B147" s="70"/>
+      <c r="C147" s="73"/>
       <c r="D147" s="67" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="148" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B148" s="32"/>
-      <c r="C148" s="32"/>
+      <c r="B148" s="70"/>
+      <c r="C148" s="73"/>
       <c r="D148" s="67" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="149" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B149" s="32"/>
-      <c r="C149" s="32"/>
+      <c r="B149" s="70"/>
+      <c r="C149" s="73"/>
       <c r="D149" s="67" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="150" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B150" s="32"/>
-      <c r="C150" s="32"/>
+      <c r="B150" s="70"/>
+      <c r="C150" s="73"/>
       <c r="D150" s="67" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="151" spans="2:4" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B151" s="32"/>
-      <c r="C151" s="32"/>
-      <c r="D151" s="67" t="s">
+    <row r="151" spans="2:4" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B151" s="71"/>
+      <c r="C151" s="74"/>
+      <c r="D151" s="68" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="152" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B152" s="32"/>
-      <c r="C152" s="32"/>
-      <c r="D152" s="67"/>
+    <row r="152" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B152" s="66">
+        <v>46088</v>
+      </c>
+      <c r="C152" s="54">
+        <v>4</v>
+      </c>
+      <c r="D152" s="63" t="s">
+        <v>184</v>
+      </c>
     </row>
     <row r="153" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B153" s="32"/>
@@ -5063,45 +5072,9 @@
       <c r="D174" s="67"/>
     </row>
   </sheetData>
-  <mergeCells count="52">
-    <mergeCell ref="B128:B142"/>
-    <mergeCell ref="C128:C142"/>
-    <mergeCell ref="B120:B122"/>
-    <mergeCell ref="C120:C122"/>
-    <mergeCell ref="B112:B115"/>
-    <mergeCell ref="C112:C115"/>
-    <mergeCell ref="B116:B119"/>
-    <mergeCell ref="C116:C119"/>
-    <mergeCell ref="B102:B106"/>
-    <mergeCell ref="C102:C106"/>
-    <mergeCell ref="B97:B100"/>
-    <mergeCell ref="C97:C100"/>
-    <mergeCell ref="B82:B88"/>
-    <mergeCell ref="C82:C88"/>
-    <mergeCell ref="B89:B93"/>
-    <mergeCell ref="C89:C93"/>
-    <mergeCell ref="B94:B96"/>
-    <mergeCell ref="C94:C96"/>
-    <mergeCell ref="B64:B68"/>
-    <mergeCell ref="C64:C68"/>
-    <mergeCell ref="B69:B74"/>
-    <mergeCell ref="C69:C74"/>
-    <mergeCell ref="B75:B81"/>
-    <mergeCell ref="C75:C81"/>
-    <mergeCell ref="B59:B63"/>
-    <mergeCell ref="C59:C63"/>
-    <mergeCell ref="B3:B6"/>
-    <mergeCell ref="C3:C6"/>
-    <mergeCell ref="B7:B10"/>
-    <mergeCell ref="C7:C10"/>
-    <mergeCell ref="B11:B15"/>
-    <mergeCell ref="C11:C15"/>
-    <mergeCell ref="B45:B49"/>
-    <mergeCell ref="C45:C49"/>
-    <mergeCell ref="B50:B54"/>
-    <mergeCell ref="C50:C54"/>
-    <mergeCell ref="B123:B127"/>
-    <mergeCell ref="C123:C127"/>
+  <mergeCells count="54">
+    <mergeCell ref="B143:B151"/>
+    <mergeCell ref="C143:C151"/>
     <mergeCell ref="B107:B111"/>
     <mergeCell ref="C107:C111"/>
     <mergeCell ref="C16:C26"/>
@@ -5116,6 +5089,44 @@
     <mergeCell ref="C42:C44"/>
     <mergeCell ref="B55:B58"/>
     <mergeCell ref="C55:C58"/>
+    <mergeCell ref="B59:B63"/>
+    <mergeCell ref="C59:C63"/>
+    <mergeCell ref="B3:B6"/>
+    <mergeCell ref="C3:C6"/>
+    <mergeCell ref="B7:B10"/>
+    <mergeCell ref="C7:C10"/>
+    <mergeCell ref="B11:B15"/>
+    <mergeCell ref="C11:C15"/>
+    <mergeCell ref="B45:B49"/>
+    <mergeCell ref="C45:C49"/>
+    <mergeCell ref="B50:B54"/>
+    <mergeCell ref="C50:C54"/>
+    <mergeCell ref="B64:B68"/>
+    <mergeCell ref="C64:C68"/>
+    <mergeCell ref="B69:B74"/>
+    <mergeCell ref="C69:C74"/>
+    <mergeCell ref="B75:B81"/>
+    <mergeCell ref="C75:C81"/>
+    <mergeCell ref="B102:B106"/>
+    <mergeCell ref="C102:C106"/>
+    <mergeCell ref="B97:B100"/>
+    <mergeCell ref="C97:C100"/>
+    <mergeCell ref="B82:B88"/>
+    <mergeCell ref="C82:C88"/>
+    <mergeCell ref="B89:B93"/>
+    <mergeCell ref="C89:C93"/>
+    <mergeCell ref="B94:B96"/>
+    <mergeCell ref="C94:C96"/>
+    <mergeCell ref="B128:B142"/>
+    <mergeCell ref="C128:C142"/>
+    <mergeCell ref="B120:B122"/>
+    <mergeCell ref="C120:C122"/>
+    <mergeCell ref="B112:B115"/>
+    <mergeCell ref="C112:C115"/>
+    <mergeCell ref="B116:B119"/>
+    <mergeCell ref="C116:C119"/>
+    <mergeCell ref="B123:B127"/>
+    <mergeCell ref="C123:C127"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5144,36 +5155,36 @@
       </c>
     </row>
     <row r="3" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D3" s="91" t="s">
+      <c r="D3" s="92" t="s">
         <v>8</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F3" s="93" t="s">
+      <c r="F3" s="94" t="s">
         <v>1</v>
       </c>
-      <c r="G3" s="94"/>
-      <c r="H3" s="94"/>
-      <c r="I3" s="95"/>
-      <c r="J3" s="93" t="s">
+      <c r="G3" s="95"/>
+      <c r="H3" s="95"/>
+      <c r="I3" s="96"/>
+      <c r="J3" s="94" t="s">
         <v>2</v>
       </c>
-      <c r="K3" s="94"/>
-      <c r="L3" s="94"/>
-      <c r="M3" s="95"/>
-      <c r="N3" s="93" t="s">
+      <c r="K3" s="95"/>
+      <c r="L3" s="95"/>
+      <c r="M3" s="96"/>
+      <c r="N3" s="94" t="s">
         <v>3</v>
       </c>
-      <c r="O3" s="94"/>
-      <c r="P3" s="94"/>
-      <c r="Q3" s="95"/>
+      <c r="O3" s="95"/>
+      <c r="P3" s="95"/>
+      <c r="Q3" s="96"/>
       <c r="R3" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="4:18" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D4" s="92"/>
+      <c r="D4" s="93"/>
       <c r="E4" s="4" t="s">
         <v>4</v>
       </c>
@@ -5344,36 +5355,36 @@
       </c>
     </row>
     <row r="15" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D15" s="91" t="s">
+      <c r="D15" s="92" t="s">
         <v>8</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F15" s="93" t="s">
+      <c r="F15" s="94" t="s">
         <v>1</v>
       </c>
-      <c r="G15" s="94"/>
-      <c r="H15" s="94"/>
-      <c r="I15" s="95"/>
-      <c r="J15" s="93" t="s">
+      <c r="G15" s="95"/>
+      <c r="H15" s="95"/>
+      <c r="I15" s="96"/>
+      <c r="J15" s="94" t="s">
         <v>2</v>
       </c>
-      <c r="K15" s="94"/>
-      <c r="L15" s="94"/>
-      <c r="M15" s="95"/>
-      <c r="N15" s="93" t="s">
+      <c r="K15" s="95"/>
+      <c r="L15" s="95"/>
+      <c r="M15" s="96"/>
+      <c r="N15" s="94" t="s">
         <v>3</v>
       </c>
-      <c r="O15" s="94"/>
-      <c r="P15" s="94"/>
-      <c r="Q15" s="95"/>
+      <c r="O15" s="95"/>
+      <c r="P15" s="95"/>
+      <c r="Q15" s="96"/>
       <c r="R15" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="16" spans="4:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D16" s="92"/>
+      <c r="D16" s="93"/>
       <c r="E16" s="4" t="s">
         <v>4</v>
       </c>
@@ -5558,36 +5569,36 @@
       <c r="R26" s="51"/>
     </row>
     <row r="27" spans="4:18" x14ac:dyDescent="0.3">
-      <c r="D27" s="91" t="s">
+      <c r="D27" s="92" t="s">
         <v>8</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F27" s="93" t="s">
+      <c r="F27" s="94" t="s">
         <v>1</v>
       </c>
-      <c r="G27" s="94"/>
-      <c r="H27" s="94"/>
-      <c r="I27" s="95"/>
-      <c r="J27" s="93" t="s">
+      <c r="G27" s="95"/>
+      <c r="H27" s="95"/>
+      <c r="I27" s="96"/>
+      <c r="J27" s="94" t="s">
         <v>2</v>
       </c>
-      <c r="K27" s="94"/>
-      <c r="L27" s="94"/>
-      <c r="M27" s="95"/>
-      <c r="N27" s="93" t="s">
+      <c r="K27" s="95"/>
+      <c r="L27" s="95"/>
+      <c r="M27" s="96"/>
+      <c r="N27" s="94" t="s">
         <v>3</v>
       </c>
-      <c r="O27" s="94"/>
-      <c r="P27" s="94"/>
-      <c r="Q27" s="95"/>
+      <c r="O27" s="95"/>
+      <c r="P27" s="95"/>
+      <c r="Q27" s="96"/>
       <c r="R27" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="28" spans="4:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D28" s="92"/>
+      <c r="D28" s="93"/>
       <c r="E28" s="4" t="s">
         <v>4</v>
       </c>

</xml_diff>